<commit_message>
record diptest in the lockfile
</commit_message>
<xml_diff>
--- a/03_Features/c_data/05_module_annotation.xlsx
+++ b/03_Features/c_data/05_module_annotation.xlsx
@@ -235,7 +235,7 @@
     <t xml:space="preserve">378/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">LDHD/PRKAA2/PCBD1/ACADM/PFKM/ACADSB/RDH13/NDUFV3/SFXN1/AK3/NAXD/KARS1/STAT5B/FBP2/PDP1/GMPPB/PFKFB1/MAT2B/THTPA/ACOT2/ECI1/DCXR/PCBD2/KYAT1/L2HGDH/MT-ATP8/PGP/ATP5F1E/THAP4/IDI1/MPI/DLD/COQ7/SHMT2/SUCLA2/PTGR2/ATP5F1C/MT-ND1/ATP5F1D/SDHD/ACSS2/PPA2/FBP1/IDH3B/STOML2/ACADS/HSD17B8/IMPA1/BPNT1/HADHB/ETFB/ENO2/QDPR/NQO2/GSTM4/PRKAB2/PGAM2/PHKA1/GOT1/GMPR/ATP5PF/CPT1B/SIRT5/MECR/ACAT1/GPT/KYAT3/ETFDH</t>
+    <t xml:space="preserve">ETFDH/MT-ATP8/ECI1/STAT5B/MECR/QDPR/BPNT1/AK3/ACADM/MT-ND1/SUCLA2/L2HGDH/ACADSB/MAT2B/ACAT1/NQO2/PRKAA2/SHMT2/ETFB/HADHB/IDH3B/PGP/GMPPB/STOML2/ACADS/CPT1B/SIRT5/ACOT2/THTPA/PPA2/ACSS2/SDHD/PDP1/FBP2/KYAT3/PCBD1/ENO2/NDUFV3/PFKM/IDI1/MPI/DLD/GPT/DCXR/KARS1/FBP1/LDHD/PHKA1/GOT1/PRKAB2/PCBD2/KYAT1/ATP5F1E/NAXD/HSD17B8/RDH13/PTGR2/ATP5F1C/PGAM2/PFKFB1/GSTM4/ATP5PF/GMPR/SFXN1/IMPA1/ATP5F1D/COQ7/THAP4</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006082</t>
@@ -250,7 +250,7 @@
     <t xml:space="preserve">197/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">LDHD/PRKAA2/PCBD1/ACADM/PFKM/ACADSB/NAXD/STAT5B/PDP1/PFKFB1/ACOT2/ECI1/DCXR/KYAT1/L2HGDH/THAP4/DLD/SHMT2/SUCLA2/PTGR2/ACSS2/PPA2/FBP1/IDH3B/ACADS/HSD17B8/BPNT1/HADHB/ETFB/ENO2/GSTM4/PRKAB2/PGAM2/GOT1/CPT1B/MECR/ACAT1/GPT/KYAT3/ETFDH</t>
+    <t xml:space="preserve">ETFDH/ECI1/STAT5B/MECR/BPNT1/ACADM/SUCLA2/L2HGDH/ACADSB/ACAT1/PRKAA2/SHMT2/ETFB/HADHB/IDH3B/ACADS/CPT1B/ACOT2/PPA2/ACSS2/PDP1/KYAT3/PCBD1/ENO2/PFKM/DLD/GPT/DCXR/FBP1/LDHD/GOT1/PRKAB2/KYAT1/NAXD/HSD17B8/PTGR2/PGAM2/PFKFB1/GSTM4/THAP4</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0043436</t>
@@ -265,7 +265,7 @@
     <t xml:space="preserve">196/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">LDHD/PRKAA2/PCBD1/ACADM/PFKM/ACADSB/NAXD/PDP1/PFKFB1/ACOT2/ECI1/DCXR/KYAT1/L2HGDH/THAP4/DLD/SHMT2/SUCLA2/PTGR2/ACSS2/PPA2/FBP1/IDH3B/ACADS/HSD17B8/BPNT1/HADHB/ETFB/ENO2/GSTM4/PRKAB2/PGAM2/GOT1/CPT1B/MECR/ACAT1/GPT/KYAT3/ETFDH</t>
+    <t xml:space="preserve">ETFDH/ECI1/MECR/BPNT1/ACADM/SUCLA2/L2HGDH/ACADSB/ACAT1/PRKAA2/SHMT2/ETFB/HADHB/IDH3B/ACADS/CPT1B/ACOT2/PPA2/ACSS2/PDP1/KYAT3/PCBD1/ENO2/PFKM/DLD/GPT/DCXR/FBP1/LDHD/GOT1/PRKAB2/KYAT1/NAXD/HSD17B8/PTGR2/PGAM2/PFKFB1/GSTM4/THAP4</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0019752</t>
@@ -280,7 +280,7 @@
     <t xml:space="preserve">193/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">LDHD/PRKAA2/PCBD1/ACADM/PFKM/ACADSB/NAXD/PDP1/PFKFB1/ACOT2/ECI1/DCXR/KYAT1/L2HGDH/THAP4/DLD/SHMT2/SUCLA2/PTGR2/ACSS2/FBP1/IDH3B/ACADS/HSD17B8/HADHB/ETFB/ENO2/GSTM4/PRKAB2/PGAM2/GOT1/CPT1B/MECR/ACAT1/GPT/KYAT3/ETFDH</t>
+    <t xml:space="preserve">ETFDH/ECI1/MECR/ACADM/SUCLA2/L2HGDH/ACADSB/ACAT1/PRKAA2/SHMT2/ETFB/HADHB/IDH3B/ACADS/CPT1B/ACOT2/ACSS2/PDP1/KYAT3/PCBD1/ENO2/PFKM/DLD/GPT/DCXR/FBP1/LDHD/GOT1/PRKAB2/KYAT1/NAXD/HSD17B8/PTGR2/PGAM2/PFKFB1/GSTM4/THAP4</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006091</t>
@@ -295,7 +295,7 @@
     <t xml:space="preserve">186/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">PPP1R3A/PRKAA2/ACADM/PFKM/PPP1R1A/UQCRQ/NDUFV3/PNPT1/PDP1/PFKFB1/THTPA/EPM2A/PYGM/MT-ATP8/ATP5F1E/DLD/SHMT2/SUCLA2/ATP5F1C/MT-ND1/ATP5F1D/SDHD/FBP1/IDH3B/STOML2/AGL/ETFB/PHKA2/ENO2/PGAM2/PHKA1/ATP5PF/PPP1R2/PHKB/ACAT1/ETFDH</t>
+    <t xml:space="preserve">ETFDH/MT-ATP8/ACADM/MT-ND1/SUCLA2/ACAT1/PRKAA2/SHMT2/ETFB/IDH3B/STOML2/THTPA/EPM2A/SDHD/UQCRQ/PDP1/PNPT1/ENO2/NDUFV3/PPP1R1A/PFKM/DLD/PPP1R2/PHKB/FBP1/PHKA1/ATP5F1E/PPP1R3A/ATP5F1C/PGAM2/PFKFB1/ATP5PF/PYGM/AGL/PHKA2/ATP5F1D</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0032787</t>
@@ -310,7 +310,7 @@
     <t xml:space="preserve">130/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">LDHD/PRKAA2/ACADM/PFKM/ACADSB/NAXD/PDP1/PFKFB1/ACOT2/ECI1/DCXR/DLD/SHMT2/PTGR2/ACSS2/FBP1/ACADS/HSD17B8/HADHB/ETFB/ENO2/GSTM4/PRKAB2/PGAM2/CPT1B/MECR/ACAT1/ETFDH</t>
+    <t xml:space="preserve">ETFDH/ECI1/MECR/ACADM/ACADSB/ACAT1/PRKAA2/SHMT2/ETFB/HADHB/ACADS/CPT1B/ACOT2/ACSS2/PDP1/ENO2/PFKM/DLD/DCXR/FBP1/LDHD/PRKAB2/NAXD/HSD17B8/PTGR2/PGAM2/PFKFB1/GSTM4</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0015980</t>
@@ -325,7 +325,7 @@
     <t xml:space="preserve">173/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">PPP1R3A/PRKAA2/ACADM/PFKM/PPP1R1A/UQCRQ/NDUFV3/PNPT1/PDP1/PFKFB1/EPM2A/PYGM/MT-ATP8/ATP5F1E/DLD/SHMT2/SUCLA2/ATP5F1C/MT-ND1/ATP5F1D/SDHD/FBP1/IDH3B/STOML2/AGL/ETFB/PHKA2/ENO2/PGAM2/PHKA1/ATP5PF/PPP1R2/PHKB/ETFDH</t>
+    <t xml:space="preserve">ETFDH/MT-ATP8/ACADM/MT-ND1/SUCLA2/PRKAA2/SHMT2/ETFB/IDH3B/STOML2/EPM2A/SDHD/UQCRQ/PDP1/PNPT1/ENO2/NDUFV3/PPP1R1A/PFKM/DLD/PPP1R2/PHKB/FBP1/PHKA1/ATP5F1E/PPP1R3A/ATP5F1C/PGAM2/PFKFB1/ATP5PF/PYGM/AGL/PHKA2/ATP5F1D</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0044282</t>
@@ -340,7 +340,7 @@
     <t xml:space="preserve">100/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">LDHD/ACADM/PFKM/ACADSB/ECI1/DCXR/KYAT1/MPI/DLD/SHMT2/ACSS2/ACADS/HADHB/ETFB/ENO2/NQO2/PGAM2/GOT1/CPT1B/ACAT1/GPT/KYAT3/ETFDH</t>
+    <t xml:space="preserve">ETFDH/ECI1/ACADM/ACADSB/ACAT1/NQO2/SHMT2/ETFB/HADHB/ACADS/CPT1B/ACSS2/KYAT3/ENO2/PFKM/MPI/DLD/GPT/DCXR/LDHD/GOT1/KYAT1/PGAM2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005977</t>
@@ -355,7 +355,7 @@
     <t xml:space="preserve">26/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">PPP1R3A/ACADM/PPP1R1A/EPM2A/PYGM/AGL/PHKA2/PHKA1/PPP1R2/PHKB</t>
+    <t xml:space="preserve">ACADM/EPM2A/PPP1R1A/PPP1R2/PHKB/PHKA1/PPP1R3A/PYGM/AGL/PHKA2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006112</t>
@@ -382,7 +382,7 @@
     <t xml:space="preserve">10/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">PCBD1/PCBD2/PGP/IMPA1/QDPR/GOT1</t>
+    <t xml:space="preserve">QDPR/PGP/PCBD1/GOT1/PCBD2/IMPA1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0044283</t>
@@ -397,7 +397,7 @@
     <t xml:space="preserve">112/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">PRKAA2/PCBD1/ACADM/FBP2/PFKFB1/THTPA/PCBD2/PGP/IDI1/COQ7/SHMT2/SUCLA2/ACSS2/FBP1/HSD17B8/IMPA1/ENO2/QDPR/GSTM4/PRKAB2/PGAM2/GOT1/SIRT5/MECR</t>
+    <t xml:space="preserve">MECR/QDPR/ACADM/SUCLA2/PRKAA2/SHMT2/PGP/SIRT5/THTPA/ACSS2/FBP2/PCBD1/ENO2/IDI1/FBP1/GOT1/PRKAB2/PCBD2/HSD17B8/PGAM2/PFKFB1/GSTM4/IMPA1/COQ7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005976</t>
@@ -421,7 +421,7 @@
     <t xml:space="preserve">204/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">RABGGTA/NAA50/PRKAA2/CAMK2G/RNF7/PFKM/RPS6KA3/MAPK12/AK3/UBE3A/KARS1/PNPT1/GMPPB/PFKFB1/LCMT1/EPM2A/NTMT1/PYGM/KYAT1/UBE2V1/MAP2K6/PCYT2/SHMT2/ARF4/RNF114/ART3/AGL/HADHB/PHKA2/GSTM4/PRKAB2/CKMT1A/PHKA1/GOT1/CPT1B/SIRT5/MYLK2/ACAT1/GPT/KYAT3</t>
+    <t xml:space="preserve">MYLK2/NTMT1/UBE3A/AK3/UBE2V1/RNF114/LCMT1/ACAT1/PRKAA2/SHMT2/RPS6KA3/HADHB/GMPPB/MAP2K6/CPT1B/SIRT5/EPM2A/ARF4/PNPT1/KYAT3/PFKM/PCYT2/GPT/MAPK12/CAMK2G/KARS1/NAA50/CKMT1A/PHKA1/GOT1/PRKAB2/RABGGTA/KYAT1/ART3/RNF7/PFKFB1/GSTM4/PYGM/AGL/PHKA2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030170</t>
@@ -436,7 +436,7 @@
     <t xml:space="preserve">14/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">PHYKPL/PYGM/KYAT1/SHMT2/GOT1/GPT/KYAT3</t>
+    <t xml:space="preserve">PHYKPL/SHMT2/KYAT3/GPT/GOT1/KYAT1/PYGM</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0070279</t>
@@ -457,7 +457,7 @@
     <t xml:space="preserve">20/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">ERO1A/LDHD/ACADM/ACADSB/DLD/ACADS/NQO2/ETFDH</t>
+    <t xml:space="preserve">ETFDH/ACADM/ACADSB/ERO1A/NQO2/ACADS/DLD/LDHD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0042578</t>
@@ -472,7 +472,7 @@
     <t xml:space="preserve">55/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">PPM1B/CAMK2G/PLCD4/FBP2/PDP1/PFKFB1/DUSP3/EPM2A/PGP/PPA2/FBP1/IMPA1/BPNT1/PLCL2</t>
+    <t xml:space="preserve">BPNT1/PLCL2/PGP/DUSP3/EPM2A/PPA2/PDP1/FBP2/CAMK2G/FBP1/PPM1B/PLCD4/PFKFB1/IMPA1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0007010</t>
@@ -487,7 +487,7 @@
     <t xml:space="preserve">221/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">CLIC4/ARPC4/CASQ1/TUBB6/ACTR3/RHOA/MSN/ARF1/MAP4/AQP1/CLTC/CAP1/SH3BGRL3/PAK2/DPYSL2/ZYX/PFN1/TUBA1B/FSCN1/SPTBN1/ILK/EPB41L2/TPM4/DYNC1H1/TAGLN2/MYH9/TUBB/RAC1/PARVA/TLN1/CLIP2/PDLIM1/FKBP4/NUDC/TPPP3/PDCD6IP/ACTR2/SKP1/MAPRE1/RAN/PFN2/CHMP2A/SYNE2/ADD1/TUBA4A</t>
+    <t xml:space="preserve">CLTC/TPM4/ACTR3/PFN2/FKBP4/TUBA4A/CLIC4/MSN/MAP4/AQP1/CASQ1/DYNC1H1/FSCN1/ARF1/PFN1/TUBB/ZYX/SPTBN1/TLN1/CLIP2/TPPP3/CHMP2A/RAC1/SH3BGRL3/PAK2/ARPC4/ACTR2/PDLIM1/SKP1/SYNE2/PDCD6IP/TUBA1B/MYH9/TAGLN2/RHOA/ADD1/MAPRE1/RAN/TUBB6/PARVA/ILK/DPYSL2/EPB41L2/NUDC/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0016477</t>
@@ -502,7 +502,7 @@
     <t xml:space="preserve">125/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">CLIC4/RHOA/MSN/HSPA5/MPP1/STAT3/PAK2/FERMT3/PPIA/PFN1/IFITM1/FSCN1/HSPA8/HSP90AA1/CTSG/MYH9/RAC1/PARVA/GNAI2/P4HB/PDLIM1/S100A11/ANXA3/MAPRE1/PFN2/ARHGDIB/SYNE2/DDT</t>
+    <t xml:space="preserve">PPIA/ARHGDIB/HSPA5/PFN2/CLIC4/MSN/DDT/FSCN1/PFN1/MPP1/P4HB/HSPA8/IFITM1/S100A11/GNAI2/RAC1/PAK2/STAT3/PDLIM1/SYNE2/HSP90AA1/MYH9/RHOA/ANXA3/MAPRE1/CTSG/PARVA/FERMT3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0044087</t>
@@ -517,7 +517,7 @@
     <t xml:space="preserve">132/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RAB1B/ACTR3/RHOA/MSN/RAB7A/HSPA5/VPS35/MAP4/PAK2/RAB11B/PFN1/FSCN1/SPTBN1/HSPA8/HSP90AA1/DYNC1H1/RAC1/TLN1/FKBP4/TPPP3/PDCD6IP/SEC22B/PSMC6/ACTR2/MAPRE1/PFN2/CHMP2A/SYNE2/ADD1</t>
+    <t xml:space="preserve">PSMC6/RAB7A/ACTR3/HSPA5/PFN2/FKBP4/MSN/MAP4/DYNC1H1/FSCN1/PFN1/SEC22B/HSPA8/SPTBN1/TLN1/TPPP3/CHMP2A/RAC1/PAK2/ACTR2/RAB1B/VPS35/SYNE2/PDCD6IP/HSP90AA1/RHOA/ADD1/MAPRE1/RAB11B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0007163</t>
@@ -532,7 +532,7 @@
     <t xml:space="preserve">31/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">CLIC4/RHOA/MSN/MAP4/AQP1/CAP1/FSCN1/RAC1/PARVA/PDLIM1/PDCD6IP/MAPRE1</t>
+    <t xml:space="preserve">CLIC4/MSN/MAP4/AQP1/FSCN1/RAC1/PDLIM1/PDCD6IP/RHOA/MAPRE1/PARVA/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0000226</t>
@@ -547,7 +547,7 @@
     <t xml:space="preserve">76/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">TUBB6/RHOA/MAP4/CLTC/TUBA1B/ILK/DYNC1H1/TUBB/TLN1/CLIP2/FKBP4/NUDC/TPPP3/PDCD6IP/SKP1/MAPRE1/RAN/CHMP2A/SYNE2/TUBA4A</t>
+    <t xml:space="preserve">CLTC/FKBP4/TUBA4A/MAP4/DYNC1H1/TUBB/TLN1/CLIP2/TPPP3/CHMP2A/SKP1/SYNE2/PDCD6IP/TUBA1B/RHOA/MAPRE1/RAN/TUBB6/ILK/NUDC</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0051301</t>
@@ -562,7 +562,7 @@
     <t xml:space="preserve">67/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RHOA/ARF1/MAP4/CLTC/TUBA1B/SPTBN1/EPB41L2/DYNC1H1/MYH9/TUBB/GNAI2/NUDC/PDCD6IP/MAPRE1/RAN/HDGF/CHMP2A/CALM1</t>
+    <t xml:space="preserve">CLTC/HDGF/CALM1/MAP4/DYNC1H1/ARF1/TUBB/SPTBN1/GNAI2/CHMP2A/PDCD6IP/TUBA1B/MYH9/RHOA/MAPRE1/RAN/EPB41L2/NUDC</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0031344</t>
@@ -577,7 +577,7 @@
     <t xml:space="preserve">56/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTR3/SHOC2/VPS35/MAP4/PAK2/RAB11B/EHD1/PFN1/FSCN1/HSP90AA1/RAC1/FKBP4/ACTR2/PFN2/SYNE2/KCTD12</t>
+    <t xml:space="preserve">ACTR3/PFN2/FKBP4/KCTD12/MAP4/EHD1/FSCN1/PFN1/SHOC2/RAC1/PAK2/ACTR2/VPS35/SYNE2/HSP90AA1/RAB11B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0120035</t>
@@ -598,7 +598,7 @@
     <t xml:space="preserve">40/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">ARPC4/CASQ1/MAP4/PFN1/SPTBN1/HSP90AA1/RAC1/FKBP4/TPPP3/MAPRE1/PFN2/CHMP2A/ADD1</t>
+    <t xml:space="preserve">PFN2/FKBP4/MAP4/CASQ1/PFN1/SPTBN1/TPPP3/CHMP2A/RAC1/ARPC4/HSP90AA1/ADD1/MAPRE1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0097435</t>
@@ -610,7 +610,7 @@
     <t xml:space="preserve">142/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">ARPC4/CASQ1/ACTR3/RHOA/ARF1/MAP4/CAP1/PAK2/ZYX/PFN1/FSCN1/SPTBN1/HSPA8/HSP90AB1/ILK/TPM4/DYNC1H1/TAGLN2/RAC1/PARVA/TLN1/CLIP2/PDLIM1/FKBP4/TPPP3/ACTR2/MAPRE1/PFN2/ADD1</t>
+    <t xml:space="preserve">TPM4/ACTR3/PFN2/FKBP4/MAP4/CASQ1/DYNC1H1/FSCN1/ARF1/PFN1/ZYX/HSPA8/SPTBN1/TLN1/CLIP2/TPPP3/RAC1/PAK2/ARPC4/ACTR2/PDLIM1/HSP90AB1/TAGLN2/RHOA/ADD1/MAPRE1/PARVA/ILK/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0033043</t>
@@ -625,7 +625,7 @@
     <t xml:space="preserve">150/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">CLIC4/VAT1/RAB1B/RHOA/MSN/RAB7A/ARF1/VPS35/MAP4/CLTC/PAK2/RAB11B/PFN1/FSCN1/SPTBN1/CCT3/CCT8/HSP90AA1/DYNC1H1/RAC1/HNRNPD/FKBP4/PDCD6IP/SEC22B/MAPRE1/PFN2/CHMP2A/SYNE2/ADD1/HNRNPC</t>
+    <t xml:space="preserve">CLTC/RAB7A/HNRNPC/PFN2/FKBP4/CLIC4/MSN/CCT8/MAP4/DYNC1H1/FSCN1/VAT1/ARF1/PFN1/SEC22B/CCT3/SPTBN1/CHMP2A/RAC1/PAK2/RAB1B/VPS35/SYNE2/PDCD6IP/HSP90AA1/RHOA/ADD1/MAPRE1/HNRNPD/RAB11B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0051017</t>
@@ -637,7 +637,7 @@
     <t xml:space="preserve">11/159</t>
   </si>
   <si>
-    <t xml:space="preserve">RHOA/PAK2/ZYX/PFN1/FSCN1/ILK/RAC1/PARVA/PDLIM1/PFN2/ADD1</t>
+    <t xml:space="preserve">PFN2/FSCN1/PFN1/ZYX/RAC1/PAK2/PDLIM1/RHOA/ADD1/PARVA/ILK</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0061572</t>
@@ -658,7 +658,7 @@
     <t xml:space="preserve">77/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">ARPC4/ACTR3/RHOA/ARF1/CAP1/PAK2/ZYX/PFN1/FSCN1/SPTBN1/ILK/TPM4/TAGLN2/RAC1/PARVA/PDLIM1/ACTR2/PFN2/ADD1</t>
+    <t xml:space="preserve">TPM4/ACTR3/PFN2/FSCN1/ARF1/PFN1/ZYX/SPTBN1/RAC1/PAK2/ARPC4/ACTR2/PDLIM1/TAGLN2/RHOA/ADD1/PARVA/ILK/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0060491</t>
@@ -673,7 +673,7 @@
     <t xml:space="preserve">27/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTR3/MAP4/RAB11B/PFN1/FSCN1/HSP90AA1/RAC1/ACTR2/PFN2/SYNE2</t>
+    <t xml:space="preserve">ACTR3/PFN2/MAP4/FSCN1/PFN1/RAC1/ACTR2/SYNE2/HSP90AA1/RAB11B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0120032</t>
@@ -691,7 +691,7 @@
     <t xml:space="preserve">24/159</t>
   </si>
   <si>
-    <t xml:space="preserve">CLIC4/RHOA/MSN/HSPA5/MPP1/STAT3/VPS35/FERMT3/PPIA/PFN1/IFITM1/HSPA8/CTSG/RAC1/PARVA/GNAI2/P4HB/S100A11/USP14/ANXA3/PFN2/ARHGDIB/SYNE2/DDT</t>
+    <t xml:space="preserve">PPIA/ARHGDIB/HSPA5/PFN2/CLIC4/MSN/DDT/PFN1/MPP1/P4HB/HSPA8/IFITM1/S100A11/GNAI2/RAC1/VPS35/STAT3/SYNE2/RHOA/USP14/ANXA3/CTSG/PARVA/FERMT3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0070527</t>
@@ -706,7 +706,7 @@
     <t xml:space="preserve">19/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">CLIC1/FERMT3/PPIA/ILK/CTSG/MYH9/TLN1/TMX1</t>
+    <t xml:space="preserve">PPIA/TMX1/TLN1/CLIC1/MYH9/CTSG/ILK/FERMT3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0048870</t>
@@ -718,7 +718,7 @@
     <t xml:space="preserve">153/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">CLIC4/ACTR3/RHOA/MSN/HSPA5/MPP1/STAT3/PAK2/FERMT3/PPIA/PFN1/IFITM1/FSCN1/HSPA8/HSP90AA1/CTSG/MYH9/RAC1/PARVA/GNAI2/P4HB/PDLIM1/S100A11/ANXA3/MAPRE1/PFN2/ARHGDIB/SYNE2/DDT</t>
+    <t xml:space="preserve">PPIA/ACTR3/ARHGDIB/HSPA5/PFN2/CLIC4/MSN/DDT/FSCN1/PFN1/MPP1/P4HB/HSPA8/IFITM1/S100A11/GNAI2/RAC1/PAK2/STAT3/PDLIM1/SYNE2/HSP90AA1/MYH9/RHOA/ANXA3/MAPRE1/CTSG/PARVA/FERMT3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0051128</t>
@@ -733,7 +733,7 @@
     <t xml:space="preserve">304/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">CLIC4/FLOT1/VAT1/RAB1B/ACTR3/RHOA/MSN/RAB7A/SHOC2/ARF1/HSPA5/STAT3/VPS35/MAP4/CLTC/PAK2/RAB11B/EHD1/PFN1/AHNAK/FSCN1/SPTBN1/CCT3/HSPA8/ETF1/RPL36/CCT8/HSP90AA1/DYNC1H1/MYH9/TUBB/RAC1/HNRNPD/TLN1/FKBP4/TPPP3/PDCD6IP/SEC22B/PSMC6/ACTR2/SKP1/MAPRE1/PFN2/CHMP2A/SYNE2/KCTD12/ADD1/HNRNPC</t>
+    <t xml:space="preserve">AHNAK/PSMC6/CLTC/RAB7A/ACTR3/HNRNPC/FLOT1/HSPA5/PFN2/FKBP4/CLIC4/MSN/KCTD12/ETF1/CCT8/MAP4/EHD1/DYNC1H1/FSCN1/VAT1/ARF1/PFN1/TUBB/SEC22B/SHOC2/HSPA8/CCT3/SPTBN1/TLN1/TPPP3/CHMP2A/RAC1/PAK2/ACTR2/RAB1B/VPS35/STAT3/SKP1/SYNE2/PDCD6IP/HSP90AA1/MYH9/RHOA/ADD1/MAPRE1/HNRNPD/RPL36/RAB11B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030031</t>
@@ -745,7 +745,7 @@
     <t xml:space="preserve">46/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTR3/MAP4/RAB11B/EHD1/PFN1/FSCN1/HSP90AA1/RAC1/PARVA/ACTR2/SKP1/PFN2/SYNE2</t>
+    <t xml:space="preserve">ACTR3/PFN2/MAP4/EHD1/FSCN1/PFN1/RAC1/ACTR2/SKP1/SYNE2/HSP90AA1/PARVA/RAB11B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0120031</t>
@@ -775,7 +775,7 @@
     <t xml:space="preserve">99/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">CLIC4/RHOA/MSN/HSPA5/MPP1/STAT3/VPS35/FERMT3/PFN1/IFITM1/HSPA8/RAC1/GNAI2/P4HB/S100A11/USP14/ANXA3/PFN2/ARHGDIB/SYNE2/DDT</t>
+    <t xml:space="preserve">ARHGDIB/HSPA5/PFN2/CLIC4/MSN/DDT/PFN1/MPP1/P4HB/HSPA8/IFITM1/S100A11/GNAI2/RAC1/VPS35/STAT3/SYNE2/RHOA/USP14/ANXA3/FERMT3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0044089</t>
@@ -790,7 +790,7 @@
     <t xml:space="preserve">61/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTR3/RHOA/RAB7A/PFN1/FSCN1/HSP90AA1/DYNC1H1/RAC1/TPPP3/PDCD6IP/PSMC6/ACTR2/MAPRE1/PFN2/CHMP2A</t>
+    <t xml:space="preserve">PSMC6/RAB7A/ACTR3/PFN2/DYNC1H1/FSCN1/PFN1/TPPP3/CHMP2A/RAC1/ACTR2/PDCD6IP/HSP90AA1/RHOA/MAPRE1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030038</t>
@@ -805,7 +805,7 @@
     <t xml:space="preserve">17/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RHOA/PAK2/ZYX/PFN1/RAC1/PDLIM1/PFN2</t>
+    <t xml:space="preserve">PFN2/PFN1/ZYX/RAC1/PAK2/PDLIM1/RHOA</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0043149</t>
@@ -826,7 +826,7 @@
     <t xml:space="preserve">131/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">ARPC4/CASQ1/ACTR3/RHOA/ARF1/AQP1/CAP1/PAK2/ZYX/PFN1/FSCN1/SPTBN1/ILK/EPB41L2/TPM4/TAGLN2/MYH9/RAC1/PARVA/TLN1/PDLIM1/PDCD6IP/ACTR2/PFN2/ADD1</t>
+    <t xml:space="preserve">TPM4/ACTR3/PFN2/AQP1/CASQ1/FSCN1/ARF1/PFN1/ZYX/SPTBN1/TLN1/RAC1/PAK2/ARPC4/ACTR2/PDLIM1/PDCD6IP/MYH9/TAGLN2/RHOA/ADD1/PARVA/ILK/EPB41L2/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0034109</t>
@@ -847,7 +847,7 @@
     <t xml:space="preserve">38/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">HNRNPUL2/QKI/ILF3/HSPA8/STRAP/PRDX6/SRSF3/HNRNPK/HNRNPL/HNRNPA3/HNRNPC</t>
+    <t xml:space="preserve">HNRNPC/HNRNPUL2/PRDX6/SRSF3/HNRNPK/HSPA8/ILF3/HNRNPA3/HNRNPL/QKI/STRAP</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0000377</t>
@@ -874,7 +874,7 @@
     <t xml:space="preserve">484/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">CLIC4/ARPC4/CASQ1/ATP6V1G1/TUBB6/VAT1/RAB1B/ACTR3/RHOA/MSN/RAB7A/ARF1/VPS35/MAP4/AQP1/CSDE1/CLTC/CAP1/SH3BGRL3/PAK2/DPYSL2/RAB11B/ZYX/EHD1/PPIA/PFN1/VAMP3/TUBA1B/FSCN1/SPTBN1/CCT3/HSP90AB1/H1-5/ILK/EPB41L2/TPM4/CCT8/HSP90AA1/DYNC1H1/TAGLN2/MYH9/TUBB/RAC1/HNRNPD/PARVA/TLN1/CLIP2/RPA2/TRAPPC3/LPCAT3/PDLIM1/FKBP4/HSPA9/NUDC/TPPP3/PDCD6IP/SEC22B/ACTR2/SKP1/MAPRE1/RAN/PFN2/CHMP2A/SYNE2/ADD1/HNRNPC/TUBA4A</t>
+    <t xml:space="preserve">CLTC/PPIA/RAB7A/TPM4/ACTR3/HSPA9/HNRNPC/CSDE1/PFN2/FKBP4/TUBA4A/TRAPPC3/CLIC4/MSN/RPA2/CCT8/MAP4/AQP1/CASQ1/EHD1/DYNC1H1/FSCN1/VAT1/ARF1/PFN1/LPCAT3/TUBB/SEC22B/ZYX/VAMP3/CCT3/SPTBN1/TLN1/CLIP2/ATP6V1G1/TPPP3/CHMP2A/RAC1/SH3BGRL3/PAK2/ARPC4/ACTR2/RAB1B/VPS35/PDLIM1/SKP1/SYNE2/PDCD6IP/HSP90AA1/H1-5/HSP90AB1/TUBA1B/MYH9/TAGLN2/RHOA/ADD1/MAPRE1/RAN/TUBB6/PARVA/HNRNPD/ILK/DPYSL2/RAB11B/EPB41L2/NUDC/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005856</t>
@@ -889,7 +889,7 @@
     <t xml:space="preserve">300/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">DCTN4/CLIC4/ARPC4/SYNC/TUBB6/FLOT1/ACTR3/RHOA/MSN/LASP1/MPP1/MAP4/CLTC/CAP1/DPYSL2/FERMT3/ZYX/PFN1/TUBA1B/AHNAK/FSCN1/SPTBN1/CCT3/ARHGDIA/ILK/EPB41L2/TPM4/CCT8/DYNC1H1/PALMD/TAGLN2/MYH9/TUBB/RAC1/PARVA/GNAI2/TLN1/CLIP2/P4HB/HNRNPK/PDLIM1/FKBP4/NUDC/TPPP3/PDCD6IP/ACTR2/SKP1/MYL12B/MAPRE1/RAN/PFN2/CHMP2A/ARHGDIB/SYNE2/ADD1/HNRNPC/TUBA4A/CALM1</t>
+    <t xml:space="preserve">AHNAK/CLTC/TPM4/ACTR3/HNRNPC/LASP1/ARHGDIB/FLOT1/PFN2/FKBP4/TUBA4A/CALM1/CLIC4/MSN/DCTN4/CCT8/MAP4/PALMD/DYNC1H1/FSCN1/PFN1/MPP1/HNRNPK/P4HB/TUBB/ZYX/ARHGDIA/CCT3/SPTBN1/GNAI2/TLN1/CLIP2/TPPP3/CHMP2A/SYNC/RAC1/ARPC4/ACTR2/PDLIM1/SKP1/SYNE2/PDCD6IP/MYL12B/TUBA1B/MYH9/TAGLN2/RHOA/ADD1/MAPRE1/RAN/TUBB6/PARVA/ILK/DPYSL2/FERMT3/EPB41L2/NUDC/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0042470</t>
@@ -904,7 +904,7 @@
     <t xml:space="preserve">46/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">GANAB/ANXA6/FLOT1/RAB7A/CANX/HSPA5/CLTC/HSPA8/HSP90AB1/HSP90AA1/RAC1/RAB5C/P4HB/NAP1L1/PDCD6IP/SEC22B/RAN</t>
+    <t xml:space="preserve">CLTC/RAB7A/FLOT1/HSPA5/CANX/RAB5C/ANXA6/P4HB/SEC22B/HSPA8/NAP1L1/RAC1/GANAB/PDCD6IP/HSP90AA1/HSP90AB1/RAN</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0048770</t>
@@ -925,7 +925,7 @@
     <t xml:space="preserve">159/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">DCTN4/ANXA6/FLOT1/ACTR3/RHOA/MSN/LASP1/ARF1/HSPA5/CLTC/CAP1/FERMT3/ZYX/PPIA/PFN1/AHNAK/HSPA8/ILK/EPB41L2/TPM4/MYH9/RAC1/PARVA/TLN1/P4HB/HNRNPK/PDLIM1/HSPA9/YWHAQ/LAP3/LAMTOR3/PDCD6IP/ACTR2/MAPRE1/SYNE2/ADD1</t>
+    <t xml:space="preserve">AHNAK/CLTC/PPIA/LAP3/TPM4/ACTR3/HSPA9/LASP1/FLOT1/HSPA5/MSN/DCTN4/ANXA6/ARF1/PFN1/HNRNPK/P4HB/ZYX/HSPA8/TLN1/YWHAQ/RAC1/ACTR2/PDLIM1/SYNE2/LAMTOR3/PDCD6IP/MYH9/RHOA/ADD1/MAPRE1/PARVA/ILK/FERMT3/EPB41L2/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030054</t>
@@ -940,7 +940,7 @@
     <t xml:space="preserve">397/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">DCTN4/CLIC4/SYNC/ANXA6/ATP6V1G1/HNRNPUL2/FLOT1/PURA/QKI/ACTR3/RHOA/MSN/RAB7A/LASP1/CANX/ARF1/HSPA5/MPP1/STAT3/VPS35/MOB4/CLTC/CAP1/PAK2/RAB11B/FERMT3/ZYX/EHD1/AKR1A1/PPIA/PFN1/VAMP3/AHNAK/FSCN1/SPTBN1/ARHGDIA/HSPA8/RPL36/ILK/EPB41L2/TPM4/PALMD/MYH9/RAC1/HNRNPD/PARVA/GNAI2/TLN1/P4HB/HNRNPK/PDLIM1/HSPA9/YWHAQ/HNRNPL/LAP3/S100A11/LAMTOR3/PDCD6IP/PSMC6/ACTR2/USP14/MAPRE1/PFN2/SYNE2/KCTD12/ADD1/CALM1</t>
+    <t xml:space="preserve">AHNAK/PSMC6/CLTC/PPIA/LAP3/RAB7A/TPM4/ACTR3/HSPA9/LASP1/FLOT1/HSPA5/PFN2/PURA/CALM1/CLIC4/MSN/CANX/DCTN4/KCTD12/HNRNPUL2/ANXA6/EHD1/PALMD/FSCN1/ARF1/PFN1/MPP1/HNRNPK/P4HB/ZYX/HSPA8/ARHGDIA/VAMP3/SPTBN1/S100A11/GNAI2/TLN1/ATP6V1G1/YWHAQ/HNRNPL/SYNC/RAC1/PAK2/ACTR2/MOB4/VPS35/STAT3/PDLIM1/AKR1A1/SYNE2/LAMTOR3/PDCD6IP/QKI/MYH9/RHOA/ADD1/USP14/MAPRE1/PARVA/HNRNPD/ILK/RPL36/RAB11B/FERMT3/EPB41L2/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0071944</t>
@@ -955,7 +955,7 @@
     <t xml:space="preserve">426/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">DCTN4/CLIC4/TMX3/RRAD/SYNC/ANXA6/CASQ1/ATP6V1G1/FLOT1/RHOA/MSN/RAB7A/LASP1/ARF1/HSPA5/HLA-B/MPP1/CLIC1/STAT3/AQP1/CLTC/CAP1/SH3BGRL3/SH3BGRL/PAK2/EHD1/AKR1A1/PPIA/PFN1/IFITM1/VAMP3/AHNAK/FSCN1/SPTBN1/ARHGDIA/HSPA8/HSP90AB1/COMT/ILK/EPB41L2/TPM4/HSP90AA1/HLA-A/DYNC1H1/ARHGAP1/CTSG/MYH9/RAC1/PARVA/GNAI2/TLN1/CLIP2/RAB5C/P4HB/S100A6/LAMTOR3/PDCD6IP/ARHGAP19/GSR/ACTR2/MYL12B/USP14/ANXA3/MAPRE1/CHMP2A/SPPL2A/SYNE2/KCTD12/ADD1/CALM1</t>
+    <t xml:space="preserve">AHNAK/CLTC/PPIA/RAB7A/RRAD/TPM4/HLA-A/LASP1/FLOT1/HSPA5/CALM1/TMX3/CLIC4/MSN/SPPL2A/DCTN4/KCTD12/RAB5C/COMT/AQP1/CASQ1/ANXA6/EHD1/DYNC1H1/FSCN1/ARF1/PFN1/ARHGAP19/MPP1/P4HB/HSPA8/ARHGDIA/VAMP3/IFITM1/SPTBN1/S100A6/GNAI2/TLN1/CLIP2/ATP6V1G1/CHMP2A/SYNC/RAC1/SH3BGRL3/PAK2/SH3BGRL/GSR/ACTR2/STAT3/AKR1A1/CLIC1/SYNE2/LAMTOR3/PDCD6IP/HSP90AA1/MYL12B/HSP90AB1/MYH9/RHOA/ADD1/USP14/ANXA3/MAPRE1/HLA-B/CTSG/ARHGAP1/PARVA/ILK/EPB41L2/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005925</t>
@@ -970,7 +970,7 @@
     <t xml:space="preserve">156/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">DCTN4/ANXA6/FLOT1/ACTR3/RHOA/MSN/LASP1/ARF1/HSPA5/CLTC/CAP1/ZYX/PPIA/PFN1/AHNAK/HSPA8/ILK/EPB41L2/TPM4/MYH9/RAC1/PARVA/TLN1/P4HB/HNRNPK/PDLIM1/HSPA9/YWHAQ/LAP3/LAMTOR3/PDCD6IP/ACTR2/MAPRE1/SYNE2/ADD1</t>
+    <t xml:space="preserve">AHNAK/CLTC/PPIA/LAP3/TPM4/ACTR3/HSPA9/LASP1/FLOT1/HSPA5/MSN/DCTN4/ANXA6/ARF1/PFN1/HNRNPK/P4HB/ZYX/HSPA8/TLN1/YWHAQ/RAC1/ACTR2/PDLIM1/SYNE2/LAMTOR3/PDCD6IP/MYH9/RHOA/ADD1/MAPRE1/PARVA/ILK/EPB41L2/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0070161</t>
@@ -985,7 +985,7 @@
     <t xml:space="preserve">200/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">DCTN4/CLIC4/ANXA6/FLOT1/ACTR3/RHOA/MSN/LASP1/ARF1/HSPA5/MPP1/CLTC/CAP1/PAK2/FERMT3/ZYX/PPIA/PFN1/AHNAK/FSCN1/HSPA8/ILK/EPB41L2/TPM4/MYH9/RAC1/PARVA/TLN1/P4HB/HNRNPK/PDLIM1/HSPA9/YWHAQ/LAP3/S100A11/LAMTOR3/PDCD6IP/ACTR2/MAPRE1/SYNE2/ADD1</t>
+    <t xml:space="preserve">AHNAK/CLTC/PPIA/LAP3/TPM4/ACTR3/HSPA9/LASP1/FLOT1/HSPA5/CLIC4/MSN/DCTN4/ANXA6/FSCN1/ARF1/PFN1/MPP1/HNRNPK/P4HB/ZYX/HSPA8/S100A11/TLN1/YWHAQ/RAC1/PAK2/ACTR2/PDLIM1/SYNE2/LAMTOR3/PDCD6IP/MYH9/RHOA/ADD1/MAPRE1/PARVA/ILK/FERMT3/EPB41L2/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005886</t>
@@ -1000,7 +1000,7 @@
     <t xml:space="preserve">386/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">CLIC4/TMX3/RRAD/SYNC/ANXA6/CASQ1/ATP6V1G1/FLOT1/RHOA/MSN/RAB7A/ARF1/HSPA5/HLA-B/MPP1/CLIC1/STAT3/AQP1/CLTC/CAP1/SH3BGRL3/SH3BGRL/PAK2/EHD1/AKR1A1/PPIA/IFITM1/VAMP3/AHNAK/FSCN1/SPTBN1/ARHGDIA/HSPA8/HSP90AB1/COMT/ILK/EPB41L2/HSP90AA1/HLA-A/ARHGAP1/CTSG/MYH9/RAC1/PARVA/GNAI2/TLN1/RAB5C/P4HB/S100A6/LAMTOR3/PDCD6IP/ARHGAP19/GSR/USP14/ANXA3/MAPRE1/CHMP2A/SPPL2A/SYNE2/KCTD12/ADD1/CALM1</t>
+    <t xml:space="preserve">AHNAK/CLTC/PPIA/RAB7A/RRAD/HLA-A/FLOT1/HSPA5/CALM1/TMX3/CLIC4/MSN/SPPL2A/KCTD12/RAB5C/COMT/AQP1/CASQ1/ANXA6/EHD1/FSCN1/ARF1/ARHGAP19/MPP1/P4HB/HSPA8/ARHGDIA/VAMP3/IFITM1/SPTBN1/S100A6/GNAI2/TLN1/ATP6V1G1/CHMP2A/SYNC/RAC1/SH3BGRL3/PAK2/SH3BGRL/GSR/STAT3/AKR1A1/CLIC1/SYNE2/LAMTOR3/PDCD6IP/HSP90AA1/HSP90AB1/MYH9/RHOA/ADD1/USP14/ANXA3/MAPRE1/HLA-B/CTSG/ARHGAP1/PARVA/ILK/EPB41L2/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0031410</t>
@@ -1015,7 +1015,7 @@
     <t xml:space="preserve">328/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">CLIC4/TMX3/GANAB/ANXA6/ATP6V1G1/FLOT1/VAT1/RAB1B/COPB2/RHOA/RAB7A/CANX/HSPA5/HLA-B/VPS35/CLTC/CAP1/PAK2/RAB11B/FERMT3/ZYX/EHD1/PPIA/FTL/VAMP3/HSPA8/HSP90AB1/MPO/CCT8/HSP90AA1/HLA-A/DYNC1H1/ARHGAP1/CTSG/MYH9/TUBB/RAC1/GNAI2/RAB5C/PRDX6/P4HB/ERP44/NAP1L1/S100A11/LAMTOR3/PDCD6IP/SEC22B/PSMC6/ACTR2/USP14/ANXA3/RAN/CHMP2A/SPPL2A/ARHGDIB</t>
+    <t xml:space="preserve">PSMC6/CLTC/PPIA/RAB7A/HLA-A/ARHGDIB/FLOT1/HSPA5/ERP44/TMX3/CLIC4/SPPL2A/CANX/RAB5C/CCT8/ANXA6/EHD1/DYNC1H1/PRDX6/VAT1/P4HB/TUBB/SEC22B/ZYX/HSPA8/COPB2/VAMP3/S100A11/NAP1L1/GNAI2/ATP6V1G1/CHMP2A/RAC1/GANAB/PAK2/ACTR2/RAB1B/VPS35/LAMTOR3/PDCD6IP/HSP90AA1/HSP90AB1/MPO/MYH9/RHOA/FTL/USP14/ANXA3/RAN/HLA-B/CTSG/ARHGAP1/RAB11B/FERMT3/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0097708</t>
@@ -1039,7 +1039,7 @@
     <t xml:space="preserve">33/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">RHOA/MSN/AQP1/SH3BGRL3/EHD1/FSCN1/SPTBN1/HSP90AA1/RAC1/TLN1/MAPRE1/SYNE2</t>
+    <t xml:space="preserve">MSN/AQP1/EHD1/FSCN1/SPTBN1/TLN1/RAC1/SH3BGRL3/SYNE2/HSP90AA1/RHOA/MAPRE1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005938</t>
@@ -1054,7 +1054,7 @@
     <t xml:space="preserve">74/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">DCTN4/FLOT1/RHOA/LASP1/MPP1/CAP1/PFN1/FSCN1/SPTBN1/ILK/EPB41L2/TPM4/DYNC1H1/MYH9/RAC1/CLIP2/ACTR2/MYL12B/MAPRE1</t>
+    <t xml:space="preserve">TPM4/LASP1/FLOT1/DCTN4/DYNC1H1/FSCN1/PFN1/MPP1/SPTBN1/CLIP2/RAC1/ACTR2/MYL12B/MYH9/RHOA/MAPRE1/ILK/EPB41L2/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0000323</t>
@@ -1069,7 +1069,7 @@
     <t xml:space="preserve">115/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">ANXA6/ATP6V1G1/FLOT1/VAT1/RAB7A/VPS35/CLTC/CAP1/FTL/IFITM1/AHNAK/HSPA8/MPO/CCT8/HSP90AA1/DYNC1H1/CTSG/TUBB/RAB5C/PRDX6/LAMTOR3/SEC22B/ACTR2/CHMP2A/SPPL2A</t>
+    <t xml:space="preserve">AHNAK/CLTC/RAB7A/FLOT1/SPPL2A/RAB5C/CCT8/ANXA6/DYNC1H1/PRDX6/VAT1/TUBB/SEC22B/HSPA8/IFITM1/ATP6V1G1/CHMP2A/ACTR2/VPS35/LAMTOR3/HSP90AA1/MPO/FTL/CTSG/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005764</t>
@@ -1087,7 +1087,7 @@
     <t xml:space="preserve">233/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">CLIC4/ARPC4/FLOT1/PURA/ACTR3/RHOA/MSN/ARF1/MPP1/VPS35/MAP4/AQP1/SH3BGRL3/DPYSL2/EHD1/VAMP3/TUBA1B/FSCN1/SPTBN1/HSP90AB1/COMT/ILK/HSP90AA1/DYNC1H1/PALMD/ARHGAP1/MYH9/TUBB/RAC1/GNAI2/TLN1/P4HB/FKBP4/S100A6/S100A11/ACTR2/MAPRE1/RAN/SYNE2/TUBA4A/CALM1</t>
+    <t xml:space="preserve">ACTR3/FLOT1/FKBP4/PURA/TUBA4A/CALM1/CLIC4/MSN/COMT/MAP4/AQP1/EHD1/PALMD/DYNC1H1/FSCN1/ARF1/MPP1/P4HB/TUBB/VAMP3/SPTBN1/S100A11/S100A6/GNAI2/TLN1/RAC1/SH3BGRL3/ARPC4/ACTR2/VPS35/SYNE2/HSP90AA1/HSP90AB1/TUBA1B/MYH9/RHOA/MAPRE1/RAN/ARHGAP1/ILK/DPYSL2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0009986</t>
@@ -1099,7 +1099,7 @@
     <t xml:space="preserve">64/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">CLIC4/TMX3/FLOT1/MSN/HSPA5/HLA-B/VAMP3/HSP90AB1/HSP90AA1/HLA-A/MYH9/APMAP/TLN1/P4HB/ERP44/GSR/USP14</t>
+    <t xml:space="preserve">HLA-A/FLOT1/HSPA5/ERP44/TMX3/CLIC4/MSN/P4HB/VAMP3/TLN1/APMAP/GSR/HSP90AA1/HSP90AB1/MYH9/USP14/HLA-B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0035578</t>
@@ -1114,7 +1114,7 @@
     <t xml:space="preserve">27/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">VAT1/CAP1/FTL/MPO/CCT8/DYNC1H1/CTSG/TUBB/PRDX6/ACTR2</t>
+    <t xml:space="preserve">CCT8/DYNC1H1/PRDX6/VAT1/TUBB/ACTR2/MPO/FTL/CTSG/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005874</t>
@@ -1126,7 +1126,7 @@
     <t xml:space="preserve">66/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">TUBB6/MAP4/CLTC/DPYSL2/TUBA1B/CCT3/CCT8/DYNC1H1/TUBB/CLIP2/FKBP4/NUDC/TPPP3/MAPRE1/CHMP2A/TUBA4A/CALM1</t>
+    <t xml:space="preserve">CLTC/FKBP4/TUBA4A/CALM1/CCT8/MAP4/DYNC1H1/TUBB/CCT3/CLIP2/TPPP3/CHMP2A/TUBA1B/MAPRE1/TUBB6/DPYSL2/NUDC</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030670</t>
@@ -1141,7 +1141,7 @@
     <t xml:space="preserve">14/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">RAB7A/HLA-B/RAB11B/VAMP3/HLA-A/SEC22B/ANXA3</t>
+    <t xml:space="preserve">RAB7A/HLA-A/SEC22B/VAMP3/ANXA3/HLA-B/RAB11B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0120025</t>
@@ -1156,7 +1156,7 @@
     <t xml:space="preserve">228/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">CLIC4/FLOT1/PURA/ACTR3/RHOA/MSN/ARF1/MPP1/VPS35/MAP4/AQP1/SH3BGRL3/DPYSL2/EHD1/VAMP3/TUBA1B/FSCN1/SPTBN1/HSP90AB1/COMT/ILK/HSP90AA1/DYNC1H1/PALMD/ARHGAP1/MYH9/TUBB/RAC1/GNAI2/TLN1/P4HB/FKBP4/S100A6/S100A11/MAPRE1/RAN/SYNE2/TUBA4A/CALM1</t>
+    <t xml:space="preserve">ACTR3/FLOT1/FKBP4/PURA/TUBA4A/CALM1/CLIC4/MSN/COMT/MAP4/AQP1/EHD1/PALMD/DYNC1H1/FSCN1/ARF1/MPP1/P4HB/TUBB/VAMP3/SPTBN1/S100A11/S100A6/GNAI2/TLN1/RAC1/SH3BGRL3/VPS35/SYNE2/HSP90AA1/HSP90AB1/TUBA1B/MYH9/RHOA/MAPRE1/RAN/ARHGAP1/ILK/DPYSL2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0015630</t>
@@ -1171,7 +1171,7 @@
     <t xml:space="preserve">145/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">DCTN4/CLIC4/TUBB6/FLOT1/MAP4/CLTC/DPYSL2/TUBA1B/CCT3/ILK/CCT8/DYNC1H1/MYH9/TUBB/RAC1/GNAI2/TLN1/CLIP2/FKBP4/NUDC/TPPP3/PDCD6IP/SKP1/MAPRE1/RAN/CHMP2A/TUBA4A/CALM1</t>
+    <t xml:space="preserve">CLTC/FLOT1/FKBP4/TUBA4A/CALM1/CLIC4/DCTN4/CCT8/MAP4/DYNC1H1/TUBB/CCT3/GNAI2/TLN1/CLIP2/TPPP3/CHMP2A/RAC1/SKP1/PDCD6IP/TUBA1B/MYH9/MAPRE1/RAN/TUBB6/ILK/DPYSL2/NUDC</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005775</t>
@@ -1183,7 +1183,7 @@
     <t xml:space="preserve">40/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">VAT1/CAP1/FTL/HSPA8/MPO/CCT8/HSP90AA1/DYNC1H1/CTSG/TUBB/PRDX6/ACTR2</t>
+    <t xml:space="preserve">CCT8/DYNC1H1/PRDX6/VAT1/TUBB/HSPA8/ACTR2/HSP90AA1/MPO/FTL/CTSG/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0000785</t>
@@ -1198,7 +1198,7 @@
     <t xml:space="preserve">52/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">STAT3/SET/H1-5/ILK/HNRNPD/RPA2/HNRNPK/HNRNPDL/HNRNPL/NAP1L1/SKP1/RAN/CHMP2A/HNRNPC</t>
+    <t xml:space="preserve">HNRNPC/HNRNPDL/RPA2/SET/HNRNPK/NAP1L1/HNRNPL/CHMP2A/STAT3/SKP1/H1-5/RAN/HNRNPD/ILK</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0031252</t>
@@ -1213,7 +1213,7 @@
     <t xml:space="preserve">65/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">FLOT1/ACTR3/RHOA/ARF1/SH3BGRL3/FSCN1/SPTBN1/ILK/ARHGAP1/MYH9/RAC1/TLN1/P4HB/S100A6/S100A11/SYNE2</t>
+    <t xml:space="preserve">ACTR3/FLOT1/FSCN1/ARF1/P4HB/SPTBN1/S100A11/S100A6/TLN1/RAC1/SH3BGRL3/SYNE2/MYH9/RHOA/ARHGAP1/ILK</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005773</t>
@@ -1237,7 +1237,7 @@
     <t xml:space="preserve">113/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">CLIC4/SYNC/ANXA6/RAB1B/MSN/CLIC1/VPS35/MOB4/PAK2/EHD1/VAMP3/S100A16/SET/HSP90AB1/HSP90AA1/ARHGAP1/S100A13/PRDX6/FKBP4/TPPP3/S100A6/ANP32A/TPD52L2</t>
+    <t xml:space="preserve">ANP32A/FKBP4/TPD52L2/CLIC4/MSN/ANXA6/EHD1/PRDX6/SET/VAMP3/S100A6/TPPP3/SYNC/PAK2/S100A13/RAB1B/MOB4/VPS35/CLIC1/HSP90AA1/HSP90AB1/S100A16/ARHGAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0015629</t>
@@ -1252,7 +1252,7 @@
     <t xml:space="preserve">137/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">DCTN4/CLIC4/ARPC4/FLOT1/ACTR3/LASP1/CAP1/FERMT3/ZYX/AHNAK/FSCN1/SPTBN1/EPB41L2/TPM4/PALMD/TAGLN2/MYH9/RAC1/PARVA/HNRNPK/PDLIM1/PDCD6IP/ACTR2/MYL12B/ADD1/HNRNPC</t>
+    <t xml:space="preserve">AHNAK/TPM4/ACTR3/HNRNPC/LASP1/FLOT1/CLIC4/DCTN4/PALMD/FSCN1/HNRNPK/ZYX/SPTBN1/RAC1/ARPC4/ACTR2/PDLIM1/PDCD6IP/MYL12B/MYH9/TAGLN2/ADD1/PARVA/FERMT3/EPB41L2/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030141</t>
@@ -1267,7 +1267,7 @@
     <t xml:space="preserve">160/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">TMX3/VAT1/RHOA/RAB7A/HLA-B/CAP1/PAK2/FERMT3/PPIA/FTL/VAMP3/HSPA8/HSP90AB1/MPO/CCT8/HSP90AA1/DYNC1H1/CTSG/MYH9/TUBB/RAC1/GNAI2/RAB5C/PRDX6/ERP44/S100A11/LAMTOR3/ACTR2/ANXA3</t>
+    <t xml:space="preserve">PPIA/RAB7A/ERP44/TMX3/RAB5C/CCT8/DYNC1H1/PRDX6/VAT1/TUBB/HSPA8/VAMP3/S100A11/GNAI2/RAC1/PAK2/ACTR2/LAMTOR3/HSP90AA1/HSP90AB1/MPO/MYH9/RHOA/FTL/ANXA3/HLA-B/CTSG/FERMT3/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0010008</t>
@@ -1279,7 +1279,7 @@
     <t xml:space="preserve">15/163</t>
   </si>
   <si>
-    <t xml:space="preserve">ANXA6/RAB7A/HLA-B/VPS35/CLTC/RAB11B/EHD1/VAMP3/HLA-A/ARHGAP1/RAC1/RAB5C/LAMTOR3/CHMP2A/SPPL2A</t>
+    <t xml:space="preserve">CLTC/RAB7A/HLA-A/SPPL2A/RAB5C/ANXA6/EHD1/VAMP3/CHMP2A/RAC1/VPS35/LAMTOR3/HLA-B/ARHGAP1/RAB11B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030863</t>
@@ -1291,7 +1291,7 @@
     <t xml:space="preserve">34/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">FLOT1/LASP1/MPP1/CAP1/SPTBN1/EPB41L2/TPM4/MYH9/ACTR2/MAPRE1</t>
+    <t xml:space="preserve">TPM4/LASP1/FLOT1/MPP1/SPTBN1/ACTR2/MYH9/MAPRE1/EPB41L2/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005911</t>
@@ -1303,7 +1303,7 @@
     <t xml:space="preserve">71/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">CLIC4/FLOT1/ACTR3/RHOA/MSN/MPP1/PAK2/ZYX/AHNAK/FSCN1/MYH9/TLN1/PDLIM1/S100A11/PDCD6IP/ADD1</t>
+    <t xml:space="preserve">AHNAK/ACTR3/FLOT1/CLIC4/MSN/FSCN1/MPP1/ZYX/S100A11/TLN1/PAK2/PDLIM1/PDCD6IP/MYH9/RHOA/ADD1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0045335</t>
@@ -1318,7 +1318,7 @@
     <t xml:space="preserve">29/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">RAB7A/HLA-B/RAB11B/ZYX/VAMP3/MPO/HLA-A/SEC22B/ANXA3</t>
+    <t xml:space="preserve">RAB7A/HLA-A/SEC22B/ZYX/VAMP3/MPO/ANXA3/HLA-B/RAB11B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005766</t>
@@ -1333,7 +1333,7 @@
     <t xml:space="preserve">41/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">VAT1/CAP1/FTL/MPO/CCT8/DYNC1H1/CTSG/TUBB/RAB5C/PRDX6/ACTR2</t>
+    <t xml:space="preserve">RAB5C/CCT8/DYNC1H1/PRDX6/VAT1/TUBB/ACTR2/MPO/FTL/CTSG/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0042582</t>
@@ -1354,7 +1354,7 @@
     <t xml:space="preserve">108/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">SYNC/TUBB6/MAP4/CLTC/DPYSL2/TUBA1B/CCT3/TPM4/CCT8/DYNC1H1/TUBB/RAC1/CLIP2/PDLIM1/FKBP4/NUDC/TPPP3/MAPRE1/CHMP2A/TUBA4A/CALM1</t>
+    <t xml:space="preserve">CLTC/TPM4/FKBP4/TUBA4A/CALM1/CCT8/MAP4/DYNC1H1/TUBB/CCT3/CLIP2/TPPP3/CHMP2A/SYNC/RAC1/PDLIM1/TUBA1B/MAPRE1/TUBB6/DPYSL2/NUDC</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030659</t>
@@ -1369,7 +1369,7 @@
     <t xml:space="preserve">133/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">CLIC4/TMX3/ANXA6/ATP6V1G1/COPB2/RHOA/RAB7A/CANX/HLA-B/VPS35/CLTC/RAB11B/EHD1/VAMP3/HSPA8/HLA-A/ARHGAP1/RAC1/RAB5C/LAMTOR3/SEC22B/ANXA3/CHMP2A/SPPL2A</t>
+    <t xml:space="preserve">CLTC/RAB7A/HLA-A/TMX3/CLIC4/SPPL2A/CANX/RAB5C/ANXA6/EHD1/SEC22B/HSPA8/COPB2/VAMP3/ATP6V1G1/CHMP2A/RAC1/VPS35/LAMTOR3/RHOA/ANXA3/HLA-B/ARHGAP1/RAB11B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005765</t>
@@ -1381,7 +1381,7 @@
     <t xml:space="preserve">62/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">ANXA6/ATP6V1G1/FLOT1/RAB7A/VPS35/CLTC/IFITM1/AHNAK/HSPA8/RAB5C/LAMTOR3/SEC22B/CHMP2A/SPPL2A</t>
+    <t xml:space="preserve">AHNAK/CLTC/RAB7A/FLOT1/SPPL2A/RAB5C/ANXA6/SEC22B/HSPA8/IFITM1/ATP6V1G1/CHMP2A/VPS35/LAMTOR3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0098852</t>
@@ -1402,7 +1402,7 @@
     <t xml:space="preserve">11/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">CANX/HLA-B/HSPA8/HLA-A/SPPL2A</t>
+    <t xml:space="preserve">HLA-A/SPPL2A/CANX/HSPA8/HLA-B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005694</t>
@@ -1417,7 +1417,7 @@
     <t xml:space="preserve">104/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">DCTN4/ARPC4/PURA/ACTR3/STAT3/SET/H1-5/ILK/HNRNPD/RPA2/HNRNPK/HNRNPDL/HNRNPL/NAP1L1/ACTR2/NONO/SKP1/RAN/CHMP2A/HNRNPC</t>
+    <t xml:space="preserve">ACTR3/HNRNPC/HNRNPDL/PURA/DCTN4/RPA2/NONO/SET/HNRNPK/NAP1L1/HNRNPL/CHMP2A/ARPC4/ACTR2/STAT3/SKP1/H1-5/RAN/HNRNPD/ILK</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030139</t>
@@ -1432,7 +1432,7 @@
     <t xml:space="preserve">56/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">RAB7A/HLA-B/CLTC/RAB11B/ZYX/EHD1/VAMP3/MPO/HSP90AA1/HLA-A/RAB5C/SEC22B/ANXA3</t>
+    <t xml:space="preserve">CLTC/RAB7A/HLA-A/RAB5C/EHD1/SEC22B/ZYX/VAMP3/HSP90AA1/MPO/ANXA3/HLA-B/RAB11B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0012506</t>
@@ -1456,7 +1456,7 @@
     <t xml:space="preserve">199/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">TMX3/ATP6V1G1/VAT1/RHOA/RAB7A/HLA-B/CAP1/PAK2/RAB11B/FERMT3/PPIA/FTL/VAMP3/HSPA8/HSP90AB1/MPO/CCT8/HSP90AA1/DYNC1H1/CTSG/MYH9/TUBB/RAC1/GNAI2/RAB5C/PRDX6/ERP44/S100A11/LAMTOR3/PSMC6/ACTR2/ANXA3</t>
+    <t xml:space="preserve">PSMC6/PPIA/RAB7A/ERP44/TMX3/RAB5C/CCT8/DYNC1H1/PRDX6/VAT1/TUBB/HSPA8/VAMP3/S100A11/GNAI2/ATP6V1G1/RAC1/PAK2/ACTR2/LAMTOR3/HSP90AA1/HSP90AB1/MPO/MYH9/RHOA/FTL/ANXA3/HLA-B/CTSG/RAB11B/FERMT3/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0031983</t>
@@ -1468,7 +1468,7 @@
     <t xml:space="preserve">85/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">VAT1/CAP1/FERMT3/PPIA/FTL/HSPA8/HSP90AB1/MPO/CCT8/HSP90AA1/DYNC1H1/CTSG/TUBB/PRDX6/ERP44/S100A11/ACTR2</t>
+    <t xml:space="preserve">PPIA/ERP44/CCT8/DYNC1H1/PRDX6/VAT1/TUBB/HSPA8/S100A11/ACTR2/HSP90AA1/HSP90AB1/MPO/FTL/CTSG/FERMT3/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0034774</t>
@@ -1489,7 +1489,7 @@
     <t xml:space="preserve">ruffle</t>
   </si>
   <si>
-    <t xml:space="preserve">RHOA/SH3BGRL3/FSCN1/ARHGAP1/MYH9/RAC1/TLN1/S100A6/S100A11</t>
+    <t xml:space="preserve">FSCN1/S100A11/S100A6/TLN1/RAC1/SH3BGRL3/MYH9/RHOA/ARHGAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030864</t>
@@ -1501,7 +1501,7 @@
     <t xml:space="preserve">22/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">FLOT1/LASP1/CAP1/SPTBN1/EPB41L2/MYH9/ACTR2</t>
+    <t xml:space="preserve">LASP1/FLOT1/SPTBN1/ACTR2/MYH9/EPB41L2/CAP1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0055037</t>
@@ -1510,7 +1510,7 @@
     <t xml:space="preserve">recycling endosome</t>
   </si>
   <si>
-    <t xml:space="preserve">HLA-B/RAB11B/EHD1/VAMP3/HLA-A/RAC1/RAN</t>
+    <t xml:space="preserve">HLA-A/EHD1/VAMP3/RAC1/RAN/HLA-B/RAB11B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0055038</t>
@@ -1525,7 +1525,7 @@
     <t xml:space="preserve">17/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">HLA-B/RAB11B/EHD1/VAMP3/HLA-A/RAC1</t>
+    <t xml:space="preserve">HLA-A/EHD1/VAMP3/RAC1/HLA-B/RAB11B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0098862</t>
@@ -1540,7 +1540,7 @@
     <t xml:space="preserve">28/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTR3/MPP1/CLIC1/AQP1/HSP90AA1/MYH9/RAC1/MYL12B</t>
+    <t xml:space="preserve">ACTR3/AQP1/MPP1/RAC1/CLIC1/HSP90AA1/MYL12B/MYH9</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0072686</t>
@@ -1552,7 +1552,7 @@
     <t xml:space="preserve">23/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">TUBB6/MAP4/CLTC/DPYSL2/TUBB/NUDC/MAPRE1</t>
+    <t xml:space="preserve">CLTC/MAP4/TUBB/MAPRE1/TUBB6/DPYSL2/NUDC</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005774</t>
@@ -1573,7 +1573,7 @@
     <t xml:space="preserve">18/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">HLA-B/EHD1/VAMP3/HLA-A/RAC1/RAB5C</t>
+    <t xml:space="preserve">HLA-A/RAB5C/EHD1/VAMP3/RAC1/HLA-B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005912</t>
@@ -1585,7 +1585,7 @@
     <t xml:space="preserve">30/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">FLOT1/MSN/ZYX/MYH9/TLN1/PDLIM1/S100A11/ADD1</t>
+    <t xml:space="preserve">FLOT1/MSN/ZYX/S100A11/TLN1/PDLIM1/MYH9/ADD1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030666</t>
@@ -1594,7 +1594,7 @@
     <t xml:space="preserve">endocytic vesicle membrane</t>
   </si>
   <si>
-    <t xml:space="preserve">RAB7A/HLA-B/CLTC/RAB11B/VAMP3/HLA-A/SEC22B/ANXA3</t>
+    <t xml:space="preserve">CLTC/RAB7A/HLA-A/SEC22B/VAMP3/ANXA3/HLA-B/RAB11B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005815</t>
@@ -1606,7 +1606,7 @@
     <t xml:space="preserve">77/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">DCTN4/CLIC4/FLOT1/MAP4/ILK/CCT8/DYNC1H1/RAC1/GNAI2/TLN1/PDCD6IP/SKP1/MAPRE1/RAN/CALM1</t>
+    <t xml:space="preserve">FLOT1/CALM1/CLIC4/DCTN4/CCT8/MAP4/DYNC1H1/GNAI2/TLN1/RAC1/SKP1/PDCD6IP/MAPRE1/RAN/ILK</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005813</t>
@@ -1618,7 +1618,7 @@
     <t xml:space="preserve">63/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">DCTN4/CLIC4/FLOT1/ILK/CCT8/DYNC1H1/RAC1/GNAI2/TLN1/PDCD6IP/SKP1/MAPRE1/CALM1</t>
+    <t xml:space="preserve">FLOT1/CALM1/CLIC4/DCTN4/CCT8/DYNC1H1/GNAI2/TLN1/RAC1/SKP1/PDCD6IP/MAPRE1/ILK</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005768</t>
@@ -1630,7 +1630,7 @@
     <t xml:space="preserve">107/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">ANXA6/FLOT1/RHOA/RAB7A/HLA-B/VPS35/CLTC/RAB11B/EHD1/VAMP3/HLA-A/ARHGAP1/RAC1/RAB5C/LAMTOR3/PDCD6IP/RAN/CHMP2A/SPPL2A</t>
+    <t xml:space="preserve">CLTC/RAB7A/HLA-A/FLOT1/SPPL2A/RAB5C/ANXA6/EHD1/VAMP3/CHMP2A/RAC1/VPS35/LAMTOR3/PDCD6IP/RHOA/RAN/HLA-B/ARHGAP1/RAB11B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030027</t>
@@ -1642,7 +1642,7 @@
     <t xml:space="preserve">31/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">FLOT1/ACTR3/RHOA/FSCN1/ILK/RAC1/P4HB/SYNE2</t>
+    <t xml:space="preserve">ACTR3/FLOT1/FSCN1/P4HB/RAC1/SYNE2/RHOA/ILK</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0050839</t>
@@ -1657,7 +1657,7 @@
     <t xml:space="preserve">141/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">MSN/LASP1/HSPA5/CLIC1/PAK2/RAB11B/FERMT3/EHD1/PPIA/PFN1/AHNAK/FSCN1/SPTBN1/HSPA8/HSP90AB1/ILK/CCT8/ARHGAP1/TAGLN2/MYH9/PARVA/TLN1/PRDX6/P4HB/HNRNPK/PDLIM1/NUDC/S100A11/MAPRE1/RAN/ADD1</t>
+    <t xml:space="preserve">AHNAK/PPIA/LASP1/HSPA5/MSN/CCT8/EHD1/PRDX6/FSCN1/PFN1/HNRNPK/P4HB/HSPA8/SPTBN1/S100A11/TLN1/PAK2/PDLIM1/CLIC1/HSP90AB1/MYH9/TAGLN2/ADD1/MAPRE1/RAN/ARHGAP1/PARVA/ILK/RAB11B/FERMT3/NUDC</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0045296</t>
@@ -1672,7 +1672,7 @@
     <t xml:space="preserve">116/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">LASP1/HSPA5/CLIC1/PAK2/RAB11B/EHD1/PFN1/AHNAK/FSCN1/SPTBN1/HSPA8/HSP90AB1/CCT8/ARHGAP1/TAGLN2/MYH9/PARVA/TLN1/PRDX6/HNRNPK/PDLIM1/NUDC/S100A11/MAPRE1/RAN/ADD1</t>
+    <t xml:space="preserve">AHNAK/LASP1/HSPA5/CCT8/EHD1/PRDX6/FSCN1/PFN1/HNRNPK/HSPA8/SPTBN1/S100A11/TLN1/PAK2/PDLIM1/CLIC1/HSP90AB1/MYH9/TAGLN2/ADD1/MAPRE1/RAN/ARHGAP1/PARVA/RAB11B/NUDC</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005102</t>
@@ -1687,7 +1687,7 @@
     <t xml:space="preserve">109/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">FLOT1/MSN/HLA-B/MPP1/STAT3/VPS35/AQP1/CLTC/FERMT3/PPIA/HSPA8/ILK/HSP90AA1/HLA-A/MYH9/TUBB/STRAP/GNAI2/TLN1/S100A13/P4HB/PDCD6IP/DDT</t>
+    <t xml:space="preserve">CLTC/PPIA/HLA-A/FLOT1/MSN/DDT/AQP1/MPP1/P4HB/TUBB/HSPA8/GNAI2/TLN1/S100A13/VPS35/STAT3/PDCD6IP/HSP90AA1/MYH9/HLA-B/STRAP/ILK/FERMT3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0048306</t>
@@ -1699,7 +1699,7 @@
     <t xml:space="preserve">21/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">ANXA6/S100A16/S100A13/S100A6/S100A11/PDCD6IP/ANXA3/CALM1</t>
+    <t xml:space="preserve">CALM1/ANXA6/S100A11/S100A6/S100A13/PDCD6IP/S100A16/ANXA3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0019904</t>
@@ -1714,7 +1714,7 @@
     <t xml:space="preserve">86/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">QKI/ARF1/HSPA5/CLTC/SH3BGRL/HSPA8/HSP90AB1/EPB41L2/HSP90AA1/ARHGAP1/MYH9/TUBB/TLN1/HNRNPK/YWHAQ/WARS1/SKP1/RAN/CHMP2A</t>
+    <t xml:space="preserve">CLTC/HSPA5/WARS1/ARF1/HNRNPK/TUBB/HSPA8/TLN1/YWHAQ/CHMP2A/SH3BGRL/SKP1/QKI/HSP90AA1/HSP90AB1/MYH9/RAN/ARHGAP1/EPB41L2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030198</t>
@@ -1729,7 +1729,7 @@
     <t xml:space="preserve">18/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">MYH11/LUM/FBLN5/ITGB1/FBLN1/MFAP4</t>
+    <t xml:space="preserve">FBLN5/MYH11/LUM/MFAP4/ITGB1/FBLN1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0043062</t>
@@ -1756,7 +1756,7 @@
     <t xml:space="preserve">128/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">THY1/AOC3/RRAS/HSPH1/S100A10/FBLN5/ITGB1/BCAM/LPP/CD9/CSRP1/FBLN1/FBLN2/MFAP4</t>
+    <t xml:space="preserve">FBLN5/LPP/HSPH1/CD9/THY1/S100A10/CSRP1/MFAP4/BCAM/RRAS/AOC3/ITGB1/FBLN1/FBLN2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005614</t>
@@ -1768,7 +1768,7 @@
     <t xml:space="preserve">8/61</t>
   </si>
   <si>
-    <t xml:space="preserve">PRELP/LUM/ASPN/FBLN5/FBLN1/FBLN2/MFAP4/DCN</t>
+    <t xml:space="preserve">FBLN5/ASPN/LUM/MFAP4/DCN/PRELP/FBLN1/FBLN2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030312</t>
@@ -1783,7 +1783,7 @@
     <t xml:space="preserve">35/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">PRELP/LUM/ASPN/S100A10/FBLN5/BCAM/FBLN1/FBLN2/MFAP4/DCN</t>
+    <t xml:space="preserve">FBLN5/ASPN/LUM/S100A10/MFAP4/BCAM/DCN/PRELP/FBLN1/FBLN2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0031012</t>
@@ -1801,7 +1801,7 @@
     <t xml:space="preserve">6/61</t>
   </si>
   <si>
-    <t xml:space="preserve">LUM/FBLN5/FBLN1/FBLN2/MFAP4/DCN</t>
+    <t xml:space="preserve">FBLN5/LUM/MFAP4/DCN/FBLN1/FBLN2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005201</t>
@@ -1828,7 +1828,7 @@
     <t xml:space="preserve">36/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">AOC3/PPP2CA/PDCD6/SNX2/ITGB1/CAV2/UBA2</t>
+    <t xml:space="preserve">PDCD6/CAV2/SNX2/PPP2CA/AOC3/ITGB1/UBA2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005509</t>
@@ -1843,7 +1843,7 @@
     <t xml:space="preserve">85/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">AOC3/PDCD6/ASPN/HPCAL1/S100A10/FBLN5/ITGB1/FBLN1/FBLN2/S100A1</t>
+    <t xml:space="preserve">FBLN5/ASPN/HPCAL1/S100A1/PDCD6/S100A10/AOC3/ITGB1/FBLN1/FBLN2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005178</t>
@@ -1858,7 +1858,7 @@
     <t xml:space="preserve">22/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">THY1/FBLN5/ITGB1/CD9/FBLN1</t>
+    <t xml:space="preserve">FBLN5/CD9/THY1/ITGB1/FBLN1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0002181</t>
@@ -1873,7 +1873,7 @@
     <t xml:space="preserve">106/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RPS28/RPL10/RPL18A/RPS25/RPL17/RPL22/RPL7/RPL11/RPL13A/NPM1/RPS21/RPS3/RPS3A/EIF3F/RPS24/RPS16/EIF4A1/RPL14/RPL4/EIF3C/EIF2S3/RPLP2/RPL27/RPL13/RPS19/RPS15A/RPLP0/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/EIF3F/RPL7A/RPL12/RPL10/RPS19/RPL10A/RPS28/RPL22/RPL27/EIF3C/RPL4/RPL11/RPL7/EIF4A1/RPS16/RPL18A/RPS25/RPS3A/RPS21/EIF2S3/RPLP2/RPL13A/NPM1/RPLP0/RPS15A/RPS24/RPL30/RPL13/RPL17/RPS3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006412</t>
@@ -1885,7 +1885,7 @@
     <t xml:space="preserve">39/74</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RPS28/PA2G4/RPL10/RPL18A/RPS25/RPL17/RPL22/RPL7/RPL11/RPL13A/ABCF1/NPM1/RPS21/RPS3/NCL/RPS3A/EIF3F/RPS24/RPS16/EIF4A1/RPL14/MSI2/FARSB/RPL4/EIF3C/EIF2S3/RPLP2/RPL27/RPL13/RPS19/RPS15A/NARS1/RPLP0/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/MSI2/EIF3F/RPL7A/RPL12/RPL10/RPS19/RPL10A/RPS28/RPL22/RPL27/EIF3C/RPL4/RPL11/RPL7/EIF4A1/RPS16/RPL18A/RPS25/RPS3A/RPS21/EIF2S3/FARSB/RPLP2/RPL13A/ABCF1/NPM1/NARS1/RPLP0/RPS15A/PA2G4/RPS24/RPL30/RPL13/RPL17/RPS3/NCL</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0160307</t>
@@ -1906,7 +1906,7 @@
     <t xml:space="preserve">32/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RPL10/RPL18A/RPL17/RPL7/RPL11/RPL13A/RPL14/RPL4/RPLP2/RPL27/RPL13/RPLP0/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/RPL7A/RPL12/RPL10/RPL10A/RPL27/RPL4/RPL11/RPL7/RPL18A/RPLP2/RPL13A/RPLP0/RPL30/RPL13/RPL17</t>
   </si>
   <si>
     <t xml:space="preserve">GO:1901740</t>
@@ -1975,7 +1975,7 @@
     <t xml:space="preserve">81/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RPS28/PA2G4/RPS25/RPL7/LSM4/RPL11/RPL13A/NPM1/RPS21/RPS3A/EIF3F/RPS24/RPS16/RPL14/EIF3C/EIF2S3/RPL27/RPS19/RPS15A/RPLP0/RPL7A</t>
+    <t xml:space="preserve">RPL14/EIF3F/RPL7A/RPS19/RPS28/RPL27/EIF3C/RPL11/RPL7/RPS16/LSM4/RPS25/RPS3A/RPS21/EIF2S3/RPL13A/NPM1/RPLP0/RPS15A/PA2G4/RPS24</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0016072</t>
@@ -1990,7 +1990,7 @@
     <t xml:space="preserve">30/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RPS28/PA2G4/RPS25/RPL7/RPL11/RPS21/NCL/RPS24/RPS16/RPL14/RPL27/RPS19/RPL7A</t>
+    <t xml:space="preserve">RPL14/RPL7A/RPS19/RPS28/RPL27/RPL11/RPL7/RPS16/RPS25/RPS21/PA2G4/RPS24/NCL</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0042254</t>
@@ -2002,7 +2002,7 @@
     <t xml:space="preserve">16/74</t>
   </si>
   <si>
-    <t xml:space="preserve">RPS28/PA2G4/RPS25/RPL7/RPL11/NPM1/RPS21/RPS3A/RPS24/RPS16/RPL14/RPL27/RPS19/RPS15A/RPLP0/RPL7A</t>
+    <t xml:space="preserve">RPL14/RPL7A/RPS19/RPS28/RPL27/RPL11/RPL7/RPS16/RPS25/RPS3A/RPS21/NPM1/RPLP0/RPS15A/PA2G4/RPS24</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006364</t>
@@ -2014,7 +2014,7 @@
     <t xml:space="preserve">12/74</t>
   </si>
   <si>
-    <t xml:space="preserve">RPS28/PA2G4/RPS25/RPL7/RPL11/RPS21/RPS24/RPS16/RPL14/RPL27/RPS19/RPL7A</t>
+    <t xml:space="preserve">RPL14/RPL7A/RPS19/RPS28/RPL27/RPL11/RPL7/RPS16/RPS25/RPS21/PA2G4/RPS24</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0051146</t>
@@ -2029,7 +2029,7 @@
     <t xml:space="preserve">89/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RPL10/RPL18A/MYBPH/RPL17/RPL7/RPL11/RPL13A/MYPN/RPL14/RPL4/RPLP2/RPL27/RPL13/RPLP0/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/RPL7A/RPL12/RPL10/RPL10A/RPL27/RPL4/RPL11/RPL7/RPL18A/MYPN/RPLP2/RPL13A/RPLP0/RPL30/RPL13/RPL17/MYBPH</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006941</t>
@@ -2041,7 +2041,7 @@
     <t xml:space="preserve">93/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RPL10/RPL18A/MYBPH/RPL17/RPL7/ASPH/RPL11/RPL13A/RPL14/RPL4/RPLP2/RPL27/RPL13/RPLP0/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/RPL7A/RPL12/RPL10/RPL10A/RPL27/RPL4/RPL11/ASPH/RPL7/RPL18A/RPLP2/RPL13A/RPLP0/RPL30/RPL13/RPL17/MYBPH</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0051129</t>
@@ -2056,7 +2056,7 @@
     <t xml:space="preserve">126/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RPL10/RPL18A/RPL17/RPL7/DNAJB1/RPL11/RPL13A/NPM1/CORO1A/PACSIN3/RPL14/RPL4/RPLP2/RPL27/RPL13/RPLP0/RPL12/RPL7A/SLC25A5/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/RPL7A/RPL12/RPL10/RPL10A/RPL27/RPL4/PACSIN3/RPL11/DNAJB1/RPL7/RPL18A/RPLP2/RPL13A/NPM1/RPLP0/RPL30/SLC25A5/RPL13/CORO1A/RPL17</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0042692</t>
@@ -2077,7 +2077,7 @@
     <t xml:space="preserve">72/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RPL18A/RPL17/RPL7/RPL11/RPL13A/RPL14/RPL4/RPLP2/RPL27/RPL13/RPLP0/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/RPL7A/RPL12/RPL10A/RPL27/RPL4/RPL11/RPL7/RPL18A/RPLP2/RPL13A/RPLP0/RPL30/RPL13/RPL17</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0048232</t>
@@ -2104,7 +2104,7 @@
     <t xml:space="preserve">19/74</t>
   </si>
   <si>
-    <t xml:space="preserve">RTRAF/RPS28/PA2G4/HNRNPR/RPS25/RPL7/LSM4/RPL11/RPS21/FUS/NCL/HNRNPH1/RPS24/RPS16/RPL14/SRSF2/RPL27/RPS19/RPL7A</t>
+    <t xml:space="preserve">RPL14/RPL7A/RPS19/HNRNPR/RPS28/RTRAF/FUS/SRSF2/RPL27/RPL11/RPL7/RPS16/LSM4/RPS25/HNRNPH1/RPS21/PA2G4/RPS24/NCL</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0048609</t>
@@ -2146,7 +2146,7 @@
     <t xml:space="preserve">143/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RPL10/RPL18A/MYBPH/RPL17/LDB3/RPL7/RPL11/RPL13A/XIRP1/MYPN/RPL14/RPL4/RPLP2/RPL27/RPL13/RPLP0/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/RPL7A/RPL12/RPL10/RPL10A/LDB3/RPL27/RPL4/RPL11/RPL7/RPL18A/MYPN/XIRP1/RPLP2/RPL13A/RPLP0/RPL30/RPL13/RPL17/MYBPH</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0051093</t>
@@ -2167,7 +2167,7 @@
     <t xml:space="preserve">135/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RPL10/RPL18A/MYBPH/RPL17/RPL7/RPL11/RPL13A/NCL/MYPN/RPL14/RPL4/RPLP2/RPL27/RPL13/RPLP0/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/RPL7A/RPL12/RPL10/RPL10A/RPL27/RPL4/RPL11/RPL7/RPL18A/MYPN/RPLP2/RPL13A/RPLP0/RPL30/RPL13/RPL17/MYBPH/NCL</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006936</t>
@@ -2188,7 +2188,7 @@
     <t xml:space="preserve">25/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RPS28/RPS25/NPM1/RPS21/RPS3A/RPS24/RPS16/RPS19/RPS15A</t>
+    <t xml:space="preserve">RPS19/RPS28/RPS16/RPS25/RPS3A/RPS21/NPM1/RPS15A/RPS24</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0022414</t>
@@ -2212,7 +2212,7 @@
     <t xml:space="preserve">256/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">DNAJB4/RTRAF/RPS28/PA2G4/RPL10/HNRNPR/RPS25/RPL7/LSM4/ASPH/DNAJB1/RPL11/NPM1/RPS21/FUS/RPS3/NCL/HNRNPH1/RPS24/RPS16/EIF4A1/RPL14/SRSF2/RPL27/VAPB/SUB1/RPS19/RPL7A</t>
+    <t xml:space="preserve">RPL14/RPL7A/VAPB/RPL10/SUB1/RPS19/HNRNPR/RPS28/RTRAF/FUS/SRSF2/RPL27/RPL11/ASPH/DNAJB1/RPL7/EIF4A1/RPS16/LSM4/RPS25/DNAJB4/HNRNPH1/RPS21/NPM1/PA2G4/RPS24/RPS3/NCL</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0016070</t>
@@ -2227,7 +2227,7 @@
     <t xml:space="preserve">289/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">DNAJB4/RTRAF/RPS28/PA2G4/RPL10/HNRNPR/RPS25/RPL7/LSM4/ASPH/DNAJB1/RPL11/NPM1/RPS21/FUS/RPS3/NCL/HNRNPH1/RPS24/RPS16/EIF4A1/RPL14/FARSB/SRSF2/RPL27/VAPB/SUB1/RPS19/NARS1/RPL7A</t>
+    <t xml:space="preserve">RPL14/RPL7A/VAPB/RPL10/SUB1/RPS19/HNRNPR/RPS28/RTRAF/FUS/SRSF2/RPL27/RPL11/ASPH/DNAJB1/RPL7/EIF4A1/RPS16/LSM4/RPS25/DNAJB4/HNRNPH1/RPS21/FARSB/NPM1/NARS1/PA2G4/RPS24/RPS3/NCL</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0003012</t>
@@ -2251,7 +2251,7 @@
     <t xml:space="preserve">29/74</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RPL10/RPL18A/RPL17/RPL7/ASPH/DNAJB1/RPL11/RPL13A/NPM1/CORO1A/MYO18A/PACSIN3/RPS3/KIF5B/RPL14/RPL4/RPLP2/RPL27/AP2M1/RPL13/RPLP0/ARPC2/RPL12/RPL7A/SLC25A5/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/MYO18A/AP2M1/RPL7A/RPL12/RPL10/RPL10A/RPL27/RPL4/PACSIN3/RPL11/ASPH/DNAJB1/ARPC2/RPL7/RPL18A/RPLP2/RPL13A/NPM1/RPLP0/KIF5B/RPL30/SLC25A5/RPL13/CORO1A/RPL17/RPS3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0090304</t>
@@ -2266,7 +2266,7 @@
     <t xml:space="preserve">345/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">DNAJB4/RTRAF/RPS28/PA2G4/RPL10/HNRNPR/RPS25/RPL7/LSM4/ASPH/DNAJB1/RPL11/NPM1/RPS21/FUS/MYO18A/RPS3/NCL/HNRNPH1/RPS24/RPS16/EIF4A1/RPL14/FARSB/SRSF2/RPL27/VAPB/SUB1/RPS19/NARS1/RPL7A</t>
+    <t xml:space="preserve">RPL14/MYO18A/RPL7A/VAPB/RPL10/SUB1/RPS19/HNRNPR/RPS28/RTRAF/FUS/SRSF2/RPL27/RPL11/ASPH/DNAJB1/RPL7/EIF4A1/RPS16/LSM4/RPS25/DNAJB4/HNRNPH1/RPS21/FARSB/NPM1/NARS1/PA2G4/RPS24/RPS3/NCL</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0071826</t>
@@ -2278,7 +2278,7 @@
     <t xml:space="preserve">45/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RPS28/LSM4/RPL11/RPL13A/EIF3F/KIF5B/EIF3C/EIF2S3/RPS19</t>
+    <t xml:space="preserve">EIF3F/RPS19/RPS28/EIF3C/RPL11/LSM4/EIF2S3/RPL13A/KIF5B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0009653</t>
@@ -2290,7 +2290,7 @@
     <t xml:space="preserve">223/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RPL10/RPL18A/MYBPH/RPL17/RPL7/RPL11/RPL13A/NCL/MYPN/KIF5B/RPL14/RPL4/RPLP2/RPL27/RPL13/RPLP0/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/RPL7A/RPL12/RPL10/RPL10A/RPL27/RPL4/RPL11/RPL7/RPL18A/MYPN/RPLP2/RPL13A/RPLP0/KIF5B/RPL30/RPL13/RPL17/MYBPH/NCL</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0002183</t>
@@ -2305,7 +2305,7 @@
     <t xml:space="preserve">23/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL13A/RPS3/EIF3F/EIF4A1/EIF3C/EIF2S3</t>
+    <t xml:space="preserve">EIF3F/EIF3C/EIF4A1/EIF2S3/RPL13A/RPS3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0022618</t>
@@ -2320,7 +2320,7 @@
     <t xml:space="preserve">43/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RPS28/LSM4/RPL11/RPL13A/EIF3F/EIF3C/EIF2S3/RPS19</t>
+    <t xml:space="preserve">EIF3F/RPS19/RPS28/EIF3C/RPL11/LSM4/EIF2S3/RPL13A</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0050793</t>
@@ -2332,7 +2332,7 @@
     <t xml:space="preserve">206/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/PA2G4/RPL10/RPL18A/RPL17/RPL7/RPL11/RPL13A/RPL14/RPL4/RPLP2/RPL27/RPL13/RPS19/RPLP0/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/RPL7A/RPL12/RPL10/RPS19/RPL10A/RPL27/RPL4/RPL11/RPL7/RPL18A/RPLP2/RPL13A/RPLP0/PA2G4/RPL30/RPL13/RPL17</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006413</t>
@@ -2341,7 +2341,7 @@
     <t xml:space="preserve">translational initiation</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL13A/ABCF1/RPS3/RPS3A/EIF3F/EIF4A1/EIF3C/EIF2S3</t>
+    <t xml:space="preserve">EIF3F/EIF3C/EIF4A1/RPS3A/EIF2S3/RPL13A/ABCF1/RPS3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030154</t>
@@ -2353,7 +2353,7 @@
     <t xml:space="preserve">363/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/PA2G4/RPL10/RPL18A/MYBPH/RPL17/RPL7/RPL11/RPL13A/NPM1/XIRP1/RPS3A/MYPN/KIF5B/RPL14/MSI2/RPL4/RPLP2/RPL27/RPL13/RPS19/RPLP0/RTN3/RPL12/RPL7A/SLC25A5/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/MSI2/RPL7A/RTN3/RPL12/RPL10/RPS19/RPL10A/RPL27/RPL4/RPL11/RPL7/RPL18A/RPS3A/MYPN/XIRP1/RPLP2/RPL13A/NPM1/RPLP0/PA2G4/KIF5B/RPL30/SLC25A5/RPL13/RPL17/MYBPH</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0048869</t>
@@ -2371,7 +2371,7 @@
     <t xml:space="preserve">post-transcriptional regulation of gene expression</t>
   </si>
   <si>
-    <t xml:space="preserve">PA2G4/RPL10/LSM4/RPL13A/ABCF1/NPM1/FUS/RPS3/NCL/MSI2/EIF3C/EIF2S3</t>
+    <t xml:space="preserve">MSI2/RPL10/FUS/EIF3C/LSM4/EIF2S3/RPL13A/ABCF1/NPM1/PA2G4/RPS3/NCL</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0003008</t>
@@ -2392,7 +2392,7 @@
     <t xml:space="preserve">382/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">DNAJB4/RTRAF/RPS28/PA2G4/RPL10/HNRNPR/RPS25/RPL7/LSM4/ASPH/DNAJB1/RPL11/NPM1/RPS21/NANS/FUS/RPS3/NCL/HNRNPH1/RPS24/RPS16/EIF4A1/RPL14/SRSF2/RPL27/VAPB/SUB1/RPS19/RPL7A</t>
+    <t xml:space="preserve">RPL14/RPL7A/VAPB/RPL10/SUB1/RPS19/HNRNPR/RPS28/RTRAF/FUS/SRSF2/RPL27/RPL11/ASPH/DNAJB1/RPL7/EIF4A1/RPS16/LSM4/RPS25/DNAJB4/HNRNPH1/RPS21/NPM1/PA2G4/RPS24/NANS/RPS3/NCL</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006417</t>
@@ -2407,7 +2407,7 @@
     <t xml:space="preserve">78/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">PA2G4/RPL10/RPL13A/ABCF1/NPM1/RPS3/NCL/MSI2/EIF3C/EIF2S3</t>
+    <t xml:space="preserve">MSI2/RPL10/EIF3C/EIF2S3/RPL13A/ABCF1/NPM1/PA2G4/RPS3/NCL</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0022626</t>
@@ -2419,7 +2419,7 @@
     <t xml:space="preserve">28/75</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RPS28/RPL10/RPL18A/RPS25/RPL17/RPL22/RPL7/RPL11/RPL13A/RPS21/RPS3/RPS3A/RPS24/RPS16/RPL14/RPL4/RPLP2/RPL27/RPL13/RPS19/RPS15A/RPLP0/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/RPL7A/RPL12/RPL10/RPS19/RPL10A/RPS28/RPL22/RPL27/RPL4/RPL11/RPL7/RPS16/RPL18A/RPS25/RPS3A/RPS21/RPLP2/RPL13A/RPLP0/RPS15A/RPS24/RPL30/RPL13/RPL17/RPS3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0044391</t>
@@ -2434,7 +2434,7 @@
     <t xml:space="preserve">79/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RPS28/RPL10/RPL18A/RPS25/RPL17/RPL22/RPL7/RPL11/RPL13A/NPM1/RPS21/RPS3/RPS3A/RPS24/RPS16/RPL14/RPL4/RPLP2/RPL27/RPL13/RPS19/RPS15A/RPLP0/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/RPL7A/RPL12/RPL10/RPS19/RPL10A/RPS28/RPL22/RPL27/RPL4/RPL11/RPL7/RPS16/RPL18A/RPS25/RPS3A/RPS21/RPLP2/RPL13A/NPM1/RPLP0/RPS15A/RPS24/RPL30/RPL13/RPL17/RPS3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:1990904</t>
@@ -2449,7 +2449,7 @@
     <t xml:space="preserve">150/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RPS28/PA2G4/RPL10/RPL18A/HNRNPR/RPS25/RPL17/RPL22/RPL7/LSM4/RPL11/RPL13A/NPM1/RPS21/RPS3/NCL/RPS3A/HNRNPH1/EIF3F/RPS24/RPS16/RPL14/RPL4/EIF3C/RPLP2/RPL27/RPL13/RPS19/RPS15A/RPLP0/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/EIF3F/RPL7A/RPL12/RPL10/RPS19/RPL10A/HNRNPR/RPS28/RPL22/RPL27/EIF3C/RPL4/RPL11/RPL7/RPS16/RPL18A/LSM4/RPS25/HNRNPH1/RPS3A/RPS21/RPLP2/RPL13A/NPM1/RPLP0/RPS15A/PA2G4/RPS24/RPL30/RPL13/RPL17/RPS3/NCL</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005840</t>
@@ -2470,7 +2470,7 @@
     <t xml:space="preserve">19/75</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RPL10/RPL18A/RPL17/RPL22/RPL7/RPL11/RPL13A/RPL14/RPL4/RPLP2/RPL27/RPL13/RPLP0/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/RPL7A/RPL12/RPL10/RPL10A/RPL22/RPL27/RPL4/RPL11/RPL7/RPL18A/RPLP2/RPL13A/RPLP0/RPL30/RPL13/RPL17</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0015934</t>
@@ -2485,7 +2485,7 @@
     <t xml:space="preserve">47/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RPL10/RPL18A/RPL17/RPL22/RPL7/RPL11/RPL13A/NPM1/RPL14/RPL4/RPLP2/RPL27/RPL13/RPLP0/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/RPL7A/RPL12/RPL10/RPL10A/RPL22/RPL27/RPL4/RPL11/RPL7/RPL18A/RPLP2/RPL13A/NPM1/RPLP0/RPL30/RPL13/RPL17</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005730</t>
@@ -2500,7 +2500,7 @@
     <t xml:space="preserve">92/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL10A/RPS28/PA2G4/RPS25/RPL7/DNAJB1/RPL11/RPL13A/NPM1/RPS3/NCL/RPS3A/RPS24/RPS16/RPL4/RPL27/RPL13/SUB1/RPS19/RPS15A/RPL7A</t>
+    <t xml:space="preserve">RPL7A/SUB1/RPS19/RPL10A/RPS28/RPL27/RPL4/RPL11/DNAJB1/RPL7/RPS16/RPS25/RPS3A/RPL13A/NPM1/RPS15A/PA2G4/RPS24/RPL13/RPS3/NCL</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0014069</t>
@@ -2515,7 +2515,7 @@
     <t xml:space="preserve">43/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL10A/RPL18A/RPS25/RPL7/DNAJB1/RPS3/RPL14/RPS19/RPLP0/RTN3/RPL12/RPL30</t>
+    <t xml:space="preserve">RPL14/RTN3/RPL12/RPS19/RPL10A/DNAJB1/RPL7/RPL18A/RPS25/RPLP0/RPL30/RPS3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0099572</t>
@@ -2539,7 +2539,7 @@
     <t xml:space="preserve">389/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">DNAJB4/RPL10A/RTRAF/RPS28/PA2G4/HNRNPR/RPS25/RPL7/LSM4/DNAJB1/RPL11/RPL13A/ABCF1/NPM1/RPS21/XIRP1/NANS/FUS/RPS3/NCL/RPS3A/MYPN/HNRNPH1/RPS24/PM20D2/RPS16/EIF4A1/FARSB/RPL4/SRSF2/RPL27/UBE2O/RPL13/SUB1/RPS19/RPS15A/ARPC2/RPL7A</t>
+    <t xml:space="preserve">RPL7A/SUB1/RPS19/RPL10A/HNRNPR/UBE2O/RPS28/RTRAF/FUS/PM20D2/SRSF2/RPL27/RPL4/RPL11/DNAJB1/ARPC2/RPL7/EIF4A1/RPS16/LSM4/RPS25/DNAJB4/HNRNPH1/RPS3A/MYPN/RPS21/XIRP1/FARSB/RPL13A/ABCF1/NPM1/RPS15A/PA2G4/RPS24/RPL13/NANS/RPS3/NCL</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0032279</t>
@@ -2569,7 +2569,7 @@
     <t xml:space="preserve">10/75</t>
   </si>
   <si>
-    <t xml:space="preserve">RPS28/RPS25/NPM1/RPS21/RPS3/RPS3A/RPS24/RPS16/RPS19/RPS15A</t>
+    <t xml:space="preserve">RPS19/RPS28/RPS16/RPS25/RPS3A/RPS21/NPM1/RPS15A/RPS24/RPS3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0098794</t>
@@ -2584,7 +2584,7 @@
     <t xml:space="preserve">102/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL10A/RPL18A/RPS25/RPL7/DNAJB1/FUS/RPS3/KIF5B/RPL14/AP2M1/VAPB/RPS19/RPLP0/ARPC2/RTN3/RPL12/RPL30</t>
+    <t xml:space="preserve">RPL14/AP2M1/RTN3/RPL12/VAPB/RPS19/RPL10A/FUS/DNAJB1/ARPC2/RPL7/RPL18A/RPS25/RPLP0/KIF5B/RPL30/RPS3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0022627</t>
@@ -2596,13 +2596,13 @@
     <t xml:space="preserve">9/75</t>
   </si>
   <si>
-    <t xml:space="preserve">RPS28/RPS25/RPS21/RPS3/RPS3A/RPS24/RPS16/RPS19/RPS15A</t>
+    <t xml:space="preserve">RPS19/RPS28/RPS16/RPS25/RPS3A/RPS21/RPS15A/RPS24/RPS3</t>
   </si>
   <si>
     <t xml:space="preserve">35/75</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RPS28/RPL18A/RPS25/RPL22/LDB3/RPL7/DNAJB1/RPL13A/NPM1/RPS21/XIRP1/CORO1A/FUS/RPS3/RPS3A/EIF3F/KIF5B/RPS16/RPL14/RPL4/RPLP2/RPL27/AP2M1/RPL13/VAPB/RPS19/RPLP0/ARPC2/RTN3/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/EIF3F/AP2M1/RPL7A/RTN3/RPL12/VAPB/RPS19/RPL10A/RPS28/FUS/LDB3/RPL22/RPL27/RPL4/DNAJB1/ARPC2/RPL7/RPS16/RPL18A/RPS25/RPS3A/RPS21/XIRP1/RPLP2/RPL13A/NPM1/RPLP0/KIF5B/RPL30/RPL13/CORO1A/RPS3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0045202</t>
@@ -2614,10 +2614,10 @@
     <t xml:space="preserve">282/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL10A/RPL15/RPS28/RPL18A/RPS25/RPL22/RPL7/DNAJB1/RPL13A/RPS21/CORO1A/FUS/RPS3/EIF3F/KIF5B/RPS16/RPL14/RPL27/AP2M1/RPL13/VAPB/RPS19/RPLP0/ARPC2/RTN3/RPL12/RPL7A/RPL30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL22/RPL7/RPL13A/NPM1/XIRP1/RPS3/RPS3A/RPS16/RPL4/RPLP2/RPL27/RPS19/RPLP0/ARPC2/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPL14/RPL15/EIF3F/AP2M1/RPL7A/RTN3/RPL12/VAPB/RPS19/RPL10A/RPS28/FUS/RPL22/RPL27/DNAJB1/ARPC2/RPL7/RPS16/RPL18A/RPS25/RPS21/RPL13A/RPLP0/KIF5B/RPL30/RPL13/CORO1A/RPS3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RPL18/RPL7A/RPL12/RPS19/RPL10A/RPL22/RPL27/RPL4/ARPC2/RPL7/RPS16/RPS3A/XIRP1/RPLP2/RPL13A/NPM1/RPLP0/RPL30/RPS3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005654</t>
@@ -2632,7 +2632,7 @@
     <t xml:space="preserve">352/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">DNAJB4/RTRAF/RPS28/HNRNPR/RPS25/LSM4/DNAJB1/RPL11/ABCF1/NPM1/RPS21/XIRP1/NANS/FUS/RPS3/NCL/RPS3A/MYPN/HNRNPH1/RPS24/PM20D2/RPS16/EIF4A1/FARSB/SRSF2/RPL27/UBE2O/SUB1/RPS19/RPS15A/ARPC2</t>
+    <t xml:space="preserve">SUB1/RPS19/HNRNPR/UBE2O/RPS28/RTRAF/FUS/PM20D2/SRSF2/RPL27/RPL11/DNAJB1/ARPC2/EIF4A1/RPS16/LSM4/RPS25/DNAJB4/HNRNPH1/RPS3A/MYPN/RPS21/XIRP1/FARSB/ABCF1/NPM1/RPS15A/RPS24/NANS/RPS3/NCL</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0032040</t>
@@ -2647,10 +2647,10 @@
     <t xml:space="preserve">19/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">RPS28/RPS3A/RPS24/RPS16/RPS19/RPS15A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL22/LDB3/RPL7/RPL13A/NPM1/XIRP1/CORO1A/RPS3/RPS3A/RPS16/RPL4/RPLP2/RPL27/RPS19/RPLP0/ARPC2/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPS19/RPS28/RPS16/RPS3A/RPS15A/RPS24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RPL18/RPL7A/RPL12/RPS19/RPL10A/LDB3/RPL22/RPL27/RPL4/ARPC2/RPL7/RPS16/RPS3A/XIRP1/RPLP2/RPL13A/NPM1/RPLP0/RPL30/CORO1A/RPS3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030684</t>
@@ -2674,7 +2674,7 @@
     <t xml:space="preserve">15/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPS28/RPS21/RPL4/RPL27</t>
+    <t xml:space="preserve">RPL18/RPS28/RPL27/RPL4/RPS21</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005783</t>
@@ -2689,7 +2689,7 @@
     <t xml:space="preserve">268/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/CNIH4/ESYT2/RPS28/RPL10/RPS25/RPL17/GABARAPL2/ASPH/RPS21/DDOST/RPS3/RPS3A/RPS24/RPS16/RPL14/RPL4/RPL27/RPL13/VAPB/RTN3</t>
+    <t xml:space="preserve">RPL18/CNIH4/RPL14/RTN3/GABARAPL2/VAPB/RPL10/RPL10A/RPS28/RPL27/RPL4/ASPH/RPS16/RPS25/RPS3A/RPS21/DDOST/ESYT2/RPS24/RPL13/RPL17/RPS3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0140513</t>
@@ -2701,7 +2701,7 @@
     <t xml:space="preserve">11/75</t>
   </si>
   <si>
-    <t xml:space="preserve">RPS28/HNRNPR/LSM4/RPS3/NCL/RPS3A/HNRNPH1/RPS24/RPS16/RPS19/RPS15A</t>
+    <t xml:space="preserve">RPS19/HNRNPR/RPS28/RPS16/LSM4/HNRNPH1/RPS3A/RPS15A/RPS24/RPS3/NCL</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0003735</t>
@@ -2728,7 +2728,7 @@
     <t xml:space="preserve">356/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RTRAF/RPS28/PA2G4/RPL10/RPL18A/HNRNPR/RPS25/RPL17/RPL22/RPL7/LSM4/RPL11/RPL13A/ABCF1/NPM1/RPS21/XIRP1/CORO1A/FUS/MYO18A/RPS3/NCL/ECHDC2/RPS3A/HNRNPH1/RPS24/RPS16/EIF4A1/RPL14/MSI2/FARSB/RPL4/EIF3C/EIF2S3/SRSF2/RPL27/UBE2O/RPL13/SUB1/RPS19/RPS15A/RPLP0/RPL12/RPL7A/SLC25A5/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/MYO18A/MSI2/RPL7A/RPL12/RPL10/SUB1/RPS19/RPL10A/HNRNPR/UBE2O/RPS28/RTRAF/FUS/RPL22/SRSF2/RPL27/EIF3C/RPL4/RPL11/RPL7/EIF4A1/RPS16/RPL18A/LSM4/RPS25/HNRNPH1/ECHDC2/RPS3A/RPS21/XIRP1/EIF2S3/FARSB/RPL13A/ABCF1/NPM1/RPLP0/RPS15A/PA2G4/RPS24/RPL30/SLC25A5/RPL13/CORO1A/RPL17/RPS3/NCL</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0003676</t>
@@ -2743,7 +2743,7 @@
     <t xml:space="preserve">394/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RTRAF/RPS28/PA2G4/RPL10/RPL18A/HNRNPR/RPS25/RPL17/RPL22/RPL7/LSM4/RPL11/RPL13A/ABCF1/NPM1/RPS21/XIRP1/CORO1A/FUS/MYO18A/RPS3/NCL/ECHDC2/RPS3A/HNRNPH1/RPS24/RPS16/EIF4A1/RPL14/MSI2/FARSB/RPL4/EIF3C/EIF2S3/SRSF2/RPL27/UBE2O/RPL13/SUB1/RPS19/RPS15A/NARS1/RPLP0/RPL12/RPL7A/SLC25A5/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/MYO18A/MSI2/RPL7A/RPL12/RPL10/SUB1/RPS19/RPL10A/HNRNPR/UBE2O/RPS28/RTRAF/FUS/RPL22/SRSF2/RPL27/EIF3C/RPL4/RPL11/RPL7/EIF4A1/RPS16/RPL18A/LSM4/RPS25/HNRNPH1/ECHDC2/RPS3A/RPS21/XIRP1/EIF2S3/FARSB/RPL13A/ABCF1/NPM1/NARS1/RPLP0/RPS15A/PA2G4/RPS24/RPL30/SLC25A5/RPL13/CORO1A/RPL17/RPS3/NCL</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005198</t>
@@ -2758,7 +2758,7 @@
     <t xml:space="preserve">189/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL18/RPL10A/RPL15/RPS28/RPL10/RPL18A/RPS25/MYBPH/RPL17/RPL22/RPL7/ASPH/RPL11/RPL13A/RPS21/RPS3/RPS3A/RPS24/RPS16/RPL14/RPL4/RPLP2/RPL27/RPL13/RPS19/RPS15A/RPLP0/ARPC2/RPL12/RPL7A/RPL30</t>
+    <t xml:space="preserve">RPL18/RPL14/RPL15/RPL7A/RPL12/RPL10/RPS19/RPL10A/RPS28/RPL22/RPL27/RPL4/RPL11/ASPH/ARPC2/RPL7/RPS16/RPL18A/RPS25/RPS3A/RPS21/RPLP2/RPL13A/RPLP0/RPS15A/RPS24/RPL30/RPL13/RPL17/MYBPH/RPS3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030029</t>
@@ -2773,13 +2773,13 @@
     <t xml:space="preserve">154/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TNNT3/TNNT1/MYL6/TTN/MYL2/MYOM2/ACTN4/SYNPO2L/MYOZ1/TPM3/MYOM1/TPM1/MYL6B/MYL1/PDLIM7/NEB/MYBPC2/ACTB/CAPZB/SYNPO2/TMOD1/MYH2/PLEC/TNNC1/MYBPC1/MYH4/SYNPO/ACTA1/TCAP/TPM2/ACTN2/PDLIM5/OBSCN/MYOM3/MYH7/CORO6/CAPZA2/ACTN3</t>
+    <t xml:space="preserve">MYL6/OBSCN/MYOM3/MYOM2/MYL2/TMOD1/TPM2/TTN/CAPZB/MYOM1/MYOZ1/PDLIM7/ACTN3/SYNPO2L/ACTN4/TNNC1/MYBPC1/MYH4/MYL1/MYH2/ACTA1/SYNPO/SYNPO2/ACTN1/ACTN2/TNNT3/PDLIM5/TPM3/MYL6B/ACTB/TPM1/TCAP/CAPZA2/MYH7/CORO6/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">37/77</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TNNT3/TNNT1/MYL6/TTN/MYL2/MYOM2/ACTN4/SYNPO2L/MYOZ1/MYOM1/TPM1/MYL6B/LMNA/PDLIM7/DES/NEB/MYBPC2/LAMC1/ACTB/MYL3/TMOD1/NID1/PLEC/TNNC1/MYBPC1/COL6A1/ACTA1/TCAP/RPL27A/ACTN2/COL6A3/PDLIM5/OBSCN/MYOM3/MYH7/ACTN3</t>
+    <t xml:space="preserve">MYL6/OBSCN/MYOM3/COL6A3/MYOM2/MYL2/TMOD1/RPL27A/TTN/MYOM1/MYOZ1/DES/PDLIM7/ACTN3/SYNPO2L/ACTN4/TNNC1/MYBPC1/LAMC1/COL6A1/ACTA1/ACTN1/ACTN2/TNNT3/PDLIM5/MYL6B/LMNA/ACTB/MYL3/TPM1/TCAP/MYH7/NID1/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0055001</t>
@@ -2794,7 +2794,7 @@
     <t xml:space="preserve">51/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TNNT3/TNNT1/TTN/MYL2/MYOM2/ACTN4/SYNPO2L/MYOZ1/MYOM1/TPM1/NEB/MYBPC2/TMOD1/PLEC/MYBPC1/COL6A1/ACTA1/TCAP/ACTN2/PDLIM5/OBSCN/MYOM3/ACTN3</t>
+    <t xml:space="preserve">OBSCN/MYOM3/MYOM2/MYL2/TMOD1/TTN/MYOM1/MYOZ1/ACTN3/SYNPO2L/ACTN4/MYBPC1/COL6A1/ACTA1/ACTN1/ACTN2/TNNT3/PDLIM5/TPM1/TCAP/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0055002</t>
@@ -2809,7 +2809,7 @@
     <t xml:space="preserve">47/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNT3/TNNT1/TTN/MYL2/MYOM2/SYNPO2L/MYOZ1/MYOM1/TPM1/NEB/MYBPC2/TMOD1/PLEC/MYBPC1/COL6A1/ACTA1/TCAP/ACTN2/PDLIM5/OBSCN/MYOM3/ACTN3</t>
+    <t xml:space="preserve">OBSCN/MYOM3/MYOM2/MYL2/TMOD1/TTN/MYOM1/MYOZ1/ACTN3/SYNPO2L/MYBPC1/COL6A1/ACTA1/ACTN2/TNNT3/PDLIM5/TPM1/TCAP/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030239</t>
@@ -2821,19 +2821,19 @@
     <t xml:space="preserve">19/77</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNT3/TNNT1/TTN/MYL2/MYOM2/SYNPO2L/MYOZ1/MYOM1/TPM1/NEB/MYBPC2/TMOD1/PLEC/MYBPC1/ACTA1/TCAP/ACTN2/OBSCN/MYOM3</t>
+    <t xml:space="preserve">OBSCN/MYOM3/MYOM2/MYL2/TMOD1/TTN/MYOM1/MYOZ1/SYNPO2L/MYBPC1/ACTA1/ACTN2/TNNT3/TPM1/TCAP/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">34/77</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNT3/TNNT1/TNNI2/MYL6/TNNC2/MYH13/TTN/MYL2/MYOM2/MYOZ1/TPM3/TPM1/MYH1/MYL6B/LMNA/MYL1/DES/SYNM/MYL3/TMOD1/MYH2/TNNC1/MYH4/ACTA1/TCAP/TPM2/RPL27A/TNNI1/PDLIM5/JPH1/MYL4/MYH7/MYOT/ACTN3</t>
+    <t xml:space="preserve">TNNI2/MYL6/MYOT/MYL4/MYOM2/MYL2/TMOD1/TPM2/RPL27A/TTN/MYH13/MYOZ1/DES/ACTN3/TNNC1/MYH4/MYL1/MYH2/ACTA1/SYNM/TNNT3/TNNI1/PDLIM5/TPM3/MYL6B/LMNA/MYH1/JPH1/MYL3/TPM1/TCAP/TNNC2/MYH7/TNNT1</t>
   </si>
   <si>
     <t xml:space="preserve">32/77</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TNNT3/TNNT1/TTN/MYL2/MYOM2/ACTN4/SYNPO2L/MYOZ1/TPM3/MYOM1/TPM1/PDLIM7/NEB/MYBPC2/ACTB/CAPZB/SYNPO2/TMOD1/PLEC/MYBPC1/SYNPO/ACTA1/TCAP/TPM2/ACTN2/PDLIM5/OBSCN/MYOM3/CORO6/CAPZA2/ACTN3</t>
+    <t xml:space="preserve">OBSCN/MYOM3/MYOM2/MYL2/TMOD1/TPM2/TTN/CAPZB/MYOM1/MYOZ1/PDLIM7/ACTN3/SYNPO2L/ACTN4/MYBPC1/ACTA1/SYNPO/SYNPO2/ACTN1/ACTN2/TNNT3/PDLIM5/TPM3/ACTB/TPM1/TCAP/CAPZA2/CORO6/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0010927</t>
@@ -2851,13 +2851,13 @@
     <t xml:space="preserve">31/77</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNT3/TNNT1/TNNI2/MYL6/TNNC2/MYH13/TTN/MYL2/MYOM2/TPM3/TPM1/MYH1/MYL6B/MYL1/DES/SYNM/MYL3/TMOD1/MYH2/TNNC1/MYH4/ACTA1/TCAP/TPM2/RPL27A/TNNI1/JPH1/MYL4/MYH7/MYOT/ACTN3</t>
+    <t xml:space="preserve">TNNI2/MYL6/MYOT/MYL4/MYOM2/MYL2/TMOD1/TPM2/RPL27A/TTN/MYH13/DES/ACTN3/TNNC1/MYH4/MYL1/MYH2/ACTA1/SYNM/TNNT3/TNNI1/TPM3/MYL6B/MYH1/JPH1/MYL3/TPM1/TCAP/TNNC2/MYH7/TNNT1</t>
   </si>
   <si>
     <t xml:space="preserve">27/77</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TNNT3/TNNT1/TTN/MYL2/MYOM2/ACTN4/SYNPO2L/MYOZ1/MYOM1/TPM1/NEB/MYBPC2/LAMC1/TMOD1/NID1/PLEC/MYBPC1/COL6A1/ACTA1/TCAP/RPL27A/ACTN2/PDLIM5/OBSCN/MYOM3/ACTN3</t>
+    <t xml:space="preserve">OBSCN/MYOM3/MYOM2/MYL2/TMOD1/RPL27A/TTN/MYOM1/MYOZ1/ACTN3/SYNPO2L/ACTN4/MYBPC1/LAMC1/COL6A1/ACTA1/ACTN1/ACTN2/TNNT3/PDLIM5/TPM1/TCAP/NID1/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0045214</t>
@@ -2869,10 +2869,10 @@
     <t xml:space="preserve">15/77</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNT3/TNNT1/TTN/MYOM2/SYNPO2L/MYOZ1/MYOM1/TPM1/MYBPC2/PLEC/MYBPC1/TCAP/ACTN2/OBSCN/MYOM3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACTN1/TNNT3/TNNT1/HSPG2/TTN/MYL2/MYOM2/SYNPO2L/MYOZ1/TPM3/MYOM1/TPM1/DES/NEB/MYBPC2/ACTB/CAPZB/SYNPO2/TMOD1/PLEC/MYBPC1/SYNPO/ACTA1/TCAP/TPM2/ACTN2/VIM/OBSCN/MYOM3/CORO6/CAPZA2</t>
+    <t xml:space="preserve">OBSCN/MYOM3/MYOM2/TTN/MYOM1/MYOZ1/SYNPO2L/MYBPC1/ACTN2/TNNT3/TPM1/TCAP/PLEC/TNNT1/MYBPC2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OBSCN/MYOM3/MYOM2/MYL2/TMOD1/TPM2/TTN/CAPZB/MYOM1/MYOZ1/DES/SYNPO2L/MYBPC1/HSPG2/ACTA1/SYNPO/SYNPO2/ACTN1/VIM/ACTN2/TNNT3/TPM3/ACTB/TPM1/TCAP/CAPZA2/CORO6/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0031032</t>
@@ -2887,22 +2887,22 @@
     <t xml:space="preserve">57/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNT3/TNNT1/TTN/MYL2/MYOM2/SYNPO2L/MYOZ1/MYOM1/TPM1/NEB/MYBPC2/TMOD1/PLEC/MYBPC1/SYNPO/ACTA1/TCAP/ACTN2/OBSCN/MYOM3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACTN1/TNNT3/TNNT1/TTN/MYL2/MYOM2/ACTN4/SYNPO2L/MYOZ1/TPM3/MYOM1/TPM1/LMNA/PDLIM7/DES/NEB/MYBPC2/SYNM/ACTB/CAPZB/SYNPO2/TMOD1/PLEC/CSNK1A1/MYBPC1/SYNPO/ACTA1/TCAP/TPM2/ACTN2/VIM/PDLIM5/OBSCN/MYOM3/CORO6/CAPZA2/ACTN3</t>
+    <t xml:space="preserve">OBSCN/MYOM3/MYOM2/MYL2/TMOD1/TTN/MYOM1/MYOZ1/SYNPO2L/MYBPC1/ACTA1/SYNPO/ACTN2/TNNT3/TPM1/TCAP/PLEC/TNNT1/MYBPC2/NEB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OBSCN/MYOM3/MYOM2/MYL2/TMOD1/TPM2/TTN/CAPZB/MYOM1/MYOZ1/DES/PDLIM7/ACTN3/SYNPO2L/ACTN4/MYBPC1/ACTA1/SYNPO/SYNPO2/SYNM/ACTN1/VIM/ACTN2/TNNT3/PDLIM5/TPM3/LMNA/ACTB/TPM1/TCAP/CAPZA2/CORO6/CSNK1A1/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">36/77</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNT3/TNNT1/TNNI2/MYL6/TNNC2/MYH13/COL1A2/TTN/MYL2/MYOM2/MYOZ1/TPM3/TPM1/MYH1/MYL6B/LMNA/MYL1/DES/SYNM/MYL3/TMOD1/MYH2/PLEC/TNNC1/MYH4/ACTA1/TCAP/TPM2/RPL27A/TNNI1/PDLIM5/JPH1/MYL4/MYH7/MYOT/ACTN3</t>
+    <t xml:space="preserve">TNNI2/MYL6/MYOT/MYL4/MYOM2/MYL2/TMOD1/TPM2/RPL27A/TTN/MYH13/MYOZ1/DES/ACTN3/TNNC1/MYH4/MYL1/MYH2/ACTA1/SYNM/TNNT3/TNNI1/PDLIM5/TPM3/MYL6B/LMNA/MYH1/JPH1/MYL3/COL1A2/TPM1/TCAP/TNNC2/MYH7/PLEC/TNNT1</t>
   </si>
   <si>
     <t xml:space="preserve">23/77</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNT3/TNNT1/TTN/MYL2/MYOM2/SYNPO2L/MYOZ1/MYOM1/TPM1/NEB/MYBPC2/TMOD1/PLEC/MYBPC1/COL6A1/ACTA1/TCAP/RPL27A/ACTN2/PDLIM5/OBSCN/MYOM3/ACTN3</t>
+    <t xml:space="preserve">OBSCN/MYOM3/MYOM2/MYL2/TMOD1/RPL27A/TTN/MYOM1/MYOZ1/ACTN3/SYNPO2L/MYBPC1/COL6A1/ACTA1/ACTN2/TNNT3/PDLIM5/TPM1/TCAP/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0014706</t>
@@ -2914,7 +2914,7 @@
     <t xml:space="preserve">18/77</t>
   </si>
   <si>
-    <t xml:space="preserve">MYL6/TTN/MYL2/MYOZ1/MYOM1/TPM1/MYL6B/NEB/MYL3/PLEC/TNNC1/COL6A1/ACTA1/TCAP/ACTN2/PDLIM5/MYH7/ACTN3</t>
+    <t xml:space="preserve">MYL6/MYL2/TTN/MYOM1/MYOZ1/ACTN3/TNNC1/COL6A1/ACTA1/ACTN2/PDLIM5/MYL6B/MYL3/TPM1/TCAP/MYH7/PLEC/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0060537</t>
@@ -2929,7 +2929,7 @@
     <t xml:space="preserve">35/77</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/COL15A1/TNNT3/TNNT1/COL4A2/HSPG2/COL1A2/TTN/MYL2/MYOM2/SYNPO2L/MYOZ1/MYOM1/TPM1/NEB/MYBPC2/ACTB/MYL3/TMOD1/PLEC/TNNC1/MYBPC1/COL6A1/ACTA1/TCAP/RPL27A/ACTN2/AGO2/VIM/PDLIM5/OBSCN/MYOM3/MYH7/MYOT/ACTN3</t>
+    <t xml:space="preserve">OBSCN/MYOT/MYOM3/MYOM2/MYL2/TMOD1/RPL27A/TTN/MYOM1/MYOZ1/ACTN3/SYNPO2L/TNNC1/MYBPC1/HSPG2/COL6A1/ACTA1/ACTN1/VIM/AGO2/COL4A2/ACTN2/TNNT3/PDLIM5/ACTB/COL15A1/MYL3/COL1A2/TPM1/TCAP/MYH7/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0007517</t>
@@ -2941,7 +2941,7 @@
     <t xml:space="preserve">63/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">MYL6/TTN/MYL2/MYOZ1/MYOM1/TPM1/MYL6B/LMNA/DES/NEB/MYL3/PLEC/TNNC1/COL6A1/ACTA1/TCAP/COL6A3/MYH7/ACTN3</t>
+    <t xml:space="preserve">MYL6/COL6A3/MYL2/TTN/MYOM1/MYOZ1/DES/ACTN3/TNNC1/COL6A1/ACTA1/MYL6B/LMNA/MYL3/TPM1/TCAP/MYH7/PLEC/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030049</t>
@@ -2956,7 +2956,7 @@
     <t xml:space="preserve">14/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">MYL6/TTN/TPM1/MYL6B/MYL1/MYH2/TNNC1/MYH4/TCAP/MYH7</t>
+    <t xml:space="preserve">MYL6/TTN/TNNC1/MYH4/MYL1/MYH2/MYL6B/TPM1/TCAP/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0033275</t>
@@ -2974,13 +2974,13 @@
     <t xml:space="preserve">21/77</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNT3/TNNT1/H3-3A/TTN/MYL2/MYOM2/SYNPO2L/MYOZ1/MYOM1/TPM1/NEB/MYBPC2/TMOD1/PLEC/MYBPC1/ACTA1/TCAP/ACTN2/AGO2/OBSCN/MYOM3</t>
+    <t xml:space="preserve">OBSCN/MYOM3/MYOM2/MYL2/TMOD1/TTN/MYOM1/MYOZ1/SYNPO2L/MYBPC1/ACTA1/AGO2/ACTN2/TNNT3/TPM1/TCAP/H3-3A/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">26/77</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/COL15A1/TNNT3/TNNT1/COL4A2/HSPG2/TTN/MYL2/MYOM2/SYNPO2L/MYOZ1/MYOM1/TPM1/NEB/MYBPC2/TMOD1/PLEC/MYBPC1/COL6A1/ACTA1/TCAP/RPL27A/ACTN2/AGO2/OBSCN/MYOM3</t>
+    <t xml:space="preserve">OBSCN/MYOM3/MYOM2/MYL2/TMOD1/RPL27A/TTN/MYOM1/MYOZ1/SYNPO2L/MYBPC1/HSPG2/COL6A1/ACTA1/ACTN1/AGO2/COL4A2/ACTN2/TNNT3/COL15A1/TPM1/TCAP/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0003009</t>
@@ -2992,7 +2992,7 @@
     <t xml:space="preserve">11/77</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNT3/TNNT1/TNNI2/TNNC2/TTN/SYNM/TNNC1/TCAP/TNNI1/MYH7/ACTN3</t>
+    <t xml:space="preserve">TNNI2/TTN/ACTN3/TNNC1/SYNM/TNNT3/TNNI1/TCAP/TNNC2/MYH7/TNNT1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0048738</t>
@@ -3001,7 +3001,7 @@
     <t xml:space="preserve">cardiac muscle tissue development</t>
   </si>
   <si>
-    <t xml:space="preserve">TTN/MYL2/TPM1/NEB/MYL3/PLEC/TNNC1/TCAP/ACTN2/PDLIM5/MYH7</t>
+    <t xml:space="preserve">MYL2/TTN/TNNC1/ACTN2/PDLIM5/MYL3/TPM1/TCAP/MYH7/PLEC/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0048468</t>
@@ -3013,7 +3013,7 @@
     <t xml:space="preserve">28/77</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TNNT3/TNNT1/TTN/MYL2/MYOM2/ACTN4/SYNPO2L/MYOZ1/H4C1/MYOM1/TPM1/NEB/MYBPC2/ACTB/TMOD1/PLEC/MYBPC1/COL6A1/ACTA1/TCAP/ACTN2/VIM/PDLIM5/OBSCN/MYOM3/MYOT/ACTN3</t>
+    <t xml:space="preserve">OBSCN/MYOT/MYOM3/MYOM2/MYL2/TMOD1/TTN/MYOM1/MYOZ1/ACTN3/SYNPO2L/ACTN4/MYBPC1/COL6A1/ACTA1/ACTN1/VIM/ACTN2/TNNT3/PDLIM5/H4C1/ACTB/TPM1/TCAP/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0050879</t>
@@ -3043,13 +3043,13 @@
     <t xml:space="preserve">475/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/COL15A1/TNNT3/TNNT1/COL4A2/MYL6/CD63/HSPG2/COL1A2/TTN/MYL2/MYOM2/ACTN4/SYNPO2L/MYOZ1/H4C1/MYOM1/TPM1/MYL6B/LMNA/PDLIM7/DES/NEB/MYBPC2/LAMC1/ACTB/MYL3/TMOD1/NID1/PLEC/TNNC1/MYBPC1/COL6A1/ACTA1/TCAP/RPL27A/ACTN2/AGO2/VIM/COL6A3/PDLIM5/OBSCN/MYOM3/MYH7/MYOT/ACTN3</t>
+    <t xml:space="preserve">MYL6/OBSCN/MYOT/MYOM3/COL6A3/MYOM2/MYL2/TMOD1/RPL27A/TTN/MYOM1/CD63/MYOZ1/DES/PDLIM7/ACTN3/SYNPO2L/ACTN4/TNNC1/MYBPC1/HSPG2/LAMC1/COL6A1/ACTA1/ACTN1/VIM/AGO2/COL4A2/ACTN2/TNNT3/PDLIM5/H4C1/MYL6B/LMNA/ACTB/COL15A1/MYL3/COL1A2/TPM1/TCAP/MYH7/NID1/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">17/77</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TTN/SYNPO2L/TPM3/TPM1/NEB/CAPZB/SYNPO2/TMOD1/PLEC/SYNPO/ACTA1/TCAP/TPM2/ACTN2/CORO6/CAPZA2</t>
+    <t xml:space="preserve">TMOD1/TPM2/TTN/CAPZB/SYNPO2L/ACTA1/SYNPO/SYNPO2/ACTN1/ACTN2/TPM3/TPM1/TCAP/CAPZA2/CORO6/PLEC/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0070925</t>
@@ -3061,7 +3061,7 @@
     <t xml:space="preserve">140/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">GORASP2/TNNT3/TNNT1/H3-3A/TTN/MYL2/MYOM2/SYNPO2L/MYOZ1/MYOM1/TPM1/NEB/MYBPC2/TMOD1/PLEC/MYBPC1/SYNPO/ACTA1/TCAP/ACTN2/AGO2/OBSCN/MYOM3</t>
+    <t xml:space="preserve">OBSCN/MYOM3/MYOM2/MYL2/TMOD1/TTN/MYOM1/MYOZ1/SYNPO2L/MYBPC1/ACTA1/SYNPO/AGO2/ACTN2/GORASP2/TNNT3/TPM1/TCAP/H3-3A/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0050905</t>
@@ -3079,7 +3079,7 @@
     <t xml:space="preserve">7/77</t>
   </si>
   <si>
-    <t xml:space="preserve">TTN/MYL2/TPM1/MYL3/TNNC1/TCAP/MYH7</t>
+    <t xml:space="preserve">MYL2/TTN/TNNC1/MYL3/TPM1/TCAP/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0009888</t>
@@ -3091,7 +3091,7 @@
     <t xml:space="preserve">141/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">COL4A2/MYL6/CD63/TTN/MYL2/MYOZ1/MYOM1/TPM1/MYL6B/NEB/LAMC1/ACTB/MYL3/TMOD1/PLEC/TNNC1/COL6A1/ACTA1/TCAP/ACTN2/PDLIM5/MYH7/ACTN3</t>
+    <t xml:space="preserve">MYL6/MYL2/TMOD1/TTN/MYOM1/CD63/MYOZ1/ACTN3/TNNC1/LAMC1/COL6A1/ACTA1/COL4A2/ACTN2/PDLIM5/MYL6B/ACTB/MYL3/TPM1/TCAP/MYH7/PLEC/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0048644</t>
@@ -3121,7 +3121,7 @@
     <t xml:space="preserve">49/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">TTN/MYL2/SYNPO2L/TPM1/PDLIM7/NEB/MYL3/PLEC/TNNC1/TCAP/ACTN2/PDLIM5/MYH7</t>
+    <t xml:space="preserve">MYL2/TTN/PDLIM7/SYNPO2L/TNNC1/ACTN2/PDLIM5/MYL3/TPM1/TCAP/MYH7/PLEC/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030048</t>
@@ -3130,7 +3130,7 @@
     <t xml:space="preserve">actin filament-based movement</t>
   </si>
   <si>
-    <t xml:space="preserve">MYL6/TTN/ACTN4/TPM1/MYL6B/MYL1/MYH2/TNNC1/MYH4/TCAP/MYH7</t>
+    <t xml:space="preserve">MYL6/TTN/ACTN4/TNNC1/MYH4/MYL1/MYH2/MYL6B/TPM1/TCAP/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0060538</t>
@@ -3139,7 +3139,7 @@
     <t xml:space="preserve">skeletal muscle organ development</t>
   </si>
   <si>
-    <t xml:space="preserve">MYL6/MYOZ1/MYOM1/MYL6B/DES/MYL3/PLEC/COL6A1/ACTA1/ACTN3</t>
+    <t xml:space="preserve">MYL6/MYOM1/MYOZ1/DES/ACTN3/COL6A1/ACTA1/MYL6B/MYL3/PLEC</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0060048</t>
@@ -3151,7 +3151,7 @@
     <t xml:space="preserve">37/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNI2/TTN/MYL2/TPM1/MYL3/TNNC1/TCAP/TNNI1/JPH1/MYL4/MYH7</t>
+    <t xml:space="preserve">TNNI2/MYL4/MYL2/TTN/TNNC1/TNNI1/JPH1/MYL3/TPM1/TCAP/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0070252</t>
@@ -3169,7 +3169,7 @@
     <t xml:space="preserve">102/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">COL15A1/COL4A2/HSPG2/COL1A2/TTN/MYL2/SYNPO2L/TPM1/PDLIM7/NEB/MYL3/PLEC/TNNC1/TCAP/ACTN2/AGO2/PDLIM5/MYH7</t>
+    <t xml:space="preserve">MYL2/TTN/PDLIM7/SYNPO2L/TNNC1/HSPG2/AGO2/COL4A2/ACTN2/PDLIM5/COL15A1/MYL3/COL1A2/TPM1/TCAP/MYH7/PLEC/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0048513</t>
@@ -3181,19 +3181,19 @@
     <t xml:space="preserve">213/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">MYL6/HSPG2/COL1A2/TTN/MYL2/SYNPO2L/MYOZ1/MYOM1/TPM1/MYL6B/LMNA/PDLIM7/DES/NEB/ACTB/MYL3/TMOD1/PLEC/TNNC1/COL6A1/ACTA1/TCAP/ACTN2/COL6A3/PDLIM5/MYH7/ACTN3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GORASP2/ACTN1/COL15A1/TNNT3/TNNT1/COL4A2/CD63/HSPG2/TTN/MYL2/MYOM2/ACTN4/SYNPO2L/MYOZ1/H4C1/MYOM1/TPM1/PDLIM7/NEB/MYBPC2/LAMC1/ACTB/TMOD1/NID1/PLEC/MYBPC1/COL6A1/ACTA1/TCAP/RPL27A/ACTN2/VIM/PDLIM5/OBSCN/MYOM3/MYOT/ACTN3</t>
+    <t xml:space="preserve">MYL6/COL6A3/MYL2/TMOD1/TTN/MYOM1/MYOZ1/DES/PDLIM7/ACTN3/SYNPO2L/TNNC1/HSPG2/COL6A1/ACTA1/ACTN2/PDLIM5/MYL6B/LMNA/ACTB/MYL3/COL1A2/TPM1/TCAP/MYH7/PLEC/NEB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OBSCN/MYOT/MYOM3/MYOM2/MYL2/TMOD1/RPL27A/TTN/MYOM1/CD63/MYOZ1/PDLIM7/ACTN3/SYNPO2L/ACTN4/MYBPC1/HSPG2/LAMC1/COL6A1/ACTA1/ACTN1/VIM/COL4A2/ACTN2/GORASP2/TNNT3/PDLIM5/H4C1/ACTB/COL15A1/TPM1/TCAP/NID1/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">44/77</t>
   </si>
   <si>
-    <t xml:space="preserve">GORASP2/ACTN1/TNNT3/TNNT1/ATP6V1B2/BANF1/H1-4/H3-3A/TTN/MYL2/MYOM2/ACTN4/SYNPO2L/MYOZ1/TPM3/H4C1/MYOM1/TPM1/LMNA/PDLIM7/DES/NEB/MYBPC2/SYNM/ACTB/CAPZB/SYNPO2/TMOD1/PLEC/CSNK1A1/MYBPC1/SYNPO/ACTA1/TCAP/TPM2/ACTN2/AGO2/VIM/PDLIM5/OBSCN/MYOM3/CORO6/CAPZA2/ACTN3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TNNT3/TNNT1/TNNI2/TNNC2/TTN/MYL2/TPM1/SYNM/MYL3/TNNC1/TCAP/RPL27A/TNNI1/JPH1/MYL4/MYH7/ACTN3</t>
+    <t xml:space="preserve">OBSCN/MYOM3/BANF1/MYOM2/MYL2/TMOD1/TPM2/TTN/CAPZB/MYOM1/MYOZ1/H1-4/DES/PDLIM7/ACTN3/SYNPO2L/ACTN4/MYBPC1/ATP6V1B2/ACTA1/SYNPO/SYNPO2/SYNM/ACTN1/VIM/AGO2/ACTN2/GORASP2/TNNT3/PDLIM5/H4C1/TPM3/LMNA/ACTB/TPM1/TCAP/H3-3A/CAPZA2/CORO6/CSNK1A1/PLEC/TNNT1/MYBPC2/NEB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TNNI2/MYL4/MYL2/RPL27A/TTN/ACTN3/TNNC1/SYNM/TNNT3/TNNI1/JPH1/MYL3/TPM1/TCAP/TNNC2/MYH7/TNNT1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0007519</t>
@@ -3205,7 +3205,7 @@
     <t xml:space="preserve">9/77</t>
   </si>
   <si>
-    <t xml:space="preserve">MYL6/MYOZ1/MYOM1/MYL6B/MYL3/PLEC/COL6A1/ACTA1/ACTN3</t>
+    <t xml:space="preserve">MYL6/MYOM1/MYOZ1/ACTN3/COL6A1/ACTA1/MYL6B/MYL3/PLEC</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0003007</t>
@@ -3217,7 +3217,7 @@
     <t xml:space="preserve">8/77</t>
   </si>
   <si>
-    <t xml:space="preserve">TTN/MYL2/SYNPO2L/TPM1/MYL3/TNNC1/TCAP/MYH7</t>
+    <t xml:space="preserve">MYL2/TTN/SYNPO2L/TNNC1/MYL3/TPM1/TCAP/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006937</t>
@@ -3229,7 +3229,7 @@
     <t xml:space="preserve">42/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNT3/TNNT1/TNNC2/MYL2/TPM1/MYL3/TNNC1/TNNI1/JPH1/MYH7/ACTN3</t>
+    <t xml:space="preserve">MYL2/ACTN3/TNNC1/TNNT3/TNNI1/JPH1/MYL3/TPM1/TNNC2/MYH7/TNNT1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0055006</t>
@@ -3241,7 +3241,7 @@
     <t xml:space="preserve">15/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">TTN/MYL2/NEB/PLEC/TCAP/ACTN2/PDLIM5</t>
+    <t xml:space="preserve">MYL2/TTN/ACTN2/PDLIM5/TCAP/PLEC/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0055013</t>
@@ -3259,7 +3259,7 @@
     <t xml:space="preserve">12/77</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNI2/TTN/MYL2/TPM1/DES/MYL3/TNNC1/TCAP/TNNI1/JPH1/MYL4/MYH7</t>
+    <t xml:space="preserve">TNNI2/MYL4/MYL2/TTN/DES/TNNC1/TNNI1/JPH1/MYL3/TPM1/TCAP/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0008015</t>
@@ -3274,7 +3274,7 @@
     <t xml:space="preserve">70/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNI2/COL1A2/TTN/MYL2/TPM1/DES/MYL3/PLEC/TNNC1/TCAP/TNNI1/JPH1/MYL4/MYH7</t>
+    <t xml:space="preserve">TNNI2/MYL4/MYL2/TTN/DES/TNNC1/TNNI1/JPH1/MYL3/COL1A2/TPM1/TCAP/MYH7/PLEC</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0009887</t>
@@ -3283,7 +3283,7 @@
     <t xml:space="preserve">animal organ morphogenesis</t>
   </si>
   <si>
-    <t xml:space="preserve">COL1A2/TTN/MYL2/SYNPO2L/TPM1/MYL3/TNNC1/ACTA1/TCAP/MYH7/ACTN3</t>
+    <t xml:space="preserve">MYL2/TTN/ACTN3/SYNPO2L/TNNC1/ACTA1/MYL3/COL1A2/TPM1/TCAP/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0003015</t>
@@ -3298,7 +3298,7 @@
     <t xml:space="preserve">tissue morphogenesis</t>
   </si>
   <si>
-    <t xml:space="preserve">TTN/MYL2/TPM1/ACTB/MYL3/TNNC1/ACTA1/TCAP/MYH7</t>
+    <t xml:space="preserve">MYL2/TTN/TNNC1/ACTA1/ACTB/MYL3/TPM1/TCAP/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0090257</t>
@@ -3310,7 +3310,7 @@
     <t xml:space="preserve">54/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNT3/TNNT1/TNNC2/MYL2/TPM1/LMNA/MYL3/TNNC1/TNNI1/JPH1/MYH7/ACTN3</t>
+    <t xml:space="preserve">MYL2/ACTN3/TNNC1/TNNT3/TNNI1/LMNA/JPH1/MYL3/TPM1/TNNC2/MYH7/TNNT1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0055007</t>
@@ -3325,7 +3325,7 @@
     <t xml:space="preserve">regulation of system process</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNT3/TNNT1/TNNC2/MYL2/TPM1/LMNA/DES/MYL3/TNNC1/TNNI1/JPH1/MYL4/MYH7/ACTN3</t>
+    <t xml:space="preserve">MYL4/MYL2/DES/ACTN3/TNNC1/TNNT3/TNNI1/LMNA/JPH1/MYL3/TPM1/TNNC2/MYH7/TNNT1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0003013</t>
@@ -3349,7 +3349,7 @@
     <t xml:space="preserve">415/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">GORASP2/ACTN1/TNNT3/H2BC4/TNNT1/BANF1/H1-4/H3-3A/TTN/MYL2/MYOM2/SYNPO2L/MYOZ1/H4C1/MYOM1/TPM1/LMNA/NEB/MYBPC2/LAMC1/ACTB/CAPZB/SYNPO2/TMOD1/PLEC/CSNK1A1/MYBPC1/SYNPO/ACTA1/TCAP/ACTN2/AGO2/PDLIM5/OBSCN/MYOM3/CAPZA2/ACTN3</t>
+    <t xml:space="preserve">OBSCN/MYOM3/BANF1/MYOM2/MYL2/TMOD1/TTN/CAPZB/MYOM1/MYOZ1/H1-4/ACTN3/SYNPO2L/MYBPC1/LAMC1/ACTA1/SYNPO/SYNPO2/ACTN1/AGO2/H2BC4/ACTN2/GORASP2/TNNT3/PDLIM5/H4C1/LMNA/ACTB/TPM1/TCAP/H3-3A/CAPZA2/CSNK1A1/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0003206</t>
@@ -3361,7 +3361,7 @@
     <t xml:space="preserve">5/77</t>
   </si>
   <si>
-    <t xml:space="preserve">MYL2/TPM1/MYL3/TNNC1/MYH7</t>
+    <t xml:space="preserve">MYL2/TNNC1/MYL3/TPM1/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0050877</t>
@@ -3370,10 +3370,10 @@
     <t xml:space="preserve">nervous system process</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNT3/TNNT1/TNNI2/TNNC2/TTN/MYH1/SYNM/TNNC1/TCAP/TNNI1/MYH7/ACTN3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACTN1/COL15A1/CD63/ACTN4/TPM1/MYBPC2/LAMC1/ACTB/NID1/MYBPC1/COL6A1/ACTN2/COL6A3/COL6A2/PDLIM5/MYOT/ACTN3</t>
+    <t xml:space="preserve">TNNI2/TTN/ACTN3/TNNC1/SYNM/TNNT3/TNNI1/MYH1/TCAP/TNNC2/MYH7/TNNT1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MYOT/COL6A3/CD63/ACTN3/ACTN4/MYBPC1/LAMC1/COL6A1/ACTN1/ACTN2/PDLIM5/COL6A2/ACTB/COL15A1/TPM1/NID1/MYBPC2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0032956</t>
@@ -3385,7 +3385,7 @@
     <t xml:space="preserve">41/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">SYNPO2L/TPM1/NEB/CAPZB/SYNPO2/TMOD1/SYNPO/ACTN2/CAPZA2</t>
+    <t xml:space="preserve">TMOD1/CAPZB/SYNPO2L/SYNPO/SYNPO2/ACTN2/TPM1/CAPZA2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0032970</t>
@@ -3397,7 +3397,7 @@
     <t xml:space="preserve">52/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">SYNPO2L/TPM1/NEB/CAPZB/SYNPO2/TMOD1/TNNC1/SYNPO/ACTN2/CAPZA2</t>
+    <t xml:space="preserve">TMOD1/CAPZB/SYNPO2L/TNNC1/SYNPO/SYNPO2/ACTN2/TPM1/CAPZA2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0003205</t>
@@ -3427,7 +3427,7 @@
     <t xml:space="preserve">236/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNT3/TNNT1/COL4A2/BANF1/TNNC2/CD63/HSPG2/MYL2/MYOZ1/H4C1/TPM1/LMNA/DES/LAMC1/ACTB/MYL3/TNNC1/AGO2/VIM/TNNI1/JPH1/MYL4/MYH7/ACTN3</t>
+    <t xml:space="preserve">MYL4/BANF1/MYL2/CD63/MYOZ1/DES/ACTN3/TNNC1/HSPG2/LAMC1/VIM/AGO2/COL4A2/TNNT3/TNNI1/H4C1/LMNA/ACTB/JPH1/MYL3/TPM1/TNNC2/MYH7/TNNT1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006942</t>
@@ -3436,7 +3436,7 @@
     <t xml:space="preserve">regulation of striated muscle contraction</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNT3/MYL2/MYL3/TNNI1/JPH1/MYH7/ACTN3</t>
+    <t xml:space="preserve">MYL2/ACTN3/TNNT3/TNNI1/JPH1/MYL3/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0110053</t>
@@ -3445,7 +3445,7 @@
     <t xml:space="preserve">regulation of actin filament organization</t>
   </si>
   <si>
-    <t xml:space="preserve">SYNPO2L/TPM1/CAPZB/SYNPO2/TMOD1/SYNPO/ACTN2/CAPZA2</t>
+    <t xml:space="preserve">TMOD1/CAPZB/SYNPO2L/SYNPO/SYNPO2/ACTN2/TPM1/CAPZA2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0002026</t>
@@ -3457,7 +3457,7 @@
     <t xml:space="preserve">4/77</t>
   </si>
   <si>
-    <t xml:space="preserve">MYL2/MYL3/MYL4/MYH7</t>
+    <t xml:space="preserve">MYL4/MYL2/MYL3/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006334</t>
@@ -3466,7 +3466,7 @@
     <t xml:space="preserve">nucleosome assembly</t>
   </si>
   <si>
-    <t xml:space="preserve">H2BC4/H1-4/H3-3A/H4C1</t>
+    <t xml:space="preserve">H1-4/H2BC4/H4C1/H3-3A</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0014904</t>
@@ -3475,7 +3475,7 @@
     <t xml:space="preserve">myotube cell development</t>
   </si>
   <si>
-    <t xml:space="preserve">PLEC/COL6A1/ACTA1/ACTN3</t>
+    <t xml:space="preserve">ACTN3/COL6A1/ACTA1/PLEC</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0048741</t>
@@ -3493,10 +3493,10 @@
     <t xml:space="preserve">55/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">HSPG2/SYNPO2L/TPM1/CAPZB/SYNPO2/TMOD1/SYNPO/ACTN2/CAPZA2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COL15A1/COL4A2/COL1A2/LAMC1/NID1</t>
+    <t xml:space="preserve">TMOD1/CAPZB/SYNPO2L/HSPG2/SYNPO/SYNPO2/ACTN2/TPM1/CAPZA2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAMC1/COL4A2/COL15A1/COL1A2/NID1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0034728</t>
@@ -3511,7 +3511,7 @@
     <t xml:space="preserve">cell-substrate junction assembly</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/LAMC1/PLEC/ACTN2/ACTN3</t>
+    <t xml:space="preserve">ACTN3/LAMC1/ACTN1/ACTN2/PLEC</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0007275</t>
@@ -3523,7 +3523,7 @@
     <t xml:space="preserve">341/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">COL15A1/COL4A2/HSPG2/COL1A2/TTN/MYL2/SYNPO2L/MYOZ1/H4C1/MYOM1/TPM1/PDLIM7/NEB/LAMC1/ACTB/MYL3/TMOD1/PLEC/TNNC1/COL6A1/TCAP/ACTN2/AGO2/VIM/PDLIM5/MYH7/MYOT/ACTN3</t>
+    <t xml:space="preserve">MYOT/MYL2/TMOD1/TTN/MYOM1/MYOZ1/PDLIM7/ACTN3/SYNPO2L/TNNC1/HSPG2/LAMC1/COL6A1/VIM/AGO2/COL4A2/ACTN2/PDLIM5/H4C1/ACTB/COL15A1/MYL3/COL1A2/TPM1/TCAP/MYH7/PLEC/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0150115</t>
@@ -3538,7 +3538,7 @@
     <t xml:space="preserve">regulation of heart contraction</t>
   </si>
   <si>
-    <t xml:space="preserve">MYL2/TPM1/DES/MYL3/JPH1/MYL4/MYH7</t>
+    <t xml:space="preserve">MYL4/MYL2/DES/JPH1/MYL3/TPM1/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030832</t>
@@ -3550,7 +3550,7 @@
     <t xml:space="preserve">21/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">NEB/CAPZB/TMOD1/ACTN2/CAPZA2</t>
+    <t xml:space="preserve">TMOD1/CAPZB/ACTN2/CAPZA2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0065004</t>
@@ -3568,7 +3568,7 @@
     <t xml:space="preserve">cardiac muscle hypertrophy</t>
   </si>
   <si>
-    <t xml:space="preserve">TTN/LMNA/TCAP/PDLIM5</t>
+    <t xml:space="preserve">TTN/PDLIM5/LMNA/TCAP</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0014896</t>
@@ -3589,7 +3589,7 @@
     <t xml:space="preserve">regulation of actin filament depolymerization</t>
   </si>
   <si>
-    <t xml:space="preserve">CAPZB/TMOD1/ACTN2/CAPZA2</t>
+    <t xml:space="preserve">TMOD1/CAPZB/ACTN2/CAPZA2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0032233</t>
@@ -3598,7 +3598,7 @@
     <t xml:space="preserve">positive regulation of actin filament bundle assembly</t>
   </si>
   <si>
-    <t xml:space="preserve">SYNPO2L/TPM1/SYNPO2/SYNPO</t>
+    <t xml:space="preserve">SYNPO2L/SYNPO/SYNPO2/TPM1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:1903522</t>
@@ -3628,7 +3628,7 @@
     <t xml:space="preserve">296/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">COL15A1/COL4A2/HSPG2/COL1A2/TTN/MYL2/SYNPO2L/MYOM1/TPM1/PDLIM7/NEB/ACTB/MYL3/TMOD1/PLEC/TNNC1/TCAP/ACTN2/AGO2/VIM/PDLIM5/MYH7/MYOT/ACTN3</t>
+    <t xml:space="preserve">MYOT/MYL2/TMOD1/TTN/MYOM1/PDLIM7/ACTN3/SYNPO2L/TNNC1/HSPG2/VIM/AGO2/COL4A2/ACTN2/PDLIM5/ACTB/COL15A1/MYL3/COL1A2/TPM1/TCAP/MYH7/PLEC/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0043292</t>
@@ -3643,7 +3643,7 @@
     <t xml:space="preserve">124/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TNNT3/TNNT1/TNNI2/TNNC2/MYH13/TTN/MYL2/MYOM2/ACTN4/SYNPO2L/MYOZ1/TPM3/MYOM1/TPM1/MYOZ3/MYH1/MYL6B/MYL1/PDLIM7/DES/NEB/MYBPC2/SYNM/MYL3/CAPZB/SYNPO2/TMOD1/MYH2/PLEC/TNNC1/MYBPC1/MYH4/SYNPO/COL6A1/ACTA1/TCAP/TPM2/ACTN2/TNNI1/PDLIM5/JPH1/OBSCN/MYL4/MYOM3/MYH7/MYOT/ACTN3</t>
+    <t xml:space="preserve">TNNI2/OBSCN/MYOT/MYOM3/MYL4/MYOM2/MYL2/TMOD1/TPM2/TTN/CAPZB/MYOM1/MYH13/MYOZ1/DES/PDLIM7/ACTN3/SYNPO2L/ACTN4/TNNC1/MYBPC1/MYH4/MYL1/MYH2/COL6A1/ACTA1/SYNPO/SYNPO2/SYNM/ACTN1/ACTN2/TNNT3/TNNI1/PDLIM5/TPM3/MYL6B/MYH1/JPH1/MYL3/MYOZ3/TPM1/TCAP/TNNC2/MYH7/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030016</t>
@@ -3658,7 +3658,7 @@
     <t xml:space="preserve">122/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TNNT3/TNNT1/TNNI2/TNNC2/MYH13/TTN/MYL2/MYOM2/ACTN4/SYNPO2L/MYOZ1/TPM3/MYOM1/TPM1/MYOZ3/MYH1/MYL1/PDLIM7/DES/NEB/MYBPC2/SYNM/MYL3/CAPZB/SYNPO2/TMOD1/MYH2/PLEC/TNNC1/MYBPC1/MYH4/SYNPO/COL6A1/ACTA1/TCAP/TPM2/ACTN2/TNNI1/PDLIM5/JPH1/OBSCN/MYL4/MYOM3/MYH7/MYOT/ACTN3</t>
+    <t xml:space="preserve">TNNI2/OBSCN/MYOT/MYOM3/MYL4/MYOM2/MYL2/TMOD1/TPM2/TTN/CAPZB/MYOM1/MYH13/MYOZ1/DES/PDLIM7/ACTN3/SYNPO2L/ACTN4/TNNC1/MYBPC1/MYH4/MYL1/MYH2/COL6A1/ACTA1/SYNPO/SYNPO2/SYNM/ACTN1/ACTN2/TNNT3/TNNI1/PDLIM5/TPM3/MYH1/JPH1/MYL3/MYOZ3/TPM1/TCAP/TNNC2/MYH7/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0099080</t>
@@ -3673,7 +3673,7 @@
     <t xml:space="preserve">294/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TNNT3/TNNT1/COL4A2/TNNI2/H1-4/H3-3A/TNNC2/MYH13/HSPG2/COL1A2/TTN/MYL2/MYOM2/ACTN4/SYNPO2L/MYOZ1/TPM3/MYOM1/TPM1/MYOZ3/MYH1/MYL6B/LMNA/MYL1/PDLIM7/DES/NEB/MYBPC2/LAMC1/SYNM/ACTB/MYL3/CAPZB/SYNPO2/TMOD1/MYH2/PLEC/CSNK1A1/TNNC1/MYBPC1/MYH4/SYNPO/COL6A1/ACTA1/TCAP/TPM2/ACTN2/AGO2/VIM/COL6A3/TNNI1/COL6A2/PDLIM5/JPH1/OBSCN/MYL4/MYOM3/MYH7/CORO6/MYOT/ACTN3</t>
+    <t xml:space="preserve">TNNI2/OBSCN/MYOT/MYOM3/MYL4/COL6A3/MYOM2/MYL2/TMOD1/TPM2/TTN/CAPZB/MYOM1/MYH13/MYOZ1/H1-4/DES/PDLIM7/ACTN3/SYNPO2L/ACTN4/TNNC1/MYBPC1/MYH4/MYL1/HSPG2/LAMC1/MYH2/COL6A1/ACTA1/SYNPO/SYNPO2/SYNM/ACTN1/VIM/AGO2/COL4A2/ACTN2/TNNT3/TNNI1/PDLIM5/COL6A2/TPM3/MYL6B/LMNA/MYH1/ACTB/JPH1/MYL3/COL1A2/MYOZ3/TPM1/TCAP/H3-3A/TNNC2/MYH7/CORO6/CSNK1A1/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0099081</t>
@@ -3688,7 +3688,7 @@
     <t xml:space="preserve">221/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TNNT3/TNNT1/TNNI2/TNNC2/MYH13/HSPG2/TTN/MYL2/MYOM2/ACTN4/SYNPO2L/MYOZ1/TPM3/MYOM1/TPM1/MYOZ3/MYH1/MYL6B/LMNA/MYL1/PDLIM7/DES/NEB/MYBPC2/SYNM/ACTB/MYL3/CAPZB/SYNPO2/TMOD1/MYH2/PLEC/CSNK1A1/TNNC1/MYBPC1/MYH4/SYNPO/COL6A1/ACTA1/TCAP/TPM2/ACTN2/VIM/COL6A3/TNNI1/COL6A2/PDLIM5/JPH1/OBSCN/MYL4/MYOM3/MYH7/CORO6/MYOT/ACTN3</t>
+    <t xml:space="preserve">TNNI2/OBSCN/MYOT/MYOM3/MYL4/COL6A3/MYOM2/MYL2/TMOD1/TPM2/TTN/CAPZB/MYOM1/MYH13/MYOZ1/DES/PDLIM7/ACTN3/SYNPO2L/ACTN4/TNNC1/MYBPC1/MYH4/MYL1/HSPG2/MYH2/COL6A1/ACTA1/SYNPO/SYNPO2/SYNM/ACTN1/VIM/ACTN2/TNNT3/TNNI1/PDLIM5/COL6A2/TPM3/MYL6B/LMNA/MYH1/ACTB/JPH1/MYL3/MYOZ3/TPM1/TCAP/TNNC2/MYH7/CORO6/CSNK1A1/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0099512</t>
@@ -3709,16 +3709,16 @@
     <t xml:space="preserve">114/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TNNT3/TNNT1/TNNI2/TNNC2/TTN/MYL2/MYOM2/ACTN4/SYNPO2L/MYOZ1/TPM3/MYOM1/TPM1/MYOZ3/MYH1/MYL1/PDLIM7/DES/NEB/MYBPC2/MYL3/CAPZB/SYNPO2/TMOD1/MYH2/PLEC/TNNC1/MYBPC1/MYH4/SYNPO/ACTA1/TCAP/TPM2/ACTN2/TNNI1/PDLIM5/JPH1/OBSCN/MYL4/MYOM3/MYH7/MYOT/ACTN3</t>
+    <t xml:space="preserve">TNNI2/OBSCN/MYOT/MYOM3/MYL4/MYOM2/MYL2/TMOD1/TPM2/TTN/CAPZB/MYOM1/MYOZ1/DES/PDLIM7/ACTN3/SYNPO2L/ACTN4/TNNC1/MYBPC1/MYH4/MYL1/MYH2/ACTA1/SYNPO/SYNPO2/ACTN1/ACTN2/TNNT3/TNNI1/PDLIM5/TPM3/MYH1/JPH1/MYL3/MYOZ3/TPM1/TCAP/TNNC2/MYH7/PLEC/TNNT1/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">42/78</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TNNT3/TNNT1/TNNI2/LANCL2/MYL6/TNNC2/MYH13/TTN/MYL2/ACTN4/SYNPO2L/MYOZ1/TPM3/TPM1/MYOZ3/MYH1/MYL6B/MYL1/PDLIM7/NEB/ACTB/MYL3/CAPZB/SYNPO2/TMOD1/MYH2/PLEC/TNNC1/MYH4/SYNPO/ACTA1/TPM2/ACTN2/TNNI1/PDLIM5/MYL4/MYH7/CORO6/CAPZA2/MYOT/ACTN3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACTN1/TNNT3/TNNT1/TNNI2/LANCL2/MYL6/TNNC2/MYH13/TTN/MYL2/ACTN4/SYNPO2L/MYOZ1/TPM3/TPM1/MYOZ3/MYH1/MYL6B/LMNA/MYL1/PDLIM7/DES/NEB/SYNM/ACTB/MYL3/CAPZB/SYNPO2/TMOD1/MYH2/PLEC/CSNK1A1/TNNC1/MYH4/SYNPO/ACTA1/TPM2/ACTN2/VIM/TNNI1/PDLIM5/MYL4/MYH7/CORO6/CAPZA2/MYOT/ACTN3</t>
+    <t xml:space="preserve">TNNI2/MYL6/MYOT/MYL4/MYL2/TMOD1/TPM2/TTN/CAPZB/MYH13/LANCL2/MYOZ1/PDLIM7/ACTN3/SYNPO2L/ACTN4/TNNC1/MYH4/MYL1/MYH2/ACTA1/SYNPO/SYNPO2/ACTN1/ACTN2/TNNT3/TNNI1/PDLIM5/TPM3/MYL6B/MYH1/ACTB/MYL3/MYOZ3/TPM1/TNNC2/CAPZA2/MYH7/CORO6/PLEC/TNNT1/NEB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TNNI2/MYL6/MYOT/MYL4/MYL2/TMOD1/TPM2/TTN/CAPZB/MYH13/LANCL2/MYOZ1/DES/PDLIM7/ACTN3/SYNPO2L/ACTN4/TNNC1/MYH4/MYL1/MYH2/ACTA1/SYNPO/SYNPO2/SYNM/ACTN1/VIM/ACTN2/TNNT3/TNNI1/PDLIM5/TPM3/MYL6B/LMNA/MYH1/ACTB/MYL3/MYOZ3/TPM1/TNNC2/CAPZA2/MYH7/CORO6/CSNK1A1/PLEC/TNNT1/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0036379</t>
@@ -3730,7 +3730,7 @@
     <t xml:space="preserve">13/78</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNT3/TNNT1/TNNI2/TNNC2/TTN/TPM3/MYOM1/TPM1/TMOD1/TNNC1/ACTA1/TPM2/TNNI1</t>
+    <t xml:space="preserve">TNNI2/TMOD1/TPM2/TTN/MYOM1/TNNC1/ACTA1/TNNT3/TNNI1/TPM3/TPM1/TNNC2/TNNT1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005865</t>
@@ -3742,7 +3742,7 @@
     <t xml:space="preserve">12/78</t>
   </si>
   <si>
-    <t xml:space="preserve">TNNT3/TNNT1/TNNI2/TNNC2/TTN/TPM3/TPM1/TMOD1/TNNC1/ACTA1/TPM2/TNNI1</t>
+    <t xml:space="preserve">TNNI2/TMOD1/TPM2/TTN/TNNC1/ACTA1/TNNT3/TNNI1/TPM3/TPM1/TNNC2/TNNT1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030018</t>
@@ -3754,7 +3754,7 @@
     <t xml:space="preserve">20/78</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TTN/ACTN4/SYNPO2L/MYOZ1/MYOZ3/PDLIM7/DES/NEB/SYNPO2/PLEC/SYNPO/TCAP/ACTN2/PDLIM5/JPH1/OBSCN/MYH7/MYOT/ACTN3</t>
+    <t xml:space="preserve">OBSCN/MYOT/TTN/MYOZ1/DES/PDLIM7/ACTN3/SYNPO2L/ACTN4/SYNPO/SYNPO2/ACTN1/ACTN2/PDLIM5/JPH1/MYOZ3/TCAP/MYH7/PLEC/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0031674</t>
@@ -3769,7 +3769,7 @@
     <t xml:space="preserve">73/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TTN/ACTN4/SYNPO2L/MYOZ1/MYOZ3/PDLIM7/DES/NEB/MYL3/SYNPO2/PLEC/SYNPO/TCAP/ACTN2/PDLIM5/JPH1/OBSCN/MYH7/MYOT/ACTN3</t>
+    <t xml:space="preserve">OBSCN/MYOT/TTN/MYOZ1/DES/PDLIM7/ACTN3/SYNPO2L/ACTN4/SYNPO/SYNPO2/ACTN1/ACTN2/PDLIM5/JPH1/MYL3/MYOZ3/TCAP/MYH7/PLEC/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0016459</t>
@@ -3784,7 +3784,7 @@
     <t xml:space="preserve">21/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">MYL6/MYH13/MYL2/MYH1/MYL6B/MYL1/MYL3/MYH2/MYH4/MYL4/MYH7</t>
+    <t xml:space="preserve">MYL6/MYL4/MYL2/MYH13/MYH4/MYL1/MYH2/MYL6B/MYH1/MYL3/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0016460</t>
@@ -3796,7 +3796,7 @@
     <t xml:space="preserve">10/78</t>
   </si>
   <si>
-    <t xml:space="preserve">MYL6/MYH13/MYH1/MYL6B/MYL1/MYL3/MYH2/MYH4/MYL4/MYH7</t>
+    <t xml:space="preserve">MYL6/MYL4/MYH13/MYH4/MYL1/MYH2/MYL6B/MYH1/MYL3/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005884</t>
@@ -3805,7 +3805,7 @@
     <t xml:space="preserve">actin filament</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TPM3/TPM1/PDLIM7/ACTB/TMOD1/ACTA1/TPM2/ACTN2/PDLIM5/CORO6/ACTN3</t>
+    <t xml:space="preserve">TMOD1/TPM2/PDLIM7/ACTN3/ACTA1/ACTN1/ACTN2/PDLIM5/TPM3/ACTB/TPM1/CORO6</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0031672</t>
@@ -3817,7 +3817,7 @@
     <t xml:space="preserve">26/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">TTN/MYL2/MYOM2/MYOM1/MYH1/MYBPC2/MYL3/MYBPC1/OBSCN/MYL4/MYOM3</t>
+    <t xml:space="preserve">OBSCN/MYOM3/MYL4/MYOM2/MYL2/TTN/MYOM1/MYBPC1/MYH1/MYL3/MYBPC2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005859</t>
@@ -3832,7 +3832,7 @@
     <t xml:space="preserve">12/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">MYH13/MYH1/MYL6B/MYL1/MYL3/MYH2/MYH4/MYH7</t>
+    <t xml:space="preserve">MYH13/MYH4/MYL1/MYH2/MYL6B/MYH1/MYL3/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0032982</t>
@@ -3844,13 +3844,13 @@
     <t xml:space="preserve">9/78</t>
   </si>
   <si>
-    <t xml:space="preserve">MYH13/MYOM2/MYOM1/MYH1/MYBPC2/MYH2/MYBPC1/MYH4/MYH7</t>
+    <t xml:space="preserve">MYOM2/MYOM1/MYH13/MYBPC1/MYH4/MYH2/MYH1/MYH7/MYBPC2</t>
   </si>
   <si>
     <t xml:space="preserve">18/78</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TPM3/TPM1/LMNA/PDLIM7/DES/SYNM/ACTB/TMOD1/PLEC/CSNK1A1/ACTA1/TPM2/ACTN2/VIM/PDLIM5/CORO6/ACTN3</t>
+    <t xml:space="preserve">TMOD1/TPM2/DES/PDLIM7/ACTN3/ACTA1/SYNM/ACTN1/VIM/ACTN2/PDLIM5/TPM3/LMNA/ACTB/TPM1/CORO6/CSNK1A1/PLEC</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005604</t>
@@ -3865,7 +3865,7 @@
     <t xml:space="preserve">10/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">COL15A1/COL4A2/HSPG2/LAMC1/NID1/COL6A1</t>
+    <t xml:space="preserve">HSPG2/LAMC1/COL6A1/COL4A2/COL15A1/NID1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005882</t>
@@ -3874,7 +3874,7 @@
     <t xml:space="preserve">intermediate filament</t>
   </si>
   <si>
-    <t xml:space="preserve">LMNA/DES/SYNM/PLEC/CSNK1A1/VIM</t>
+    <t xml:space="preserve">DES/SYNM/VIM/LMNA/CSNK1A1/PLEC</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0001725</t>
@@ -3886,7 +3886,7 @@
     <t xml:space="preserve">36/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/ACTN4/TPM3/TPM1/PDLIM7/SYNPO2/SYNPO/ACTA1/PDLIM5/MYH7</t>
+    <t xml:space="preserve">PDLIM7/ACTN4/ACTA1/SYNPO/SYNPO2/ACTN1/PDLIM5/TPM3/TPM1/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0097517</t>
@@ -3928,13 +3928,13 @@
     <t xml:space="preserve">7/78</t>
   </si>
   <si>
-    <t xml:space="preserve">TTN/MYOM2/MYOM1/MYBPC2/MYBPC1/OBSCN/MYOM3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACTN1/LANCL2/ACTN4/ACTB/CAPZB/TMOD1/ACTN2/CAPZA2/ACTN3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COL15A1/COL4A2/HSPG2/COL1A2/LAMC1/NID1/COL6A1/COL6A3/COL6A2</t>
+    <t xml:space="preserve">OBSCN/MYOM3/MYOM2/TTN/MYOM1/MYBPC1/MYBPC2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TMOD1/CAPZB/LANCL2/ACTN3/ACTN4/ACTN1/ACTN2/ACTB/CAPZA2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COL6A3/HSPG2/LAMC1/COL6A1/COL4A2/COL6A2/COL15A1/COL1A2/NID1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0031143</t>
@@ -3946,7 +3946,7 @@
     <t xml:space="preserve">5/78</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/ACTN4/MYOZ1/ACTN2/ACTN3</t>
+    <t xml:space="preserve">MYOZ1/ACTN3/ACTN4/ACTN1/ACTN2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005903</t>
@@ -3955,10 +3955,10 @@
     <t xml:space="preserve">brush border</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/MYL6/ACTB/CAPZB/PLEC/CAPZA2/ACTN3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSPG2/COL1A2/COL6A1/COL6A3/COL6A2</t>
+    <t xml:space="preserve">MYL6/CAPZB/ACTN3/ACTN1/ACTB/CAPZA2/PLEC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COL6A3/HSPG2/COL6A1/COL6A2/COL1A2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0045177</t>
@@ -3970,7 +3970,7 @@
     <t xml:space="preserve">48/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/ATP6V1B2/MYL6/ACTB/CAPZB/PLEC/CAPZA2/ACTN3</t>
+    <t xml:space="preserve">MYL6/CAPZB/ACTN3/ATP6V1B2/ACTN1/ACTB/CAPZA2/PLEC</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005788</t>
@@ -3979,7 +3979,7 @@
     <t xml:space="preserve">endoplasmic reticulum lumen</t>
   </si>
   <si>
-    <t xml:space="preserve">COL15A1/COL4A2/COL1A2/LAMC1/COL6A1/COL6A3/COL6A2</t>
+    <t xml:space="preserve">COL6A3/LAMC1/COL6A1/COL4A2/COL6A2/COL15A1/COL1A2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0032993</t>
@@ -3994,10 +3994,10 @@
     <t xml:space="preserve">13/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/LANCL2/ACTN4/ACTN2/ACTN3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACTN1/ATP6V1B2/TPM1/PDLIM7/ACTB/CAPZB/ACTA1/VIM/CORO6</t>
+    <t xml:space="preserve">LANCL2/ACTN3/ACTN4/ACTN1/ACTN2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAPZB/PDLIM7/ATP6V1B2/ACTA1/ACTN1/VIM/ACTB/TPM1/CORO6</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0000793</t>
@@ -4009,10 +4009,10 @@
     <t xml:space="preserve">25/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">BANF1/H3-3A/TTN/ACTB/CSNK1A1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACTN1/MYH1/PDLIM7/DES/SYNM/ACTB/MYH2/SYNPO/PDLIM5</t>
+    <t xml:space="preserve">BANF1/TTN/ACTB/H3-3A/CSNK1A1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DES/PDLIM7/MYH2/SYNPO/SYNM/ACTN1/PDLIM5/MYH1/ACTB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0003779</t>
@@ -4027,7 +4027,7 @@
     <t xml:space="preserve">124/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TNNT3/TNNI2/TNNC2/MYH13/TTN/MYL2/ACTN4/SYNPO2L/MYOZ1/TPM3/TPM1/MYOZ3/MYH1/PDLIM7/NEB/MYBPC2/MYL3/CAPZB/SYNPO2/TMOD1/MYH2/PLEC/TNNC1/MYBPC1/MYH4/SYNPO/TPM2/ACTN2/TNNI1/PDLIM5/MYL4/MYH7/CORO6/CAPZA2/MYOT/ACTN3</t>
+    <t xml:space="preserve">TNNI2/MYOT/MYL4/MYL2/TMOD1/TPM2/TTN/CAPZB/MYH13/MYOZ1/PDLIM7/ACTN3/SYNPO2L/ACTN4/TNNC1/MYBPC1/MYH4/MYH2/SYNPO/SYNPO2/ACTN1/ACTN2/TNNT3/TNNI1/PDLIM5/TPM3/MYH1/MYL3/MYOZ3/TPM1/TNNC2/CAPZA2/MYH7/CORO6/PLEC/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0008307</t>
@@ -4042,7 +4042,7 @@
     <t xml:space="preserve">35/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">MYL6/TTN/MYL2/MYOM2/MYOM1/TPM1/MYL6B/MYL1/NEB/MYBPC2/SYNM/MYL3/PLEC/MYBPC1/TCAP/TPM2/ACTN2/JPH1/OBSCN/MYOM3/MYOT/ACTN3</t>
+    <t xml:space="preserve">MYL6/OBSCN/MYOT/MYOM3/MYOM2/MYL2/TPM2/TTN/MYOM1/ACTN3/MYBPC1/MYL1/SYNM/ACTN2/MYL6B/JPH1/MYL3/TPM1/TCAP/PLEC/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0008092</t>
@@ -4054,10 +4054,10 @@
     <t xml:space="preserve">208/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/TNNT3/TNNT1/TNNI2/TNNC2/MYH13/TTN/MYL2/ACTN4/SYNPO2L/MYOZ1/TPM3/TPM1/MYOZ3/MYH1/PDLIM7/DES/NEB/MYBPC2/SYNM/ACTB/MYL3/CAPZB/SYNPO2/TMOD1/MYH2/PLEC/TNNC1/MYBPC1/MYH4/SYNPO/ACTA1/TCAP/TPM2/ACTN2/TNNI1/PDLIM5/OBSCN/MYL4/MYH7/CORO6/CAPZA2/MYOT/ACTN3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACTN1/COL15A1/H2BC4/COL4A2/H1-4/MYL6/H3-3A/HSPG2/COL1A2/TTN/MYL2/MYOM2/H4C1/MYOM1/TPM1/MYL6B/LMNA/MYL1/DES/NEB/MYBPC2/LAMC1/SYNM/ACTB/MYL3/NID1/PLEC/MYBPC1/COL6A1/ACTA1/TCAP/TPM2/RPL27A/ACTN2/VIM/COL6A3/COL6A2/JPH1/OBSCN/MYOM3/MYOT/ACTN3</t>
+    <t xml:space="preserve">TNNI2/OBSCN/MYOT/MYL4/MYL2/TMOD1/TPM2/TTN/CAPZB/MYH13/MYOZ1/DES/PDLIM7/ACTN3/SYNPO2L/ACTN4/TNNC1/MYBPC1/MYH4/MYH2/ACTA1/SYNPO/SYNPO2/SYNM/ACTN1/ACTN2/TNNT3/TNNI1/PDLIM5/TPM3/MYH1/ACTB/MYL3/MYOZ3/TPM1/TCAP/TNNC2/CAPZA2/MYH7/CORO6/PLEC/TNNT1/MYBPC2/NEB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MYL6/OBSCN/MYOT/MYOM3/COL6A3/MYOM2/MYL2/TPM2/RPL27A/TTN/MYOM1/H1-4/DES/ACTN3/MYBPC1/MYL1/HSPG2/LAMC1/COL6A1/ACTA1/SYNM/ACTN1/VIM/COL4A2/H2BC4/ACTN2/COL6A2/H4C1/MYL6B/LMNA/ACTB/JPH1/COL15A1/MYL3/COL1A2/TPM1/TCAP/H3-3A/NID1/PLEC/MYBPC2/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0051015</t>
@@ -4072,7 +4072,7 @@
     <t xml:space="preserve">65/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/MYH13/TTN/ACTN4/TPM3/TPM1/MYH1/NEB/MYH2/PLEC/TNNC1/MYH4/TPM2/ACTN2/MYL4/MYH7/CORO6/CAPZA2/ACTN3</t>
+    <t xml:space="preserve">MYL4/TPM2/TTN/MYH13/ACTN3/ACTN4/TNNC1/MYH4/MYH2/ACTN1/ACTN2/TPM3/MYH1/TPM1/CAPZA2/MYH7/CORO6/PLEC/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0000146</t>
@@ -4084,7 +4084,7 @@
     <t xml:space="preserve">16/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">MYL6/MYH13/MYH1/MYL6B/MYL1/MYH2/MYH4/MYH7</t>
+    <t xml:space="preserve">MYL6/MYH13/MYH4/MYL1/MYH2/MYL6B/MYH1/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0003774</t>
@@ -4093,7 +4093,7 @@
     <t xml:space="preserve">cytoskeletal motor activity</t>
   </si>
   <si>
-    <t xml:space="preserve">MYL6/MYH13/MYH1/MYL6B/MYL1/MYL3/MYH2/MYH4/MYH7</t>
+    <t xml:space="preserve">MYL6/MYH13/MYH4/MYL1/MYH2/MYL6B/MYH1/MYL3/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0044877</t>
@@ -4108,13 +4108,13 @@
     <t xml:space="preserve">225/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/H1-4/H3-3A/CD63/MYH13/HSPG2/TTN/ACTN4/TPM3/TPM1/MYH1/NEB/ACTB/MYH2/NID1/PLEC/TNNC1/MYH4/COL6A1/TPM2/ACTN2/COL6A2/MYL4/MYH7/CORO6/CAPZA2/ACTN3</t>
+    <t xml:space="preserve">MYL4/TPM2/TTN/MYH13/CD63/H1-4/ACTN3/ACTN4/TNNC1/MYH4/HSPG2/MYH2/COL6A1/ACTN1/ACTN2/COL6A2/TPM3/MYH1/ACTB/TPM1/H3-3A/CAPZA2/MYH7/CORO6/NID1/PLEC/NEB</t>
   </si>
   <si>
     <t xml:space="preserve">15/78</t>
   </si>
   <si>
-    <t xml:space="preserve">ACTN1/MYL6/TNNC2/HSPG2/TTN/MYL2/ACTN4/MYL6B/MYL1/MYL3/NID1/TNNC1/ACTN2/MYL4/ACTN3</t>
+    <t xml:space="preserve">MYL6/MYL4/MYL2/TTN/ACTN3/ACTN4/TNNC1/MYL1/HSPG2/ACTN1/ACTN2/MYL6B/MYL3/TNNC2/NID1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0120544</t>
@@ -4132,7 +4132,7 @@
     <t xml:space="preserve">actinin binding</t>
   </si>
   <si>
-    <t xml:space="preserve">TTN/MYOZ1/PDLIM7/SYNPO2/PDLIM5/MYOT</t>
+    <t xml:space="preserve">MYOT/TTN/MYOZ1/PDLIM7/SYNPO2/PDLIM5</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005200</t>
@@ -4141,7 +4141,7 @@
     <t xml:space="preserve">structural constituent of cytoskeleton</t>
   </si>
   <si>
-    <t xml:space="preserve">TPM1/LMNA/DES/SYNM/ACTB/PLEC/ACTA1/ACTN2/VIM</t>
+    <t xml:space="preserve">DES/ACTA1/SYNM/VIM/ACTN2/LMNA/ACTB/TPM1/PLEC</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0051393</t>
@@ -4153,7 +4153,7 @@
     <t xml:space="preserve">11/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">TTN/PDLIM7/SYNPO2/PDLIM5/MYOT</t>
+    <t xml:space="preserve">MYOT/TTN/PDLIM7/SYNPO2/PDLIM5</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0120543</t>
@@ -4174,7 +4174,7 @@
     <t xml:space="preserve">18/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">MYL2/MYL3/MYBPC1/ACTA1/MYL4</t>
+    <t xml:space="preserve">MYL4/MYL2/MYBPC1/ACTA1/MYL3</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0031490</t>
@@ -4183,10 +4183,10 @@
     <t xml:space="preserve">chromatin DNA binding</t>
   </si>
   <si>
-    <t xml:space="preserve">H1-4/H3-3A/ACTN4/ACTB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ACTN1/HSPG2/ACTN4/ACTN2/ACTN3</t>
+    <t xml:space="preserve">H1-4/ACTN4/ACTB/H3-3A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACTN3/ACTN4/HSPG2/ACTN1/ACTN2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005516</t>
@@ -4198,76 +4198,76 @@
     <t xml:space="preserve">44/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">MYH13/TTN/MYH1/MYH2/MYH4/OBSCN/MYH7</t>
+    <t xml:space="preserve">OBSCN/TTN/MYH13/MYH4/MYH2/MYH1/MYH7</t>
   </si>
   <si>
     <t xml:space="preserve">26/66</t>
   </si>
   <si>
-    <t xml:space="preserve">RACK1/RPL23/RPS8/NACA/RPL38/EIF1/EIF5B/RPSA/RPS11/RPS9/RPS4X/MRPS23/UFL1/EIF3A/RPL5/RPL9/RPL19/MRPL55/LRRC47/PABPC4/RPS6/EIF3B/EIF3I/RPS18/RPL23A/RPS12</t>
+    <t xml:space="preserve">RPS6/NACA/RPS8/EIF5B/PABPC4/RPL38/EIF1/RPSA/LRRC47/MRPL55/RPS4X/EIF3I/RPS9/RPS11/EIF3B/MRPS23/RPL5/EIF3A/RPS12/RPL9/RPL19/RPL23/UFL1/RPS18/RPL23A/RACK1</t>
   </si>
   <si>
     <t xml:space="preserve">19/66</t>
   </si>
   <si>
-    <t xml:space="preserve">RACK1/RPL23/RPS8/RPL38/RPSA/RPS11/RPS9/RPS4X/UFL1/EIF3A/RPL5/RPL9/RPL19/RPS6/EIF3B/EIF3I/RPS18/RPL23A/RPS12</t>
+    <t xml:space="preserve">RPS6/RPS8/RPL38/RPSA/RPS4X/EIF3I/RPS9/RPS11/EIF3B/RPL5/EIF3A/RPS12/RPL9/RPL19/RPL23/UFL1/RPS18/RPL23A/RACK1</t>
   </si>
   <si>
     <t xml:space="preserve">13/66</t>
   </si>
   <si>
-    <t xml:space="preserve">RPS8/EIF5B/RPSA/RPS11/RPS9/RPS4X/SNRPG/EIF3A/RPL5/RPS6/EIF3B/EIF3I/RPS12</t>
+    <t xml:space="preserve">RPS6/RPS8/EIF5B/RPSA/RPS4X/EIF3I/RPS9/RPS11/EIF3B/RPL5/SNRPG/EIF3A/RPS12</t>
   </si>
   <si>
     <t xml:space="preserve">7/66</t>
   </si>
   <si>
-    <t xml:space="preserve">RPS8/RPSA/RPS11/RPS9/RPS4X/RPS6/RPS12</t>
+    <t xml:space="preserve">RPS6/RPS8/RPSA/RPS4X/RPS9/RPS11/RPS12</t>
   </si>
   <si>
     <t xml:space="preserve">9/66</t>
   </si>
   <si>
-    <t xml:space="preserve">RPS8/EIF5B/RPSA/RPS11/RPS9/RPS4X/RPL5/RPS6/RPS12</t>
+    <t xml:space="preserve">RPS6/RPS8/EIF5B/RPSA/RPS4X/RPS9/RPS11/RPL5/RPS12</t>
   </si>
   <si>
     <t xml:space="preserve">23/67</t>
   </si>
   <si>
-    <t xml:space="preserve">RACK1/RPL23/RPS8/RPL38/EIF1/RPSA/RPS11/RPS9/RPS4X/SNRPG/MRPS23/EIF3A/RPL5/RPL9/RPL19/MRPL55/PABPC4/RPS6/EIF3B/EIF3I/RPS18/RPL23A/RPS12</t>
+    <t xml:space="preserve">RPS6/RPS8/PABPC4/RPL38/EIF1/RPSA/MRPL55/RPS4X/EIF3I/RPS9/RPS11/EIF3B/MRPS23/RPL5/SNRPG/EIF3A/RPS12/RPL9/RPL19/RPL23/RPS18/RPL23A/RACK1</t>
   </si>
   <si>
     <t xml:space="preserve">16/67</t>
   </si>
   <si>
-    <t xml:space="preserve">RACK1/RPL23/RPS8/RPL38/RPSA/RPS11/RPS9/RPS4X/RPL5/RPL9/RPL19/MRPL55/RPS6/RPS18/RPL23A/RPS12</t>
+    <t xml:space="preserve">RPS6/RPS8/RPL38/RPSA/MRPL55/RPS4X/RPS9/RPS11/RPL5/RPS12/RPL9/RPL19/RPL23/RPS18/RPL23A/RACK1</t>
   </si>
   <si>
     <t xml:space="preserve">17/67</t>
   </si>
   <si>
-    <t xml:space="preserve">RACK1/RPL23/RPS8/RPL38/RPSA/RPS11/RPS9/RPS4X/MRPS23/RPL5/RPL9/RPL19/MRPL55/RPS6/RPS18/RPL23A/RPS12</t>
+    <t xml:space="preserve">RPS6/RPS8/RPL38/RPSA/MRPL55/RPS4X/RPS9/RPS11/MRPS23/RPL5/RPS12/RPL9/RPL19/RPL23/RPS18/RPL23A/RACK1</t>
   </si>
   <si>
     <t xml:space="preserve">14/67</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL23/RPS8/RPL38/RPSA/RPS11/RPS9/RPS4X/RPL5/RPL9/RPL19/RPS6/RPS18/RPL23A/RPS12</t>
+    <t xml:space="preserve">RPS6/RPS8/RPL38/RPSA/RPS4X/RPS9/RPS11/RPL5/RPS12/RPL9/RPL19/RPL23/RPS18/RPL23A</t>
   </si>
   <si>
     <t xml:space="preserve">9/67</t>
   </si>
   <si>
-    <t xml:space="preserve">RACK1/RPS8/RPSA/RPS11/RPS9/RPS4X/RPS6/RPS18/RPS12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RPL23/RPS8/CAPN3/RPS11/RPS9/RPS4X/UBE2I/H1-0/RPL5/RPL9/RPL19/RPS6/RPL23A/RPS12</t>
+    <t xml:space="preserve">RPS6/RPS8/RPSA/RPS4X/RPS9/RPS11/RPS12/RPS18/RACK1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RPS6/RPS8/CAPN3/UBE2I/RPS4X/RPS9/RPS11/RPL5/RPS12/RPL9/RPL19/RPL23/H1-0/RPL23A</t>
   </si>
   <si>
     <t xml:space="preserve">8/67</t>
   </si>
   <si>
-    <t xml:space="preserve">RPS8/RPSA/RPS11/RPS9/RPS4X/RPS6/RPS18/RPS12</t>
+    <t xml:space="preserve">RPS6/RPS8/RPSA/RPS4X/RPS9/RPS11/RPS12/RPS18</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0016010</t>
@@ -4279,7 +4279,7 @@
     <t xml:space="preserve">5/67</t>
   </si>
   <si>
-    <t xml:space="preserve">PGM5/SGCB/SGCD/UTRN/SNTB1</t>
+    <t xml:space="preserve">SGCB/SGCD/PGM5/SNTB1/UTRN</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0090665</t>
@@ -4291,25 +4291,25 @@
     <t xml:space="preserve">18/67</t>
   </si>
   <si>
-    <t xml:space="preserve">PGM5/RPL23/RPS8/NEXN/RPL38/ARPC5L/RPS11/RPS9/RPS4X/CLASP2/CHP1/SNTB1/RPL5/RPL9/RPL19/TNS1/RPS18/RRAS2</t>
+    <t xml:space="preserve">RPS8/CLASP2/RPL38/NEXN/RPS4X/PGM5/RRAS2/RPS9/RPS11/TNS1/SNTB1/RPL5/CHP1/RPL9/RPL19/RPL23/RPS18/ARPC5L</t>
   </si>
   <si>
     <t xml:space="preserve">6/67</t>
   </si>
   <si>
-    <t xml:space="preserve">RPS8/RPS11/RPS9/RPS4X/RPS6/RPS12</t>
+    <t xml:space="preserve">RPS6/RPS8/RPS4X/RPS9/RPS11/RPS12</t>
   </si>
   <si>
     <t xml:space="preserve">30/67</t>
   </si>
   <si>
-    <t xml:space="preserve">PGM5/RPL23/RPS8/NEXN/RPL38/SGCB/ARPC5L/SGCD/EIF5B/RPS11/RPS9/VAPA/RPS4X/AP2A1/UBE2I/CLASP2/UTRN/CHP1/EIF3A/SNTB1/RPL5/ATP1A3/RPL9/RPL19/RPS6/EIF3B/TNS1/EIF3I/RPS18/RRAS2</t>
+    <t xml:space="preserve">RPS6/RPS8/CLASP2/EIF5B/SGCB/RPL38/SGCD/UBE2I/NEXN/RPS4X/PGM5/RRAS2/EIF3I/RPS9/RPS11/EIF3B/TNS1/SNTB1/AP2A1/RPL5/ATP1A3/CHP1/EIF3A/VAPA/UTRN/RPL9/RPL19/RPL23/RPS18/ARPC5L</t>
   </si>
   <si>
     <t xml:space="preserve">19/67</t>
   </si>
   <si>
-    <t xml:space="preserve">PGM5/RPL23/RPS8/NEXN/RPL38/ARPC5L/RPS11/RPS9/VAPA/RPS4X/CLASP2/CHP1/SNTB1/RPL5/RPL9/RPL19/TNS1/RPS18/RRAS2</t>
+    <t xml:space="preserve">RPS8/CLASP2/RPL38/NEXN/RPS4X/PGM5/RRAS2/RPS9/RPS11/TNS1/SNTB1/RPL5/CHP1/VAPA/RPL9/RPL19/RPL23/RPS18/ARPC5L</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0016282</t>
@@ -4321,7 +4321,7 @@
     <t xml:space="preserve">4/67</t>
   </si>
   <si>
-    <t xml:space="preserve">EIF1/EIF3A/EIF3B/EIF3I</t>
+    <t xml:space="preserve">EIF1/EIF3I/EIF3B/EIF3A</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0033290</t>
@@ -4342,10 +4342,10 @@
     <t xml:space="preserve">plasma membrane protein complex</t>
   </si>
   <si>
-    <t xml:space="preserve">PGM5/SGCB/SGCD/RYR1/AP2A1/UTRN/SNTB1/ATP1A3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RPL23/RPL38/RPL5/RPL9/RPL19/RPL23A</t>
+    <t xml:space="preserve">SGCB/SGCD/RYR1/PGM5/SNTB1/AP2A1/ATP1A3/UTRN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RPL38/RPL5/RPL9/RPL19/RPL23/RPL23A</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0042383</t>
@@ -4357,31 +4357,31 @@
     <t xml:space="preserve">58/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">PGM5/CAPN3/SGCB/SGCD/RYR1/UTRN/MLIP/SNTB1</t>
+    <t xml:space="preserve">CAPN3/SGCB/SGCD/RYR1/PGM5/MLIP/SNTB1/UTRN</t>
   </si>
   <si>
     <t xml:space="preserve">7/67</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL23/RPL38/RPL5/RPL9/RPL19/MRPL55/RPL23A</t>
+    <t xml:space="preserve">RPL38/MRPL55/RPL5/RPL9/RPL19/RPL23/RPL23A</t>
   </si>
   <si>
     <t xml:space="preserve">20/67</t>
   </si>
   <si>
-    <t xml:space="preserve">MGST3/EPHX1/RPS8/TMED1/RPL38/SGCB/SGCD/RYR1/VAPA/OSTC/KLHL41/UFL1/CHP1/LRPAP1/RPL5/ATP1A3/RPL9/RPS6/ERP29/RRAS2</t>
+    <t xml:space="preserve">RPS6/RPS8/TMED1/SGCB/RPL38/SGCD/RYR1/RRAS2/ERP29/RPL5/LRPAP1/ATP1A3/OSTC/CHP1/EPHX1/VAPA/MGST3/RPL9/KLHL41/UFL1</t>
   </si>
   <si>
     <t xml:space="preserve">16/68</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL23/RPS8/RPL38/RPSA/RPS11/RPS9/RPS4X/MRPS23/RPL5/RPL9/RPL19/MRPL55/RPS6/RPS18/RPL23A/RPS12</t>
+    <t xml:space="preserve">RPS6/RPS8/RPL38/RPSA/MRPL55/RPS4X/RPS9/RPS11/MRPS23/RPL5/RPS12/RPL9/RPL19/RPL23/RPS18/RPL23A</t>
   </si>
   <si>
     <t xml:space="preserve">23/68</t>
   </si>
   <si>
-    <t xml:space="preserve">PGM5/RPL23/RPS8/CAPN3/NEXN/RPL38/RPSA/RPS11/RPS9/RPS4X/MRPS23/H1-0/EIF3A/SNTB1/RPL5/RPL9/RPL19/MRPL55/MYH8/RPS6/RPS18/RPL23A/RPS12</t>
+    <t xml:space="preserve">RPS6/RPS8/CAPN3/RPL38/RPSA/MRPL55/NEXN/RPS4X/PGM5/RPS9/RPS11/SNTB1/MRPS23/RPL5/EIF3A/RPS12/RPL9/RPL19/MYH8/RPL23/H1-0/RPS18/RPL23A</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0019843</t>
@@ -4393,19 +4393,19 @@
     <t xml:space="preserve">8/68</t>
   </si>
   <si>
-    <t xml:space="preserve">RPL23/RPS11/RPS9/RPS4X/RPL5/RPL9/RPS18/RPL23A</t>
+    <t xml:space="preserve">RPS4X/RPS9/RPS11/RPL5/RPL9/RPL23/RPS18/RPL23A</t>
   </si>
   <si>
     <t xml:space="preserve">31/68</t>
   </si>
   <si>
-    <t xml:space="preserve">RACK1/RPL23/RPS8/RPL38/EIF1/FAM98A/EIF5B/RPSA/RPS11/RPS9/CLUH/RPS4X/SNRPG/MRPS23/UBE2I/H1-0/SFPQ/EIF3A/APOBEC2/RPL5/RPL9/RPL19/LRRC47/PABPC4/RPS6/EIF3B/TNS1/EIF3I/RPS18/RPL23A/RPS12</t>
+    <t xml:space="preserve">RPS6/RPS8/EIF5B/PABPC4/RPL38/FAM98A/EIF1/RPSA/LRRC47/UBE2I/RPS4X/EIF3I/RPS9/RPS11/EIF3B/TNS1/APOBEC2/MRPS23/RPL5/SNRPG/EIF3A/CLUH/RPS12/SFPQ/RPL9/RPL19/RPL23/H1-0/RPS18/RPL23A/RACK1</t>
   </si>
   <si>
     <t xml:space="preserve">33/68</t>
   </si>
   <si>
-    <t xml:space="preserve">RACK1/RPL23/RPS8/NACA/RPL38/PDCD5/EIF1/FAM98A/EIF5B/RPSA/RPS11/RPS9/CLUH/RPS4X/SNRPG/MRPS23/UBE2I/H1-0/SFPQ/EIF3A/APOBEC2/RPL5/RPL9/RPL19/LRRC47/PABPC4/RPS6/EIF3B/TNS1/EIF3I/RPS18/RPL23A/RPS12</t>
+    <t xml:space="preserve">RPS6/NACA/RPS8/EIF5B/PABPC4/RPL38/PDCD5/FAM98A/EIF1/RPSA/LRRC47/UBE2I/RPS4X/EIF3I/RPS9/RPS11/EIF3B/TNS1/APOBEC2/MRPS23/RPL5/SNRPG/EIF3A/CLUH/RPS12/SFPQ/RPL9/RPL19/RPL23/H1-0/RPS18/RPL23A/RACK1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0019646</t>
@@ -4420,7 +4420,7 @@
     <t xml:space="preserve">58/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/COX7C/NDUFB3/NDUFB1/NDUFS2/COX7A1/NDUFA8/NDUFS3/NDUFAB1/NDUFV2/NDUFS1/UQCRB/NDUFC2/COX7A2/NDUFB6/NDUFV1/MT-ND5/NDUFA10/COX6C/UQCRFS1/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/COX7C/MT-ND5/NDUFV1/NDUFS2/SDHB/UQCRFS1/COX7A1/NDUFS3/NDUFA8/NDUFV2/NDUFS1/UQCRB/COX7A2/NDUFB6/NDUFAB1/COX6C/NDUFC2/NDUFA10/NDUFS4</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0022900</t>
@@ -4432,7 +4432,7 @@
     <t xml:space="preserve">26/57</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/COX7C/NDUFB3/NDUFB1/NDUFS2/COX7A1/NDUFA8/NDUFS3/NDUFAB1/NDUFV2/NDUFS1/UQCRB/NDUFC2/COX7A2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/COX6C/UQCRFS1/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/COX7C/NDUFA13/MT-ND5/NDUFV1/NDUFS2/SDHB/UQCRFS1/COX7A1/NDUFS3/NDUFA8/NDUFV2/NDUFS1/UQCRB/COX7A2/NDUFB6/NDUFAB1/COX6C/NDUFC2/NDUFA10/NDUFS4</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0022904</t>
@@ -4468,7 +4468,7 @@
     <t xml:space="preserve">82/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/COX7C/NDUFB3/NDUFB1/NDUFS2/COX7A1/NDUFA8/NDUFS3/NDUFAB1/NDUFV2/NDUFS1/ATP5PD/UQCRB/NDUFC2/COX7A2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/COX6C/UQCRFS1/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/COX7C/NDUFA13/MT-ND5/NDUFV1/NDUFS2/SDHB/UQCRFS1/COX7A1/NDUFS3/NDUFA8/NDUFV2/NDUFS1/UQCRB/COX7A2/NDUFB6/NDUFAB1/COX6C/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0015986</t>
@@ -4480,7 +4480,7 @@
     <t xml:space="preserve">21/57</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/NDUFA8/NDUFS3/NDUFAB1/NDUFV2/NDUFS1/ATP5PD/NDUFC2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/NDUFA13/MT-ND5/NDUFV1/NDUFS2/SDHB/NDUFS3/NDUFA8/NDUFV2/NDUFS1/NDUFB6/NDUFAB1/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0042776</t>
@@ -4501,7 +4501,7 @@
     <t xml:space="preserve">36/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/NDUFA8/NDUFS3/NDUFAB1/NDUFV2/NDUFS1/NDUFC2/NDUFB6/NDUFV1/MT-ND5/NDUFA10</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/MT-ND5/NDUFV1/NDUFS2/NDUFS3/NDUFA8/NDUFV2/NDUFS1/NDUFB6/NDUFAB1/NDUFC2/NDUFA10/NDUFS4</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006754</t>
@@ -4549,7 +4549,7 @@
     <t xml:space="preserve">22/57</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/COX7A1/NDUFA8/NDUFS3/NDUFV2/NDUFS1/ATP5PD/ATP1B1/NDUFC2/NDUFB6/NDUFV1/MT-ND5/NDUFA10/SLC25A12/UQCRFS1</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/MT-ND5/NDUFV1/NDUFS2/UQCRFS1/COX7A1/NDUFS3/NDUFA8/ATP1B1/SLC25A12/NDUFV2/NDUFS1/NDUFB6/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0009152</t>
@@ -4558,7 +4558,7 @@
     <t xml:space="preserve">purine ribonucleotide biosynthetic process</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/NDUFA8/NDUFS3/AK2/NDUFAB1/NDUFV2/NDUFS1/ATP5PD/NDUFC2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/AK2/NDUFB1/NDUFS5/NDUFA13/MT-ND5/NDUFV1/NDUFS2/SDHB/NDUFS3/NDUFA8/NDUFV2/NDUFS1/NDUFB6/NDUFAB1/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0009260</t>
@@ -4618,7 +4618,7 @@
     <t xml:space="preserve">23/57</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/NDUFA8/NDUFS3/AK2/NDUFAB1/NDUFV2/NDUFS1/ATP5PD/ATP1B1/NDUFC2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/AK2/NDUFB1/NDUFS5/NDUFA13/MT-ND5/NDUFV1/NDUFS2/SDHB/NDUFS3/NDUFA8/ATP1B1/NDUFV2/NDUFS1/NDUFB6/NDUFAB1/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0009144</t>
@@ -4687,7 +4687,7 @@
     <t xml:space="preserve">11/57</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS8/NDUFS5/NDUFS4/NDUFS2/NDUFS3/NDUFS1/TIMM21/NDUFC2/NDUFA13/MT-ND5/NDUFAF4</t>
+    <t xml:space="preserve">NDUFS8/NDUFS5/NDUFA13/MT-ND5/NDUFS2/TIMM21/NDUFS3/NDUFS1/NDUFAF4/NDUFC2/NDUFS4</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0032981</t>
@@ -4723,7 +4723,7 @@
     <t xml:space="preserve">163/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/NDUFA8/NDUFS3/AK2/NDUFAB1/NDUFV2/NDUFS1/ATP5PD/ATP1B1/NDUFC2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/NAXE/SLC25A12/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/AK2/NDUFB1/NDUFS5/NDUFA13/MT-ND5/NDUFV1/NAXE/NDUFS2/SDHB/NDUFS3/NDUFA8/ATP1B1/SLC25A12/NDUFV2/NDUFS1/NDUFB6/NDUFAB1/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006163</t>
@@ -4738,7 +4738,7 @@
     <t xml:space="preserve">152/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/NDUFA8/NDUFS3/AK2/NDUFAB1/NDUFV2/NDUFS1/ATP5PD/ATP1B1/NDUFC2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/SLC25A12/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/AK2/NDUFB1/NDUFS5/NDUFA13/MT-ND5/NDUFV1/NDUFS2/SDHB/NDUFS3/NDUFA8/ATP1B1/SLC25A12/NDUFV2/NDUFS1/NDUFB6/NDUFAB1/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0033108</t>
@@ -4750,7 +4750,7 @@
     <t xml:space="preserve">13/57</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS8/NDUFS5/NDUFS4/NDUFS2/COX7A1/NDUFS3/NDUFS1/TIMM21/NDUFC2/NDUFA13/MT-ND5/NDUFAF4/UQCRFS1</t>
+    <t xml:space="preserve">NDUFS8/NDUFS5/NDUFA13/MT-ND5/NDUFS2/UQCRFS1/COX7A1/TIMM21/NDUFS3/NDUFS1/NDUFAF4/NDUFC2/NDUFS4</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0007005</t>
@@ -4762,7 +4762,7 @@
     <t xml:space="preserve">20/57</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS8/NDUFS5/NDUFS4/NDUFS2/CAMK2A/COX7A1/NDUFS3/RALA/NDUFS1/TIMM21/PHB2/CHCHD10/NDUFC2/IMMT/NDUFA13/MT-ND5/APOOL/CHCHD3/NDUFAF4/UQCRFS1</t>
+    <t xml:space="preserve">NDUFS8/NDUFS5/NDUFA13/MT-ND5/NDUFS2/CHCHD3/UQCRFS1/APOOL/COX7A1/TIMM21/CAMK2A/NDUFS3/PHB2/IMMT/NDUFS1/RALA/CHCHD10/NDUFAF4/NDUFC2/NDUFS4</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0034220</t>
@@ -4774,7 +4774,7 @@
     <t xml:space="preserve">148/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/COX7A1/NDUFA8/NDUFS3/NDUFV2/NDUFS1/ATP5PD/ATP1B1/NDUFC2/NDUFB6/NDUFV1/MT-ND5/NDUFA10/VDAC3/SLC25A12/UQCRFS1</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/MT-ND5/NDUFV1/NDUFS2/UQCRFS1/VDAC3/COX7A1/NDUFS3/NDUFA8/ATP1B1/SLC25A12/NDUFV2/NDUFS1/NDUFB6/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0098655</t>
@@ -4792,7 +4792,7 @@
     <t xml:space="preserve">monoatomic ion transport</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/CAMK2A/COX7A1/NDUFA8/NDUFS3/NDUFV2/NDUFS1/ATP5PD/ATP1B1/NDUFC2/NDUFB6/NDUFV1/MT-ND5/NDUFA10/VDAC3/SLC25A12/UQCRFS1</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/MT-ND5/NDUFV1/NDUFS2/UQCRFS1/VDAC3/COX7A1/CAMK2A/NDUFS3/NDUFA8/ATP1B1/SLC25A12/NDUFV2/NDUFS1/NDUFB6/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006812</t>
@@ -4804,7 +4804,7 @@
     <t xml:space="preserve">162/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/CAMK2A/COX7A1/NDUFA8/NDUFS3/NDUFV2/NDUFS1/ATP5PD/ATP1B1/NDUFC2/NDUFB6/NDUFV1/MT-ND5/NDUFA10/SLC25A12/UQCRFS1</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/MT-ND5/NDUFV1/NDUFS2/UQCRFS1/COX7A1/CAMK2A/NDUFS3/NDUFA8/ATP1B1/SLC25A12/NDUFV2/NDUFS1/NDUFB6/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0090407</t>
@@ -4825,7 +4825,7 @@
     <t xml:space="preserve">190/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/COX7A1/NDUFA8/NDUFS3/NDUFV2/NDUFS1/ATP5PD/TIMM21/ATP1B1/NDUFC2/NDUFB6/NDUFV1/MT-ND5/NDUFA10/VDAC3/SLC25A12/UQCRFS1</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/MT-ND5/NDUFV1/NDUFS2/UQCRFS1/VDAC3/COX7A1/TIMM21/NDUFS3/NDUFA8/ATP1B1/SLC25A12/NDUFV2/NDUFS1/NDUFB6/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0072521</t>
@@ -4861,7 +4861,7 @@
     <t xml:space="preserve">251/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/ABHD16A/NDUFA8/NDUFS3/AK2/NDUFAB1/NDUFV2/NDUFS1/ATP5PD/PHB2/ATP1B1/NDUFC2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/NAXE/SLC25A12/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/AK2/NDUFB1/NDUFS5/NDUFA13/MT-ND5/NDUFV1/NAXE/NDUFS2/SDHB/ABHD16A/NDUFS3/NDUFA8/ATP1B1/PHB2/SLC25A12/NDUFV2/NDUFS1/NDUFB6/NDUFAB1/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:1901135</t>
@@ -4885,7 +4885,7 @@
     <t xml:space="preserve">317/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/CDC37/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/ABHD16A/NDUFA8/NDUFS3/AK2/NDUFAB1/NDUFV2/NDUFS1/ATP5PD/PHB2/ATP1B1/NDUFC2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/NAXE/SLC25A12/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/AK2/NDUFB1/NDUFS5/NDUFA13/MT-ND5/NDUFV1/NAXE/NDUFS2/SDHB/ABHD16A/NDUFS3/NDUFA8/ATP1B1/PHB2/SLC25A12/NDUFV2/NDUFS1/NDUFB6/NDUFAB1/CDC37/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006796</t>
@@ -4894,7 +4894,7 @@
     <t xml:space="preserve">phosphate-containing compound metabolic process</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/NDUFA8/NDUFS3/AK2/MGST2/NDUFAB1/NDUFV2/NDUFS1/ATP5PD/FAHD2A/ATP1B1/ECHDC3/NDUFC2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/NAXE/SLC25A12/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/AK2/MGST2/NDUFB1/NDUFS5/NDUFA13/MT-ND5/NDUFV1/NAXE/NDUFS2/SDHB/NDUFS3/NDUFA8/ATP1B1/SLC25A12/NDUFV2/NDUFS1/FAHD2A/ECHDC3/NDUFB6/NDUFAB1/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006123</t>
@@ -4909,7 +4909,7 @@
     <t xml:space="preserve">COX7C/COX7A1/COX7A2/COX6C</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/NDUFA8/ZBTB9/NDUFS3/AK2/NDUFAB1/NDUFV2/NDUFS1/ATP5PD/FHOD1/PHB2/NDUFC2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/AK2/NDUFB1/NDUFS5/NDUFA13/MT-ND5/NDUFV1/NDUFS2/SDHB/FHOD1/NDUFS3/NDUFA8/ZBTB9/PHB2/NDUFV2/NDUFS1/NDUFB6/NDUFAB1/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0007007</t>
@@ -4921,7 +4921,7 @@
     <t xml:space="preserve">5/57</t>
   </si>
   <si>
-    <t xml:space="preserve">CHCHD10/IMMT/NDUFA13/APOOL/CHCHD3</t>
+    <t xml:space="preserve">NDUFA13/CHCHD3/APOOL/IMMT/CHCHD10</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006810</t>
@@ -4933,7 +4933,7 @@
     <t xml:space="preserve">481/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/CAMK2A/COX7A1/NDUFA8/NDUFS3/NDUFV2/RALA/NDUFS1/ATP5PD/TIMM21/PHB2/ATP1B1/NDUFC2/NDUFB6/NDUFV1/MT-ND5/NDUFA10/VDAC3/NAXE/SLC25A12/UQCRFS1</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/MT-ND5/NDUFV1/NAXE/NDUFS2/UQCRFS1/VDAC3/COX7A1/TIMM21/CAMK2A/NDUFS3/NDUFA8/ATP1B1/PHB2/SLC25A12/NDUFV2/NDUFS1/RALA/NDUFB6/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0007006</t>
@@ -4954,7 +4954,7 @@
     <t xml:space="preserve">174/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/COX7C/NDUFB3/NDUFB1/NDUFS2/BDH1/COX7A1/NDUFA8/NDUFS3/MRPS22/NDUFAB1/NDUFV2/NDUFS1/ATP5PD/TIMM21/UQCRB/PHB2/MRPL22/CHCHD10/NDUFC2/IMMT/COX7A2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/APOOL/CHCHD3/SLC25A12/NDUFAF4/COX6C/UQCRFS1/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/MRPS22/NDUFB1/NDUFS5/COX7C/NDUFA13/MT-ND5/NDUFV1/NDUFS2/CHCHD3/SDHB/UQCRFS1/APOOL/COX7A1/TIMM21/NDUFS3/NDUFA8/PHB2/SLC25A12/IMMT/NDUFV2/NDUFS1/UQCRB/BDH1/CHCHD10/COX7A2/NDUFB6/NDUFAB1/NDUFAF4/COX6C/NDUFC2/MRPL22/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0019866</t>
@@ -4984,7 +4984,7 @@
     <t xml:space="preserve">246/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/COX7C/NDUFB3/NDUFB1/NDUFS2/BDH1/COX7A1/NDUFA8/NDUFS3/AK2/MRPS22/NDUFAB1/NDUFV2/NDUFS1/ATP5PD/TIMM21/UQCRB/PHB2/MRPL22/CHCHD10/NDUFC2/IMMT/COX7A2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/APOOL/VDAC3/CHCHD3/SLC25A12/NDUFAF4/COX6C/UQCRFS1/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/MRPS22/AK2/NDUFB1/NDUFS5/COX7C/NDUFA13/MT-ND5/NDUFV1/NDUFS2/CHCHD3/SDHB/UQCRFS1/VDAC3/APOOL/COX7A1/TIMM21/NDUFS3/NDUFA8/PHB2/SLC25A12/IMMT/NDUFV2/NDUFS1/UQCRB/BDH1/CHCHD10/COX7A2/NDUFB6/NDUFAB1/NDUFAF4/COX6C/NDUFC2/MRPL22/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0031966</t>
@@ -4999,7 +4999,7 @@
     <t xml:space="preserve">231/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/COX7C/NDUFB3/NDUFB1/NDUFS2/BDH1/COX7A1/NDUFA8/NDUFS3/MRPS22/NDUFAB1/NDUFV2/NDUFS1/ATP5PD/TIMM21/UQCRB/PHB2/MRPL22/CHCHD10/NDUFC2/IMMT/COX7A2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/APOOL/VDAC3/CHCHD3/SLC25A12/NDUFAF4/COX6C/UQCRFS1/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/MRPS22/NDUFB1/NDUFS5/COX7C/NDUFA13/MT-ND5/NDUFV1/NDUFS2/CHCHD3/SDHB/UQCRFS1/VDAC3/APOOL/COX7A1/TIMM21/NDUFS3/NDUFA8/PHB2/SLC25A12/IMMT/NDUFV2/NDUFS1/UQCRB/BDH1/CHCHD10/COX7A2/NDUFB6/NDUFAB1/NDUFAF4/COX6C/NDUFC2/MRPL22/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030964</t>
@@ -5014,7 +5014,7 @@
     <t xml:space="preserve">37/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/NDUFA8/NDUFS3/NDUFAB1/NDUFV2/NDUFS1/NDUFC2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/NDUFA13/MT-ND5/NDUFV1/NDUFS2/NDUFS3/NDUFA8/NDUFV2/NDUFS1/NDUFB6/NDUFAB1/NDUFC2/NDUFA10/NDUFS4</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0045271</t>
@@ -5035,7 +5035,7 @@
     <t xml:space="preserve">293/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/COX7C/NDUFB3/NDUFB1/NDUFS2/BDH1/COX7A1/NDUFA8/NDUFS3/AK2/MGST2/MRPS22/NDUFAB1/NDUFV2/NDUFS1/ATP5PD/TIMM21/UQCRB/PHB2/MRPL22/CHCHD10/NDUFC2/IMMT/COX7A2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/APOOL/VDAC3/CHCHD3/SLC25A12/NDUFAF4/COX6C/UQCRFS1/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/MRPS22/AK2/MGST2/NDUFB1/NDUFS5/COX7C/NDUFA13/MT-ND5/NDUFV1/NDUFS2/CHCHD3/SDHB/UQCRFS1/VDAC3/APOOL/COX7A1/TIMM21/NDUFS3/NDUFA8/PHB2/SLC25A12/IMMT/NDUFV2/NDUFS1/UQCRB/BDH1/CHCHD10/COX7A2/NDUFB6/NDUFAB1/NDUFAF4/COX6C/NDUFC2/MRPL22/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:1902495</t>
@@ -5047,7 +5047,7 @@
     <t xml:space="preserve">99/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/COX7C/NDUFB3/NDUFB1/NDUFS2/COX7A1/NDUFA8/NDUFS3/NDUFAB1/NDUFV2/NDUFS1/ATP5PD/UQCRB/ATP1B1/NDUFC2/COX7A2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/COX6C/UQCRFS1</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/COX7C/NDUFA13/MT-ND5/NDUFV1/NDUFS2/UQCRFS1/COX7A1/NDUFS3/NDUFA8/ATP1B1/NDUFV2/NDUFS1/UQCRB/COX7A2/NDUFB6/NDUFAB1/COX6C/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:1990351</t>
@@ -5071,7 +5071,7 @@
     <t xml:space="preserve">211/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/COX7C/NDUFB3/NDUFB1/NDUFS2/COX7A1/NDUFA8/NDUFS3/NDUFAB1/NDUFV2/NDUFS1/ATP5PD/TIMM21/UQCRB/PHB2/ATP1B1/CHCHD10/NDUFC2/IMMT/COX7A2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/APOOL/VDAC3/CHCHD3/COX6C/UQCRFS1/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/COX7C/NDUFA13/MT-ND5/NDUFV1/NDUFS2/CHCHD3/SDHB/UQCRFS1/VDAC3/APOOL/COX7A1/TIMM21/NDUFS3/NDUFA8/ATP1B1/PHB2/IMMT/NDUFV2/NDUFS1/UQCRB/CHCHD10/COX7A2/NDUFB6/NDUFAB1/COX6C/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005739</t>
@@ -5086,7 +5086,7 @@
     <t xml:space="preserve">490/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/HSPE1/NDUFS5/NDUFS4/CLYBL/COX7C/NDUFB3/NDUFB1/NDUFS2/BDH1/CAMK2A/COX7A1/NDUFA8/NDUFS3/AK2/MRPS22/NDUFAB1/NDUFV2/RALA/NDUFS1/ATP5PD/TIMM21/UQCRB/FAHD2A/PHB2/MRPL22/CHCHD10/ECHDC3/NDUFC2/IMMT/COX7A2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/LACTB/NDUFA10/APOOL/VDAC3/NAXE/CHCHD3/SLC25A12/NDUFAF4/COX6C/UQCRFS1/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/MRPS22/AK2/NDUFB1/NDUFS5/COX7C/NDUFA13/MT-ND5/NDUFV1/NAXE/NDUFS2/CHCHD3/SDHB/UQCRFS1/VDAC3/APOOL/COX7A1/TIMM21/CAMK2A/NDUFS3/NDUFA8/PHB2/SLC25A12/IMMT/NDUFV2/NDUFS1/RALA/FAHD2A/UQCRB/BDH1/ECHDC3/CHCHD10/COX7A2/NDUFB6/NDUFAB1/NDUFAF4/COX6C/NDUFC2/MRPL22/NDUFA10/LACTB/CLYBL/NDUFS4/HSPE1/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:1990204</t>
@@ -5095,7 +5095,7 @@
     <t xml:space="preserve">oxidoreductase complex</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/NDUFA8/NDUFS3/NDUFAB1/NDUFV2/NDUFS1/NDUFC2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/NDUFA13/MT-ND5/NDUFV1/NDUFS2/SDHB/NDUFS3/NDUFA8/NDUFV2/NDUFS1/NDUFB6/NDUFAB1/NDUFC2/NDUFA10/NDUFS4</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0031090</t>
@@ -5110,7 +5110,7 @@
     <t xml:space="preserve">496/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/COX7C/NDUFB3/NDUFB1/NDUFS2/BDH1/CAMK2A/COX7A1/NDUFA8/NDUFS3/MGST2/MRPS22/NDUFAB1/NDUFV2/RALA/NDUFS1/ATP5PD/TIMM21/UQCRB/PHB2/ATP1B1/MRPL22/CHCHD10/NDUFC2/IMMT/COX7A2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/APOOL/VDAC3/CHCHD3/SLC25A12/NDUFAF4/COX6C/UQCRFS1/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/MRPS22/MGST2/NDUFB1/NDUFS5/COX7C/NDUFA13/MT-ND5/NDUFV1/NDUFS2/CHCHD3/SDHB/UQCRFS1/VDAC3/APOOL/COX7A1/TIMM21/CAMK2A/NDUFS3/NDUFA8/ATP1B1/PHB2/SLC25A12/IMMT/NDUFV2/NDUFS1/RALA/UQCRB/BDH1/CHCHD10/COX7A2/NDUFB6/NDUFAB1/NDUFAF4/COX6C/NDUFC2/MRPL22/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:1902494</t>
@@ -5122,7 +5122,7 @@
     <t xml:space="preserve">305/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/COX7C/NDUFB3/NDUFB1/NDUFS2/CAMK2A/COX7A1/NDUFA8/NDUFS3/NDUFAB1/NDUFV2/NDUFS1/ATP5PD/UQCRB/NDUFC2/COX7A2/NDUFB6/NDUFV1/NDUFA13/MT-ND5/NDUFA10/COX6C/UQCRFS1/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/COX7C/NDUFA13/MT-ND5/NDUFV1/NDUFS2/SDHB/UQCRFS1/COX7A1/CAMK2A/NDUFS3/NDUFA8/NDUFV2/NDUFS1/UQCRB/COX7A2/NDUFB6/NDUFAB1/COX6C/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005758</t>
@@ -5134,7 +5134,7 @@
     <t xml:space="preserve">9/57</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS5/NDUFA8/AK2/NDUFS1/TIMM21/CHCHD10/IMMT/COX6C</t>
+    <t xml:space="preserve">NDUFB7/AK2/NDUFS5/TIMM21/NDUFA8/IMMT/NDUFS1/CHCHD10/COX6C</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0031970</t>
@@ -5152,7 +5152,7 @@
     <t xml:space="preserve">6/57</t>
   </si>
   <si>
-    <t xml:space="preserve">TIMM21/PHB2/CHCHD10/IMMT/APOOL/CHCHD3</t>
+    <t xml:space="preserve">CHCHD3/APOOL/TIMM21/PHB2/IMMT/CHCHD10</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0070069</t>
@@ -5161,7 +5161,7 @@
     <t xml:space="preserve">cytochrome complex</t>
   </si>
   <si>
-    <t xml:space="preserve">COX7C/COX7A1/UQCRB/COX7A2/COX6C/UQCRFS1</t>
+    <t xml:space="preserve">COX7C/UQCRFS1/COX7A1/UQCRB/COX7A2/COX6C</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0098798</t>
@@ -5173,7 +5173,7 @@
     <t xml:space="preserve">53/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">MRPS22/NDUFAB1/TIMM21/PHB2/MRPL22/CHCHD10/IMMT/APOOL/CHCHD3</t>
+    <t xml:space="preserve">MRPS22/CHCHD3/APOOL/TIMM21/PHB2/IMMT/CHCHD10/NDUFAB1/MRPL22</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005742</t>
@@ -5185,7 +5185,7 @@
     <t xml:space="preserve">3/57</t>
   </si>
   <si>
-    <t xml:space="preserve">IMMT/APOOL/CHCHD3</t>
+    <t xml:space="preserve">CHCHD3/APOOL/IMMT</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0098799</t>
@@ -5206,7 +5206,7 @@
     <t xml:space="preserve">34/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/NDUFA8/NDUFS3/NDUFV2/NDUFS1/NDUFC2/NDUFB6/NDUFV1/MT-ND5/NDUFA10</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/MT-ND5/NDUFV1/NDUFS2/NDUFS3/NDUFA8/NDUFV2/NDUFS1/NDUFB6/NDUFC2/NDUFA10/NDUFS4</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0015453</t>
@@ -5221,7 +5221,7 @@
     <t xml:space="preserve">47/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/COX7A1/NDUFA8/NDUFS3/NDUFV2/NDUFS1/NDUFC2/NDUFB6/NDUFV1/MT-ND5/NDUFA10/UQCRFS1</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/MT-ND5/NDUFV1/NDUFS2/UQCRFS1/COX7A1/NDUFS3/NDUFA8/NDUFV2/NDUFS1/NDUFB6/NDUFC2/NDUFA10/NDUFS4</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0015399</t>
@@ -5236,7 +5236,7 @@
     <t xml:space="preserve">58/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/COX7A1/NDUFA8/NDUFS3/NDUFV2/NDUFS1/ATP1B1/NDUFC2/NDUFB6/NDUFV1/MT-ND5/NDUFA10/UQCRFS1</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/MT-ND5/NDUFV1/NDUFS2/UQCRFS1/COX7A1/NDUFS3/NDUFA8/ATP1B1/NDUFV2/NDUFS1/NDUFB6/NDUFC2/NDUFA10/NDUFS4</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0022853</t>
@@ -5257,7 +5257,7 @@
     <t xml:space="preserve">72/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/COX7A1/NDUFA8/NDUFS3/NDUFV2/NDUFS1/ATP1B1/NDUFC2/NDUFB6/NDUFV1/MT-ND5/NDUFA10/SLC25A12/UQCRFS1</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/MT-ND5/NDUFV1/NDUFS2/UQCRFS1/COX7A1/NDUFS3/NDUFA8/ATP1B1/SLC25A12/NDUFV2/NDUFS1/NDUFB6/NDUFC2/NDUFA10/NDUFS4</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0015078</t>
@@ -5266,7 +5266,7 @@
     <t xml:space="preserve">proton transmembrane transporter activity</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/COX7A1/NDUFA8/NDUFS3/NDUFV2/NDUFS1/ATP5PD/NDUFC2/NDUFB6/NDUFV1/MT-ND5/NDUFA10/SLC25A12/UQCRFS1</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/MT-ND5/NDUFV1/NDUFS2/UQCRFS1/COX7A1/NDUFS3/NDUFA8/SLC25A12/NDUFV2/NDUFS1/NDUFB6/NDUFC2/NDUFA10/NDUFS4/ATP5PD</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0009055</t>
@@ -5275,7 +5275,7 @@
     <t xml:space="preserve">electron transfer activity</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFB7/NDUFS8/NDUFB5/NDUFS5/NDUFS4/NDUFB3/NDUFB1/NDUFS2/COX7A1/NDUFA8/NDUFS3/NDUFV2/NDUFS1/NDUFC2/NDUFB6/NDUFV1/MT-ND5/NDUFA10/UQCRFS1/SDHB</t>
+    <t xml:space="preserve">NDUFB7/NDUFB5/NDUFB3/NDUFS8/NDUFB1/NDUFS5/MT-ND5/NDUFV1/NDUFS2/SDHB/UQCRFS1/COX7A1/NDUFS3/NDUFA8/NDUFV2/NDUFS1/NDUFB6/NDUFC2/NDUFA10/NDUFS4</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0008324</t>
@@ -5329,7 +5329,7 @@
     <t xml:space="preserve">7/56</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS8/NDUFS2/NDUFV2/NDUFS1/NDUFV1/UQCRFS1/SDHB</t>
+    <t xml:space="preserve">NDUFS8/NDUFV1/NDUFS2/SDHB/UQCRFS1/NDUFV2/NDUFS1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0051540</t>
@@ -5350,7 +5350,7 @@
     <t xml:space="preserve">13/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS8/NDUFS2/NDUFS1/NDUFV1/SDHB</t>
+    <t xml:space="preserve">NDUFS8/NDUFV1/NDUFS2/SDHB/NDUFS1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0051537</t>
@@ -5365,7 +5365,7 @@
     <t xml:space="preserve">10/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFV2/NDUFS1/UQCRFS1/SDHB</t>
+    <t xml:space="preserve">SDHB/UQCRFS1/NDUFV2/NDUFS1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0016651</t>
@@ -5383,7 +5383,7 @@
     <t xml:space="preserve">68/352</t>
   </si>
   <si>
-    <t xml:space="preserve">ANP32E/PSMD1/CAB39/OSTF1/SLC44A2/ANXA4/DNM1L/PSMD13/RAB8A/HSPD1/CAV1/AP1B1/PSMC3/ATP6V1H/RAB10/GARS1/PARK7/IQGAP1/RAP2B/PSMD6/PSMC2/AP2B1/LAMP2/NAPA/CACNA2D1/SCCPDH/DIAPH1/GAA/SPTAN1/MAPK1/CPNE1/COPB1/RAB2B/PADI2/PRKACA/PSMA2/COPS5/CPPED1/PSMC4/XRCC5/KPNB1/TMED2/IDH1/ATP6V1E1/APRT/CYB5R1/PSMC1/IST1/DDX3X/ANXA7/PKM/LAMP1/PSMB4/BIN1/PSMA4/VCP/GDI2/ANXA11/GSTP1/NME2/RAB5B/TOM1/OLA1/CCT2/DYSF/CD36/ANXA2/RAP1B</t>
+    <t xml:space="preserve">DNM1L/HSPD1/SLC44A2/XRCC5/CAB39/RAB10/RAB5B/PSMA4/KPNB1/GAA/LAMP2/NAPA/PSMC3/PSMD6/PSMA2/PSMC4/AP2B1/PSMC1/ATP6V1E1/APRT/PSMD1/ANP32E/IQGAP1/ANXA2/GARS1/PSMC2/PADI2/MAPK1/PKM/RAP2B/IST1/OSTF1/ANXA11/RAB2B/PRKACA/COPB1/GDI2/RAP1B/CD36/DYSF/LAMP1/PSMB4/TMED2/DIAPH1/SCCPDH/PSMD13/SPTAN1/COPS5/CPPED1/CAV1/IDH1/CPNE1/DDX3X/ANXA7/ANXA4/VCP/GSTP1/ATP6V1H/RAB8A/PARK7/CACNA2D1/CYB5R1/NME2/TOM1/AP1B1/CCT2/OLA1/BIN1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005930</t>
@@ -5395,7 +5395,7 @@
     <t xml:space="preserve">9/352</t>
   </si>
   <si>
-    <t xml:space="preserve">SEPTIN9/PRKAR2A/RAB8A/PRKAR1A/SEPTIN2/PRKACA/NUBP2/USP9X/SEPTIN7</t>
+    <t xml:space="preserve">PRKACA/NUBP2/SEPTIN9/SEPTIN2/USP9X/RAB8A/PRKAR2A/SEPTIN7/PRKAR1A</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0097014</t>
@@ -5416,7 +5416,7 @@
     <t xml:space="preserve">59/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">ANP32E/PSMD1/DNM1L/PSMD13/RAB8A/AP1B1/PSMC3/ATP6V1H/RAB10/PARK7/PSMD6/PSMC2/AP2B1/NAPA/PSMA2/COPS5/PSMC4/ATP6V1E1/PSMC1/LAMP1/PSMB4/BIN1/PSMA4/RAB5B/DYSF</t>
+    <t xml:space="preserve">DNM1L/RAB10/RAB5B/PSMA4/NAPA/PSMC3/PSMD6/PSMA2/PSMC4/AP2B1/PSMC1/ATP6V1E1/PSMD1/ANP32E/PSMC2/DYSF/LAMP1/PSMB4/PSMD13/COPS5/ATP6V1H/RAB8A/PARK7/AP1B1/BIN1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0008021</t>
@@ -5428,19 +5428,19 @@
     <t xml:space="preserve">24/352</t>
   </si>
   <si>
-    <t xml:space="preserve">ANP32E/PSMD1/DNM1L/PSMD13/RAB8A/AP1B1/PSMC3/ATP6V1H/PARK7/PSMD6/PSMC2/AP2B1/NAPA/PSMA2/COPS5/PSMC4/ATP6V1E1/PSMC1/LAMP1/PSMB4/BIN1/PSMA4/RAB5B/DYSF</t>
+    <t xml:space="preserve">DNM1L/RAB5B/PSMA4/NAPA/PSMC3/PSMD6/PSMA2/PSMC4/AP2B1/PSMC1/ATP6V1E1/PSMD1/ANP32E/PSMC2/DYSF/LAMP1/PSMB4/PSMD13/COPS5/ATP6V1H/RAB8A/PARK7/AP1B1/BIN1</t>
   </si>
   <si>
     <t xml:space="preserve">96/352</t>
   </si>
   <si>
-    <t xml:space="preserve">UBA1/ANP32E/PSMD1/CAB39/OSTF1/SLC44A2/ANXA4/GOSR2/DNM1L/SAR1B/PSMD13/RAB8A/HSPD1/PDIA3/OPTN/CAV1/AP1B1/PSMC3/ATP6V1H/RAB10/COPZ1/EHD2/GARS1/PARK7/PDIA6/CAMK2D/IQGAP1/RAP2B/PSMD6/PSMC2/AP2B1/YWHAE/LAMP2/NAPA/PRKAR1A/CACNA2D1/SCCPDH/DIAPH1/GAA/SPTAN1/MAPK1/CPNE1/EZR/CDC42/COPB1/RAB2B/YWHAZ/PADI2/PRKACA/PSMA2/MYO1C/COPS5/CPPED1/PRDX5/SLC1A4/PSMC4/XRCC5/KPNB1/TMED2/IDH1/ATP6V1E1/APRT/CYB5R1/YWHAB/PSMC1/IST1/SEC31A/DDX3X/RAB21/ANXA7/PKM/ESD/SND1/LAMP1/PSMB4/MAP2K1/BIN1/PSMA4/VCP/GDI2/ANXA11/GSTP1/NME2/RAB5B/TOM1/MTM1/OLA1/CCT2/ECPAS/RPN1/OSBPL1A/DYSF/CD36/ANXA2/RAP1B/SCARB2</t>
+    <t xml:space="preserve">DNM1L/HSPD1/SLC44A2/XRCC5/CAB39/RAB10/COPZ1/RAB5B/PSMA4/KPNB1/GAA/MAP2K1/LAMP2/NAPA/PSMC3/PSMD6/MYO1C/PSMA2/SND1/PSMC4/SLC1A4/AP2B1/PSMC1/ATP6V1E1/APRT/PSMD1/ANP32E/RPN1/IQGAP1/ANXA2/SEC31A/CAMK2D/EHD2/GARS1/PSMC2/PADI2/MAPK1/YWHAB/PKM/RAP2B/IST1/OSTF1/ANXA11/RAB2B/PRKACA/COPB1/GDI2/RAP1B/CD36/DYSF/LAMP1/PSMB4/TMED2/DIAPH1/SCCPDH/PSMD13/SPTAN1/COPS5/PRDX5/CPPED1/CAV1/YWHAE/OSBPL1A/IDH1/UBA1/EZR/CDC42/CPNE1/RAB21/DDX3X/ANXA7/ANXA4/VCP/ESD/GSTP1/ATP6V1H/RAB8A/OPTN/PARK7/CACNA2D1/YWHAZ/ECPAS/MTM1/CYB5R1/SCARB2/SAR1B/NME2/TOM1/AP1B1/CCT2/OLA1/BIN1/GOSR2/PDIA3/PDIA6/PRKAR1A</t>
   </si>
   <si>
     <t xml:space="preserve">53/352</t>
   </si>
   <si>
-    <t xml:space="preserve">PSMD1/CAB39/OSTF1/SLC44A2/ANXA4/PSMD13/HSPD1/CAV1/PSMC3/RAB10/GARS1/IQGAP1/RAP2B/PSMD6/PSMC2/LAMP2/NAPA/CACNA2D1/SCCPDH/DIAPH1/GAA/SPTAN1/MAPK1/CPNE1/COPB1/RAB2B/PADI2/PRKACA/PSMA2/CPPED1/XRCC5/KPNB1/TMED2/IDH1/APRT/CYB5R1/IST1/DDX3X/ANXA7/PKM/LAMP1/VCP/GDI2/ANXA11/GSTP1/NME2/RAB5B/TOM1/OLA1/CCT2/CD36/ANXA2/RAP1B</t>
+    <t xml:space="preserve">HSPD1/SLC44A2/XRCC5/CAB39/RAB10/RAB5B/KPNB1/GAA/LAMP2/NAPA/PSMC3/PSMD6/PSMA2/APRT/PSMD1/IQGAP1/ANXA2/GARS1/PSMC2/PADI2/MAPK1/PKM/RAP2B/IST1/OSTF1/ANXA11/RAB2B/PRKACA/COPB1/GDI2/RAP1B/CD36/LAMP1/TMED2/DIAPH1/SCCPDH/PSMD13/SPTAN1/CPPED1/CAV1/IDH1/CPNE1/DDX3X/ANXA7/ANXA4/VCP/GSTP1/CACNA2D1/CYB5R1/NME2/TOM1/CCT2/OLA1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005929</t>
@@ -5452,7 +5452,7 @@
     <t xml:space="preserve">26/352</t>
   </si>
   <si>
-    <t xml:space="preserve">SEPTIN9/PRKAR2A/CUL3/AK1/RAB8A/TUBB2A/HSPD1/CAV1/PIN1/RAB10/PRKAR1A/EZR/SEPTIN2/GNB1/LDHA/GSTM3/PRKACA/NUBP2/PRKAA1/ATXN10/ATP2B4/PKM/USP9X/PSMB4/MAP2K1/SEPTIN7</t>
+    <t xml:space="preserve">HSPD1/RAB10/MAP2K1/GSTM3/GNB1/PIN1/PKM/PRKACA/ATXN10/NUBP2/SEPTIN9/SEPTIN2/PRKAA1/PSMB4/ATP2B4/CAV1/LDHA/EZR/USP9X/TUBB2A/RAB8A/PRKAR2A/CUL3/AK1/SEPTIN7/PRKAR1A</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0098772</t>
@@ -5467,7 +5467,7 @@
     <t xml:space="preserve">243/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">ANP32E/PSMD1/PRKAR2A/CAB39/TYMP/ANXA4/RPS15/DNM1L/SAR1B/EIF5/RAB8A/HSPD1/FERMT2/CAV1/PIN1/PLAA/AHSA1/PRKAG1/PSME2/ATP6V1H/RAB10/COQ9/DNAJA2/TRMT112/SNTA1/RPS7/PARK7/CAMK2D/IQGAP1/OGN/RAP2B/YWHAE/LAMP2/PRKRA/PRKAR1A/PPP1R12B/PRPSAP2/SSBP1/FNTA/CDC42/PRPSAP1/SEPTIN2/RAB2B/RPLP1/GSTM2/PRKACA/PRDX5/ANXA5/XRCC5/UBE2L3/ABCE1/ATP2B4/PPP2R1A/GCN1/YWHAB/HSPB2/DDX3X/RAB21/CAST/RIC8A/LAMP1/TIPRL/MAP2K1/STAC3/BIN1/VCP/PRKG1/IPO5/GDI2/GSTP1/RAB5B/FLNA/ARL1/OSBPL1A/PPP1R14B/ANXA2/RAP1B</t>
+    <t xml:space="preserve">PLAA/DNM1L/HSPD1/XRCC5/UBE2L3/CAB39/SNTA1/RAB10/PRKAG1/RAB5B/ABCE1/MAP2K1/LAMP2/EIF5/PRPSAP2/PPP1R12B/PPP1R14B/TIPRL/CAST/PSMD1/ANP32E/TRMT112/TYMP/COQ9/FERMT2/PIN1/DNAJA2/IQGAP1/PRPSAP1/ANXA2/HSPB2/AHSA1/CAMK2D/PRKRA/YWHAB/RAP2B/PPP2R1A/RPS15/RAB2B/RIC8A/PRKACA/PRKG1/OGN/SEPTIN2/FNTA/GDI2/IPO5/RPS7/SSBP1/RAP1B/LAMP1/ATP2B4/ARL1/PRDX5/ANXA5/CAV1/YWHAE/OSBPL1A/STAC3/CDC42/RAB21/DDX3X/ANXA4/VCP/GSTP1/ATP6V1H/PSME2/RAB8A/FLNA/PARK7/GSTM2/RPLP1/GCN1/PRKAR2A/SAR1B/BIN1/PRKAR1A</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0043168</t>
@@ -5482,7 +5482,7 @@
     <t xml:space="preserve">414/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">SEPTIN9/UBA1/PRKAR2A/ANXA4/AK1/DNM1L/SAR1B/EIF5/RAB8A/TUBB2A/COASY/HSPD1/FERMT2/PSMC3/OPA1/PRKAG1/RAB10/CCT6A/MCCC1/DNAJA2/EHD2/ARF5/GARS1/PIP4K2B/CAMK2D/IQGAP1/RAP2B/PSMC2/RBKS/PKLR/JPH2/CMPK1/CARNS1/ATAD1/GSTM1/PRKAR1A/COQ6/ATP12A/DDX1/TIMM44/CHORDC1/ACTR1A/OGDH/DRG1/ATL2/GART/CCT7/BCS1L/MAPK1/CPNE1/CDC42/BCKDK/NUDT2/SEPTIN2/ACTBL2/RAB2B/GSTM2/GSTM3/ATP2A1/SIRT3/PRKACA/HADHA/MYO1C/FARSA/NUBP2/ANXA5/PRKAA1/LANCL1/PSMC4/MTHFD1/XRCC5/UBE2G1/GSS/UBE2L3/ABCE1/CTPS1/MYH6/ATP2B4/DHTKD1/APRT/MAP2K4/CYB5R1/PITPNA/PSMC1/SARS1/DDX3X/RAB21/ANXA7/PKM/CFL1/MAPK9/PLPBP/RTCB/ADSS1/HADH/MAP2K1/UQCC3/VCP/PRKG1/ANXA11/GSTP1/NME2/RAB5B/SEPTIN7/NUBPL/FUNDC2/MYH3/OLA1/CCT2/PGK1/ALPK3/ARL1/ASS1/RTCA/ACAD10/ANXA2/RAP1B/NT5C2/SCARB2</t>
+    <t xml:space="preserve">DNM1L/HSPD1/XRCC5/PLPBP/UBE2L3/RAB10/PRKAG1/RAB5B/ARF5/COQ6/ABCE1/MAP2K1/GART/SARS1/PSMC3/COASY/MYO1C/EIF5/PSMC4/PSMC1/ACTR1A/APRT/ADSS1/GSTM3/RTCB/UBE2G1/FERMT2/ATAD1/GSTM1/DNAJA2/DRG1/IQGAP1/CCT6A/ANXA2/ACAD10/FARSA/OPA1/CAMK2D/EHD2/CARNS1/GARS1/RBKS/PSMC2/HADHA/ATP2A1/MAPK1/PITPNA/CFL1/PKM/RAP2B/MAPK9/ANXA11/RAB2B/MTHFD1/PRKACA/SIRT3/NUBP2/NUDT2/BCKDK/PRKG1/PKLR/TIMM44/SEPTIN9/SEPTIN2/ACTBL2/ATP12A/DDX1/PRKAA1/BCS1L/MYH6/CTPS1/RAP1B/CHORDC1/ATP2B4/MCCC1/ATL2/ARL1/CCT7/ANXA5/NT5C2/ASS1/RTCA/HADH/DHTKD1/GSS/UBA1/CDC42/CPNE1/RAB21/DDX3X/ANXA7/ANXA4/VCP/GSTP1/CMPK1/JPH2/TUBB2A/RAB8A/FUNDC2/NUBPL/GSTM2/PGK1/ALPK3/OGDH/PRKAR2A/AK1/CYB5R1/MAP2K4/SCARB2/SAR1B/NME2/SEPTIN7/CCT2/MYH3/OLA1/UQCC3/PIP4K2B/PRKAR1A/LANCL1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0008047</t>
@@ -5497,7 +5497,7 @@
     <t xml:space="preserve">66/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">CAB39/DNM1L/EIF5/HSPD1/FERMT2/CAV1/PIN1/PLAA/PSME2/COQ9/TRMT112/PARK7/IQGAP1/PRKRA/PPP1R12B/SSBP1/FNTA/RPLP1/XRCC5/UBE2L3/GCN1/HSPB2/DDX3X/TIPRL/MAP2K1/VCP/GDI2/ARL1</t>
+    <t xml:space="preserve">PLAA/DNM1L/HSPD1/XRCC5/UBE2L3/CAB39/MAP2K1/EIF5/PPP1R12B/TIPRL/TRMT112/COQ9/FERMT2/PIN1/IQGAP1/HSPB2/PRKRA/FNTA/GDI2/SSBP1/ARL1/CAV1/DDX3X/VCP/PSME2/PARK7/RPLP1/GCN1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0030234</t>
@@ -5512,7 +5512,7 @@
     <t xml:space="preserve">158/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">ANP32E/PSMD1/PRKAR2A/CAB39/ANXA4/RPS15/DNM1L/EIF5/HSPD1/FERMT2/CAV1/PIN1/PLAA/PRKAG1/PSME2/ATP6V1H/COQ9/TRMT112/RPS7/PARK7/IQGAP1/YWHAE/PRKRA/PRKAR1A/PPP1R12B/PRPSAP2/SSBP1/FNTA/PRPSAP1/SEPTIN2/RPLP1/PRDX5/ANXA5/XRCC5/UBE2L3/ABCE1/ATP2B4/PPP2R1A/GCN1/YWHAB/HSPB2/DDX3X/CAST/RIC8A/TIPRL/MAP2K1/BIN1/VCP/IPO5/GDI2/GSTP1/ARL1/PPP1R14B/ANXA2</t>
+    <t xml:space="preserve">PLAA/DNM1L/HSPD1/XRCC5/UBE2L3/CAB39/PRKAG1/ABCE1/MAP2K1/EIF5/PRPSAP2/PPP1R12B/PPP1R14B/TIPRL/CAST/PSMD1/ANP32E/TRMT112/COQ9/FERMT2/PIN1/IQGAP1/PRPSAP1/ANXA2/HSPB2/PRKRA/YWHAB/PPP2R1A/RPS15/RIC8A/SEPTIN2/FNTA/GDI2/IPO5/RPS7/SSBP1/ATP2B4/ARL1/PRDX5/ANXA5/CAV1/YWHAE/DDX3X/ANXA4/VCP/GSTP1/ATP6V1H/PSME2/PARK7/RPLP1/GCN1/PRKAR2A/BIN1/PRKAR1A</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0017076</t>
@@ -5527,7 +5527,7 @@
     <t xml:space="preserve">340/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">SEPTIN9/UBA1/PRKAR2A/AK1/DNM1L/SAR1B/EIF5/RAB8A/TUBB2A/COASY/HSPD1/PSMC3/OPA1/PRKAG1/RAB10/CCT6A/MCCC1/DNAJA2/EHD2/ARF5/GARS1/PIP4K2B/CAMK2D/RAP2B/PSMC2/RBKS/PKLR/CMPK1/CARNS1/ATAD1/PRKAR1A/SPR/ATP12A/DDX1/TIMM44/CHORDC1/ACTR1A/DRG1/ATL2/GART/CCT7/BCS1L/MAPK1/CDC42/ME2/BCKDK/NUDT2/SEPTIN2/ACTBL2/RAB2B/ATP2A1/SIRT3/PRKACA/HADHA/MYO1C/FARSA/NUBP2/PRKAA1/PSMC4/MTHFD1/XRCC5/UBE2G1/GSS/UBE2L3/ABCE1/CTPS1/MYH6/ATP2B4/IDH1/APRT/MAP2K4/PSMC1/SARS1/DDX3X/RAB21/PKM/MAPK9/RTCB/ADSS1/HADH/GPD1/MAP2K1/VCP/PRKG1/NME2/RAB5B/SEPTIN7/NUBPL/MYH3/OLA1/CCT2/PGK1/ALPK3/ARL1/ASS1/RTCA/RAP1B/NT5C2</t>
+    <t xml:space="preserve">DNM1L/HSPD1/XRCC5/UBE2L3/RAB10/PRKAG1/RAB5B/ARF5/ABCE1/MAP2K1/GART/SARS1/PSMC3/COASY/MYO1C/EIF5/SPR/PSMC4/PSMC1/ACTR1A/APRT/ADSS1/RTCB/UBE2G1/ATAD1/DNAJA2/DRG1/CCT6A/FARSA/OPA1/CAMK2D/EHD2/CARNS1/GARS1/RBKS/PSMC2/HADHA/ATP2A1/MAPK1/PKM/RAP2B/MAPK9/RAB2B/MTHFD1/PRKACA/SIRT3/NUBP2/NUDT2/ME2/BCKDK/PRKG1/PKLR/TIMM44/SEPTIN9/SEPTIN2/ACTBL2/ATP12A/DDX1/PRKAA1/BCS1L/MYH6/CTPS1/RAP1B/CHORDC1/GPD1/ATP2B4/MCCC1/ATL2/ARL1/CCT7/NT5C2/ASS1/RTCA/HADH/IDH1/GSS/UBA1/CDC42/RAB21/DDX3X/VCP/CMPK1/TUBB2A/RAB8A/NUBPL/PGK1/ALPK3/PRKAR2A/AK1/MAP2K4/SAR1B/NME2/SEPTIN7/CCT2/MYH3/OLA1/PIP4K2B/PRKAR1A</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0032555</t>
@@ -5542,7 +5542,7 @@
     <t xml:space="preserve">312/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">SEPTIN9/UBA1/PRKAR2A/AK1/DNM1L/SAR1B/EIF5/RAB8A/TUBB2A/COASY/HSPD1/PSMC3/OPA1/PRKAG1/RAB10/CCT6A/MCCC1/DNAJA2/EHD2/ARF5/GARS1/PIP4K2B/CAMK2D/RAP2B/PSMC2/RBKS/PKLR/CMPK1/CARNS1/ATAD1/PRKAR1A/ATP12A/DDX1/TIMM44/CHORDC1/ACTR1A/DRG1/ATL2/GART/CCT7/BCS1L/MAPK1/CDC42/BCKDK/NUDT2/SEPTIN2/ACTBL2/RAB2B/ATP2A1/PRKACA/MYO1C/FARSA/NUBP2/PRKAA1/PSMC4/MTHFD1/XRCC5/UBE2G1/GSS/UBE2L3/ABCE1/CTPS1/MYH6/ATP2B4/APRT/MAP2K4/PSMC1/SARS1/DDX3X/RAB21/PKM/MAPK9/RTCB/ADSS1/MAP2K1/VCP/PRKG1/NME2/RAB5B/SEPTIN7/NUBPL/MYH3/OLA1/CCT2/PGK1/ALPK3/ARL1/ASS1/RTCA/RAP1B/NT5C2</t>
+    <t xml:space="preserve">DNM1L/HSPD1/XRCC5/UBE2L3/RAB10/PRKAG1/RAB5B/ARF5/ABCE1/MAP2K1/GART/SARS1/PSMC3/COASY/MYO1C/EIF5/PSMC4/PSMC1/ACTR1A/APRT/ADSS1/RTCB/UBE2G1/ATAD1/DNAJA2/DRG1/CCT6A/FARSA/OPA1/CAMK2D/EHD2/CARNS1/GARS1/RBKS/PSMC2/ATP2A1/MAPK1/PKM/RAP2B/MAPK9/RAB2B/MTHFD1/PRKACA/NUBP2/NUDT2/BCKDK/PRKG1/PKLR/TIMM44/SEPTIN9/SEPTIN2/ACTBL2/ATP12A/DDX1/PRKAA1/BCS1L/MYH6/CTPS1/RAP1B/CHORDC1/ATP2B4/MCCC1/ATL2/ARL1/CCT7/NT5C2/ASS1/RTCA/GSS/UBA1/CDC42/RAB21/DDX3X/VCP/CMPK1/TUBB2A/RAB8A/NUBPL/PGK1/ALPK3/PRKAR2A/AK1/MAP2K4/SAR1B/NME2/SEPTIN7/CCT2/MYH3/OLA1/PIP4K2B/PRKAR1A</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0032553</t>
@@ -5563,7 +5563,7 @@
     <t xml:space="preserve">13/352</t>
   </si>
   <si>
-    <t xml:space="preserve">ANXA4/JPH2/GSTM1/CPNE1/GSTM2/GSTM3/ANXA5/LANCL1/GSS/ANXA7/ANXA11/ANXA2/SCARB2</t>
+    <t xml:space="preserve">GSTM3/GSTM1/ANXA2/ANXA11/ANXA5/GSS/CPNE1/ANXA7/ANXA4/JPH2/GSTM2/SCARB2/LANCL1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005544</t>
@@ -5578,7 +5578,7 @@
     <t xml:space="preserve">12/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">ANXA4/ESYT1/CPNE1/ANXA5/ANXA7/ANXA11/DYSF/ANXA2</t>
+    <t xml:space="preserve">ANXA2/ANXA11/DYSF/ANXA5/CPNE1/ANXA7/ANXA4/ESYT1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0140677</t>
@@ -5593,7 +5593,7 @@
     <t xml:space="preserve">93/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">CAB39/TYMP/DNM1L/EIF5/HSPD1/FERMT2/CAV1/PIN1/PLAA/AHSA1/PSME2/COQ9/DNAJA2/TRMT112/PARK7/IQGAP1/OGN/PRKRA/PPP1R12B/SSBP1/FNTA/RPLP1/PRKACA/XRCC5/UBE2L3/GCN1/HSPB2/DDX3X/TIPRL/MAP2K1/VCP/GDI2/ARL1</t>
+    <t xml:space="preserve">PLAA/DNM1L/HSPD1/XRCC5/UBE2L3/CAB39/MAP2K1/EIF5/PPP1R12B/TIPRL/TRMT112/TYMP/COQ9/FERMT2/PIN1/DNAJA2/IQGAP1/HSPB2/AHSA1/PRKRA/PRKACA/OGN/FNTA/GDI2/SSBP1/ARL1/CAV1/DDX3X/VCP/PSME2/PARK7/RPLP1/GCN1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0017111</t>
@@ -5608,7 +5608,7 @@
     <t xml:space="preserve">135/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">SEPTIN9/DNM1L/SAR1B/RAB8A/TUBB2A/HSPD1/GNB2/TPPP/PSMC3/OPA1/ATP6V1H/RAB10/CCT6A/ARF5/RAP2B/PSMC2/CARNS1/ATAD1/ATP12A/DDX1/DRG1/ATL2/CCT7/BCS1L/CDC42/SEPTIN2/GNB1/RAB2B/ATP2A1/PSMC4/XRCC5/ABCE1/ATP2B4/PSMC1/DDX3X/RAB21/VCP/RAB5B/SEPTIN7/MYH3/OLA1/CCT2/ARL1/RAP1B</t>
+    <t xml:space="preserve">DNM1L/HSPD1/XRCC5/RAB10/RAB5B/ARF5/ABCE1/PSMC3/PSMC4/PSMC1/GNB1/ATAD1/DRG1/CCT6A/OPA1/CARNS1/PSMC2/ATP2A1/RAP2B/TPPP/RAB2B/SEPTIN9/SEPTIN2/ATP12A/DDX1/BCS1L/RAP1B/ATP2B4/ATL2/ARL1/CCT7/CDC42/RAB21/DDX3X/VCP/ATP6V1H/TUBB2A/RAB8A/SAR1B/GNB2/SEPTIN7/CCT2/MYH3/OLA1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0016879</t>
@@ -5617,7 +5617,7 @@
     <t xml:space="preserve">ligase activity, forming carbon-nitrogen bonds</t>
   </si>
   <si>
-    <t xml:space="preserve">MCCC1/CARNS1/GART/MTHFD1/GSS/CTPS1/ADSS1/ASS1</t>
+    <t xml:space="preserve">GART/ADSS1/CARNS1/MTHFD1/CTPS1/MCCC1/ASS1/GSS</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0035639</t>
@@ -5632,7 +5632,7 @@
     <t xml:space="preserve">307/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">SEPTIN9/UBA1/AK1/DNM1L/SAR1B/EIF5/RAB8A/TUBB2A/COASY/HSPD1/PSMC3/OPA1/PRKAG1/RAB10/CCT6A/MCCC1/DNAJA2/EHD2/ARF5/GARS1/PIP4K2B/CAMK2D/RAP2B/PSMC2/RBKS/PKLR/CMPK1/CARNS1/ATAD1/ATP12A/DDX1/TIMM44/CHORDC1/ACTR1A/DRG1/ATL2/GART/CCT7/BCS1L/MAPK1/CDC42/BCKDK/NUDT2/SEPTIN2/ACTBL2/RAB2B/ATP2A1/PRKACA/MYO1C/FARSA/NUBP2/PRKAA1/PSMC4/MTHFD1/XRCC5/UBE2G1/GSS/UBE2L3/ABCE1/CTPS1/MYH6/ATP2B4/MAP2K4/PSMC1/SARS1/DDX3X/RAB21/PKM/MAPK9/RTCB/ADSS1/MAP2K1/VCP/PRKG1/RAB5B/SEPTIN7/NUBPL/MYH3/OLA1/CCT2/PGK1/ALPK3/ARL1/ASS1/RTCA/RAP1B/NT5C2</t>
+    <t xml:space="preserve">DNM1L/HSPD1/XRCC5/UBE2L3/RAB10/PRKAG1/RAB5B/ARF5/ABCE1/MAP2K1/GART/SARS1/PSMC3/COASY/MYO1C/EIF5/PSMC4/PSMC1/ACTR1A/ADSS1/RTCB/UBE2G1/ATAD1/DNAJA2/DRG1/CCT6A/FARSA/OPA1/CAMK2D/EHD2/CARNS1/GARS1/RBKS/PSMC2/ATP2A1/MAPK1/PKM/RAP2B/MAPK9/RAB2B/MTHFD1/PRKACA/NUBP2/NUDT2/BCKDK/PRKG1/PKLR/TIMM44/SEPTIN9/SEPTIN2/ACTBL2/ATP12A/DDX1/PRKAA1/BCS1L/MYH6/CTPS1/RAP1B/CHORDC1/ATP2B4/MCCC1/ATL2/ARL1/CCT7/NT5C2/ASS1/RTCA/GSS/UBA1/CDC42/RAB21/DDX3X/VCP/CMPK1/TUBB2A/RAB8A/NUBPL/PGK1/ALPK3/AK1/MAP2K4/SAR1B/SEPTIN7/CCT2/MYH3/OLA1/PIP4K2B</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0016462</t>
@@ -5647,7 +5647,7 @@
     <t xml:space="preserve">144/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">SEPTIN9/DNM1L/SAR1B/RAB8A/TUBB2A/HSPD1/GNB2/TPPP/PSMC3/OPA1/ATP6V1H/RAB10/CCT6A/ARF5/GARS1/RAP2B/PSMC2/CARNS1/ATAD1/ATP12A/DDX1/DRG1/ATL2/CCT7/BCS1L/CDC42/NUDT2/SEPTIN2/GNB1/RAB2B/ATP2A1/PSMC4/XRCC5/ABCE1/ATP2B4/PSMC1/DDX3X/RAB21/VCP/RAB5B/SEPTIN7/MYH3/OLA1/CCT2/ARL1/RAP1B</t>
+    <t xml:space="preserve">DNM1L/HSPD1/XRCC5/RAB10/RAB5B/ARF5/ABCE1/PSMC3/PSMC4/PSMC1/GNB1/ATAD1/DRG1/CCT6A/OPA1/CARNS1/GARS1/PSMC2/ATP2A1/RAP2B/TPPP/RAB2B/NUDT2/SEPTIN9/SEPTIN2/ATP12A/DDX1/BCS1L/RAP1B/ATP2B4/ATL2/ARL1/CCT7/CDC42/RAB21/DDX3X/VCP/ATP6V1H/TUBB2A/RAB8A/SAR1B/GNB2/SEPTIN7/CCT2/MYH3/OLA1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0016817</t>
@@ -5674,7 +5674,7 @@
     <t xml:space="preserve">60/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">PSMD1/PRKAR2A/CUL3/DNM1L/DBT/HSPD1/RTN4/ERLIN2/YWHAE/PRKAR1A/NPLOC4/NAE1/LRPPRC/YWHAZ/CUL5/CUL4B/XRCC5/UBE2G1/UBE2L3/CUL4A/FBXO7/VCP/CCT2</t>
+    <t xml:space="preserve">DNM1L/HSPD1/XRCC5/UBE2L3/DBT/PSMD1/UBE2G1/CUL4A/RTN4/NAE1/NPLOC4/FBXO7/CUL4B/LRPPRC/YWHAE/VCP/CUL5/YWHAZ/PRKAR2A/CUL3/CCT2/ERLIN2/PRKAR1A</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0044389</t>
@@ -5695,7 +5695,7 @@
     <t xml:space="preserve">40/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">DNM1L/RAB8A/GNB2/CAV1/XPO1/ENO1/IQGAP1/DIAPH1/GNB1/CSE1L/MYO1C/KPNB1/MAP2K1/BIN1/IPO5/GDI2/FLNA</t>
+    <t xml:space="preserve">DNM1L/KPNB1/MAP2K1/MYO1C/GNB1/IQGAP1/CSE1L/GDI2/IPO5/DIAPH1/CAV1/RAB8A/FLNA/XPO1/GNB2/BIN1/ENO1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0019899</t>
@@ -5710,7 +5710,7 @@
     <t xml:space="preserve">296/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">PXN/PSMD1/PRKAR2A/CAB39/CUL3/DNM1L/POTEI/RAB8A/DBT/HSPD1/GNB2/FERMT2/CAV1/PIN1/AP1B1/PPP1CA/XPO1/PRKAG1/ENO1/PPP1CB/SNTA1/RPS7/PARK7/IQGAP1/CRADD/RTN4/ERLIN2/YWHAE/LAMP2/PRKRA/GSTM1/PRKAR1A/NPLOC4/PPP1R12B/NAE1/LRPPRC/DIAPH1/FNTA/MAPK1/EZR/CDC42/ACTBL2/GNB1/PLIN5/CSE1L/GSTM2/YWHAZ/CUL5/GSTM3/SIRT3/PRKACA/MYO1C/COPS5/CUL4B/DCUN1D1/XRCC5/UBE2G1/UBE2L3/KPNB1/MYH6/ATP2B4/CUL4A/FBXO7/ATP6V1E1/RPS2/MAP2K4/YWHAB/AKAP12/SARS1/CFL1/ARIH2/RDX/POTEF/LAMP1/MAP2K1/BIN1/VCP/IPO5/GDI2/GSTP1/FLNA/CCT2/ANXA2/SCARB2</t>
+    <t xml:space="preserve">DNM1L/HSPD1/XRCC5/UBE2L3/CAB39/SNTA1/PRKAG1/KPNB1/MAP2K1/CRADD/SARS1/LAMP2/DBT/MYO1C/POTEF/POTEI/PPP1R12B/ATP6V1E1/GSTM3/PSMD1/GNB1/UBE2G1/RPS2/FERMT2/PIN1/GSTM1/CUL4A/RTN4/IQGAP1/ANXA2/RDX/ARIH2/PRKRA/PXN/MAPK1/YWHAB/CFL1/AKAP12/CSE1L/PRKACA/SIRT3/DCUN1D1/ACTBL2/FNTA/GDI2/IPO5/RPS7/MYH6/NAE1/PPP1CB/NPLOC4/FBXO7/CUL4B/LAMP1/ATP2B4/LRPPRC/DIAPH1/COPS5/CAV1/YWHAE/EZR/CDC42/VCP/GSTP1/RAB8A/FLNA/CUL5/PARK7/GSTM2/YWHAZ/XPO1/PRKAR2A/CUL3/MAP2K4/SCARB2/GNB2/AP1B1/CCT2/BIN1/ENO1/PLIN5/ERLIN2/PRKAR1A/PPP1CA</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0016787</t>
@@ -5722,31 +5722,31 @@
     <t xml:space="preserve">326/1596</t>
   </si>
   <si>
-    <t xml:space="preserve">SEPTIN9/DNM1L/SAR1B/RAB8A/TUBB2A/HSPD1/PDIA3/GNB2/TPPP/SCRN3/PPP1CA/PREP/PSMC3/EPHX2/OPA1/ATP6V1H/RAB10/CCT6A/EHD2/ARF5/GARS1/PPP1CB/PARK7/IAH1/DNPEP/PUDP/RAP2B/PSMC2/ACOT9/CARNS1/ATAD1/ATP12A/DDX1/INPP1/DRG1/ATL2/GAA/SCRN2/CCT7/BCS1L/CPNE1/CDC42/BCKDK/NUDT2/SEPTIN2/NLN/MOGS/ACAA2/GNB1/RAB2B/ATP2A1/PADI2/HADHA/COPS5/CPPED1/PSMC4/DNPH1/MTHFD1/ATIC/XRCC5/DHODH/ABCE1/CTPS1/MYH6/ATP2B4/PPP2R1A/AGMAT/USP5/CMBL/ERAP1/PSMC1/DDX3X/RAB21/ACOT13/CAPNS1/ESD/USP9X/SND1/VCP/RAB5B/NT5C/SEPTIN7/MTM1/MYH3/OLA1/CCT2/ARL1/PTRHD1/RAP1B/PPP2CB/NT5C2</t>
+    <t xml:space="preserve">DNM1L/HSPD1/SCRN3/XRCC5/RAB10/RAB5B/ARF5/ACOT13/ABCE1/GAA/PSMC3/SND1/PSMC4/PSMC1/ACAA2/GNB1/ATAD1/DRG1/PUDP/CCT6A/NT5C/OPA1/DNPEP/CAPNS1/EHD2/CARNS1/EPHX2/GARS1/PSMC2/HADHA/NLN/MOGS/IAH1/ATP2A1/PADI2/RAP2B/PPP2R1A/AGMAT/TPPP/RAB2B/ATIC/MTHFD1/NUDT2/BCKDK/DNPH1/SEPTIN9/SEPTIN2/ATP12A/DDX1/BCS1L/MYH6/CTPS1/PPP1CB/RAP1B/ATP2B4/INPP1/ATL2/ARL1/CCT7/COPS5/CPPED1/PPP2CB/NT5C2/PTRHD1/SCRN2/CDC42/CPNE1/RAB21/DDX3X/VCP/USP9X/ESD/ATP6V1H/ACOT9/TUBB2A/RAB8A/PARK7/DHODH/PREP/MTM1/SAR1B/GNB2/SEPTIN7/CCT2/MYH3/OLA1/ERAP1/CMBL/PDIA3/USP5/PPP1CA</t>
   </si>
   <si>
     <t xml:space="preserve">42/156</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/IDH3G/HCCS/DLST/ATP5F1A/MFN2/NNT/MT-CO2/PPIF/IDH3A/COX5B/ALDOA/DLAT/FH/UQCRC1/COX6B1/IDH2/COX5A/PDHX/NDUFB9/MDH2/NDUFB8/SLC25A13/UQCRC2/NDUFA7/NDUFB10/ATP5ME/PDHA1/ATP5PO/NDUFA2/NDUFB4/SUCLG1/MT-ND3/PDPR/PDK2/NDUFA3/COX4I1/NDUFA12/CHCHD2/PDHB/TRAP1/CS</t>
+    <t xml:space="preserve">PDK2/PDHB/COX5A/PDHA1/MFN2/COX5B/COX4I1/CHCHD2/DLAT/UQCRC2/IDH2/NDUFB8/CS/UQCRC1/FH/TRAP1/NNT/PPIF/MT-CO2/SUCLG1/COX6B1/NDUFB10/ALDOA/SLC25A13/PDHX/ATP5PO/NDUFA2/HCCS/DLST/MDH2/NDUFA12/NDUFA7/NDUFS7/ATP5ME/IDH3G/MT-ND3/PDPR/NDUFB4/NDUFA3/NDUFB9/ATP5F1A/IDH3A</t>
   </si>
   <si>
     <t xml:space="preserve">46/156</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/IDH3G/HCCS/DLST/ATP5F1A/MFN2/NNT/MT-CO2/PPIF/IDH3A/COX5B/ALDOA/DLAT/FH/UQCRC1/COX6B1/IDH2/COX5A/PHKG1/PDHX/NDUFB9/MDH2/NDUFB8/SLC25A13/UQCRC2/NDUFA7/NDUFB10/ATP5ME/PDHA1/ATP5PO/NDUFA2/NDUFB4/SUCLG1/MT-ND3/PDPR/PDK2/NDUFA3/COX4I1/NDUFA12/CHCHD2/PDHB/GYG1/TRAP1/GYS1/CS/PYGB</t>
+    <t xml:space="preserve">GYG1/PDK2/PDHB/COX5A/PDHA1/MFN2/COX5B/COX4I1/CHCHD2/DLAT/GYS1/UQCRC2/IDH2/NDUFB8/CS/UQCRC1/FH/PYGB/TRAP1/NNT/PPIF/MT-CO2/SUCLG1/COX6B1/NDUFB10/ALDOA/SLC25A13/PDHX/ATP5PO/NDUFA2/PHKG1/HCCS/DLST/MDH2/NDUFA12/NDUFA7/NDUFS7/ATP5ME/IDH3G/MT-ND3/PDPR/NDUFB4/NDUFA3/NDUFB9/ATP5F1A/IDH3A</t>
   </si>
   <si>
     <t xml:space="preserve">47/156</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/IDH3G/HCCS/DLST/ATP5F1A/MFN2/NNT/MT-CO2/PPIF/IDH3A/COX5B/ALDOA/DLAT/FH/UQCRC1/COX6B1/IDH2/COX5A/PHKG1/PDHX/NDUFB9/MDH2/NDUFB8/SLC25A13/UQCRC2/NDUFA7/NDUFB10/ATP5ME/PDHA1/ATP5PO/NDUFA2/NDUFB4/HMGCL/SUCLG1/MT-ND3/PDPR/PDK2/NDUFA3/COX4I1/NDUFA12/CHCHD2/PDHB/GYG1/TRAP1/GYS1/CS/PYGB</t>
+    <t xml:space="preserve">GYG1/HMGCL/PDK2/PDHB/COX5A/PDHA1/MFN2/COX5B/COX4I1/CHCHD2/DLAT/GYS1/UQCRC2/IDH2/NDUFB8/CS/UQCRC1/FH/PYGB/TRAP1/NNT/PPIF/MT-CO2/SUCLG1/COX6B1/NDUFB10/ALDOA/SLC25A13/PDHX/ATP5PO/NDUFA2/PHKG1/HCCS/DLST/MDH2/NDUFA12/NDUFA7/NDUFS7/ATP5ME/IDH3G/MT-ND3/PDPR/NDUFB4/NDUFA3/NDUFB9/ATP5F1A/IDH3A</t>
   </si>
   <si>
     <t xml:space="preserve">39/156</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/IDH3G/DLST/ATP5F1A/MFN2/NNT/MT-CO2/PPIF/IDH3A/COX5B/ALDOA/DLAT/FH/UQCRC1/COX6B1/IDH2/COX5A/PDHX/NDUFB9/MDH2/NDUFB8/UQCRC2/NDUFA7/NDUFB10/ATP5ME/PDHA1/ATP5PO/NDUFA2/NDUFB4/SUCLG1/MT-ND3/PDPR/PDK2/NDUFA3/COX4I1/NDUFA12/CHCHD2/PDHB/CS</t>
+    <t xml:space="preserve">PDK2/PDHB/COX5A/PDHA1/MFN2/COX5B/COX4I1/CHCHD2/DLAT/UQCRC2/IDH2/NDUFB8/CS/UQCRC1/FH/NNT/PPIF/MT-CO2/SUCLG1/COX6B1/NDUFB10/ALDOA/PDHX/ATP5PO/NDUFA2/DLST/MDH2/NDUFA12/NDUFA7/NDUFS7/ATP5ME/IDH3G/MT-ND3/PDPR/NDUFB4/NDUFA3/NDUFB9/ATP5F1A/IDH3A</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006637</t>
@@ -5758,7 +5758,7 @@
     <t xml:space="preserve">17/156</t>
   </si>
   <si>
-    <t xml:space="preserve">DLST/PCCA/DLAT/ACSL1/MMUT/PDHX/GCDH/PDHA1/CBR4/OXSM/SUCLG1/PDPR/PDK2/ALDH7A1/PDHB/ACACA/ACSF2</t>
+    <t xml:space="preserve">PDK2/PDHB/PDHA1/ALDH7A1/DLAT/ACSL1/ACSF2/SUCLG1/PDHX/CBR4/DLST/MMUT/PCCA/OXSM/PDPR/GCDH/ACACA</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0071616</t>
@@ -5770,19 +5770,19 @@
     <t xml:space="preserve">13/156</t>
   </si>
   <si>
-    <t xml:space="preserve">DLST/PCCA/DLAT/ACSL1/MMUT/PDHX/GCDH/PDHA1/CBR4/PDPR/PDK2/PDHB/ACACA</t>
+    <t xml:space="preserve">PDK2/PDHB/PDHA1/DLAT/ACSL1/PDHX/CBR4/DLST/MMUT/PCCA/PDPR/GCDH/ACACA</t>
   </si>
   <si>
     <t xml:space="preserve">30/156</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/DLST/ATP5F1A/PCCA/ALDOA/DLAT/IDH2/ACSL1/MMUT/PDHX/DMAC2L/NDUFB9/GCDH/NDUFB8/SLC25A13/NDUFA7/NDUFB10/ATP5ME/PDHA1/ATP5PO/NDUFA2/CBR4/NDUFB4/MT-ND3/PDPR/PDK2/NDUFA3/NDUFA12/PDHB/ACACA</t>
+    <t xml:space="preserve">PDK2/PDHB/PDHA1/DMAC2L/DLAT/IDH2/NDUFB8/ACSL1/NDUFB10/ALDOA/SLC25A13/PDHX/CBR4/ATP5PO/NDUFA2/DLST/MMUT/NDUFA12/PCCA/NDUFA7/NDUFS7/ATP5ME/MT-ND3/PDPR/NDUFB4/NDUFA3/NDUFB9/GCDH/ATP5F1A/ACACA</t>
   </si>
   <si>
     <t xml:space="preserve">24/156</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/SLC16A1/ATP5F1A/NNT/MT-CO2/COX5B/UQCRC1/LETM1/COX6B1/COX5A/DMAC2L/NDUFB9/NDUFB8/SLC25A13/NDUFA7/NDUFB10/ATP5ME/ATP5PO/NDUFA2/NDUFB4/MT-ND3/NDUFA3/COX4I1/NDUFA12</t>
+    <t xml:space="preserve">COX5A/SLC16A1/COX5B/COX4I1/DMAC2L/NDUFB8/LETM1/UQCRC1/NNT/MT-CO2/COX6B1/NDUFB10/SLC25A13/ATP5PO/NDUFA2/NDUFA12/NDUFA7/NDUFS7/ATP5ME/MT-ND3/NDUFB4/NDUFA3/NDUFB9/ATP5F1A</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006099</t>
@@ -5794,7 +5794,7 @@
     <t xml:space="preserve">12/156</t>
   </si>
   <si>
-    <t xml:space="preserve">IDH3G/DLST/NNT/IDH3A/DLAT/FH/IDH2/MDH2/PDHA1/SUCLG1/PDHB/CS</t>
+    <t xml:space="preserve">PDHB/PDHA1/DLAT/IDH2/CS/FH/NNT/SUCLG1/DLST/MDH2/IDH3G/IDH3A</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006084</t>
@@ -5806,34 +5806,34 @@
     <t xml:space="preserve">10/156</t>
   </si>
   <si>
-    <t xml:space="preserve">DLST/DLAT/PDHX/GCDH/PDHA1/PDPR/PDK2/ALDH7A1/PDHB/ACACA</t>
+    <t xml:space="preserve">PDK2/PDHB/PDHA1/ALDH7A1/DLAT/PDHX/DLST/PDPR/GCDH/ACACA</t>
   </si>
   <si>
     <t xml:space="preserve">27/156</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/MFN2/PPIF/SAMM50/MTX1/ATAD3A/LETM1/ENDOG/COX20/NDUFAF3/FXN/MTCH2/ATPAF2/LONP1/DNAJA3/TIMM10/HTRA2/APOO/VDAC2/TIMM9/COX19/NDUFAF5/AIFM1/CHCHD2/TMEM11/TIMM13/SLC25A46</t>
+    <t xml:space="preserve">TIMM9/MFN2/TIMM13/APOO/NDUFAF5/ATPAF2/CHCHD2/TMEM11/ATAD3A/TIMM10/DNAJA3/SLC25A46/LETM1/ENDOG/COX19/PPIF/HTRA2/AIFM1/SAMM50/VDAC2/FXN/LONP1/NDUFAF3/MTX1/NDUFS7/COX20/MTCH2</t>
   </si>
   <si>
     <t xml:space="preserve">38/156</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/SLC16A1/ATP5F1A/NNT/MT-CO2/SAMM50/COX5B/ANK2/CACNB1/VDAC1/UQCRC1/LETM1/COX6B1/ACSL1/COX5A/STIM1/DMAC2L/NDUFB9/NDUFB8/SLC25A6/SLC25A13/NDUFA7/NDUFB10/ATP5ME/ATP5PO/NDUFA2/AFG3L2/NDUFB4/VDAC2/ANK3/MT-ND3/CPT1A/NDUFA3/COX4I1/CLIC5/NDUFA12/AIFM1/MPC2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NDUFS7/DLST/ATP5F1A/NNT/GOT2/PCCA/ALDOA/DLAT/MCCC2/IDH2/ACSL1/MMUT/PDHX/DMAC2L/NDUFB9/GCDH/MDH2/NDUFB8/SLC25A13/NDUFA7/NDUFB10/ATP5ME/PDHA1/ATP5PO/NDUFA2/CBR4/OXSM/NDUFB4/SUCLG1/MT-ND3/PDPR/PDK2/NDUFA3/ALDH7A1/NDUFA12/PDHB/ACACA/ACSF2</t>
+    <t xml:space="preserve">COX5A/SLC16A1/COX5B/COX4I1/DMAC2L/NDUFB8/LETM1/UQCRC1/ACSL1/ANK2/NNT/MT-CO2/ANK3/COX6B1/NDUFB10/AIFM1/SLC25A13/SLC25A6/ATP5PO/NDUFA2/SAMM50/AFG3L2/STIM1/VDAC2/CLIC5/NDUFA12/VDAC1/NDUFA7/NDUFS7/ATP5ME/CACNB1/MT-ND3/CPT1A/NDUFB4/NDUFA3/NDUFB9/ATP5F1A/MPC2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOT2/PDK2/MCCC2/PDHB/PDHA1/ALDH7A1/DMAC2L/DLAT/IDH2/NDUFB8/ACSL1/ACSF2/NNT/SUCLG1/NDUFB10/ALDOA/SLC25A13/PDHX/CBR4/ATP5PO/NDUFA2/DLST/MMUT/MDH2/NDUFA12/PCCA/NDUFA7/NDUFS7/ATP5ME/OXSM/MT-ND3/PDPR/NDUFB4/NDUFA3/NDUFB9/GCDH/ATP5F1A/ACACA</t>
   </si>
   <si>
     <t xml:space="preserve">22/156</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/ATP5F1A/MT-CO2/PPIF/COX5B/UQCRC1/COX6B1/COX5A/NDUFB9/NDUFB8/UQCRC2/NDUFA7/NDUFB10/ATP5ME/ATP5PO/NDUFA2/NDUFB4/MT-ND3/NDUFA3/COX4I1/NDUFA12/CHCHD2</t>
+    <t xml:space="preserve">COX5A/COX5B/COX4I1/CHCHD2/UQCRC2/NDUFB8/UQCRC1/PPIF/MT-CO2/COX6B1/NDUFB10/ATP5PO/NDUFA2/NDUFA12/NDUFA7/NDUFS7/ATP5ME/MT-ND3/NDUFB4/NDUFA3/NDUFB9/ATP5F1A</t>
   </si>
   <si>
     <t xml:space="preserve">32/156</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/SLC16A1/ATP5F1A/NNT/MT-CO2/COX5B/ANK2/CACNB1/VDAC1/UQCRC1/LETM1/COX6B1/COX5A/STIM1/DMAC2L/NDUFB9/NDUFB8/SLC25A13/NDUFA7/NDUFB10/ATP5ME/ATP5PO/NDUFA2/AFG3L2/NDUFB4/VDAC2/ANK3/MT-ND3/NDUFA3/COX4I1/CLIC5/NDUFA12</t>
+    <t xml:space="preserve">COX5A/SLC16A1/COX5B/COX4I1/DMAC2L/NDUFB8/LETM1/UQCRC1/ANK2/NNT/MT-CO2/ANK3/COX6B1/NDUFB10/SLC25A13/ATP5PO/NDUFA2/AFG3L2/STIM1/VDAC2/CLIC5/NDUFA12/VDAC1/NDUFA7/NDUFS7/ATP5ME/CACNB1/MT-ND3/NDUFB4/NDUFA3/NDUFB9/ATP5F1A</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0044272</t>
@@ -5845,31 +5845,31 @@
     <t xml:space="preserve">14/156</t>
   </si>
   <si>
-    <t xml:space="preserve">DLST/PCCA/DLAT/ACSL1/APIP/MMUT/PDHX/GCDH/PDHA1/CBR4/PDPR/PDK2/PDHB/ACACA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLC16A1/ASPA/IDH3G/DLST/IDH3A/GOT2/VDAC1/PCCA/ALDOA/GLUD1/DLAT/MCCC2/FH/IDH2/ACSL1/APIP/MMUT/ECI2/PDHX/GCDH/MDH2/ALDH4A1/PDHA1/CBR4/AUH/OXSM/HMGCL/SUCLG1/PDPR/DECR1/CPT1A/PDK2/CRAT/ALDH7A1/PDHB/ACACA/CS/ACSF2</t>
+    <t xml:space="preserve">PDK2/PDHB/APIP/PDHA1/DLAT/ACSL1/PDHX/CBR4/DLST/MMUT/PCCA/PDPR/GCDH/ACACA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOT2/HMGCL/PDK2/MCCC2/PDHB/APIP/PDHA1/SLC16A1/ALDH4A1/ALDH7A1/DLAT/IDH2/CS/ACSL1/ACSF2/FH/ASPA/CRAT/SUCLG1/ALDOA/PDHX/CBR4/AUH/DLST/MMUT/MDH2/PCCA/VDAC1/IDH3G/OXSM/PDPR/GLUD1/CPT1A/ECI2/GCDH/DECR1/IDH3A/ACACA</t>
   </si>
   <si>
     <t xml:space="preserve">18/156</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/MT-CO2/COX5B/UQCRC1/COX6B1/COX5A/NDUFB9/NDUFB8/UQCRC2/NDUFA7/NDUFB10/NDUFA2/NDUFB4/MT-ND3/NDUFA3/COX4I1/NDUFA12/CHCHD2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NDUFS7/SLC16A1/ATP5F1A/NNT/MT-CO2/COX5B/ANK2/CACNB1/VDAC1/UQCRC1/LETM1/COX6B1/COX5A/STIM1/DMAC2L/NDUFB9/NDUFB8/SLC25A13/NDUFA7/NDUFB10/ATP5ME/ATP5PO/NDUFA2/AFG3L2/NDUFB4/ANK3/MT-ND3/NDUFA3/COX4I1/NDUFA12</t>
+    <t xml:space="preserve">COX5A/COX5B/COX4I1/CHCHD2/UQCRC2/NDUFB8/UQCRC1/MT-CO2/COX6B1/NDUFB10/NDUFA2/NDUFA12/NDUFA7/NDUFS7/MT-ND3/NDUFB4/NDUFA3/NDUFB9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COX5A/SLC16A1/COX5B/COX4I1/DMAC2L/NDUFB8/LETM1/UQCRC1/ANK2/NNT/MT-CO2/ANK3/COX6B1/NDUFB10/SLC25A13/ATP5PO/NDUFA2/AFG3L2/STIM1/NDUFA12/VDAC1/NDUFA7/NDUFS7/ATP5ME/CACNB1/MT-ND3/NDUFB4/NDUFA3/NDUFB9/ATP5F1A</t>
   </si>
   <si>
     <t xml:space="preserve">19/156</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/HCCS/MT-CO2/COX5B/UQCRC1/COX6B1/COX5A/NDUFB9/NDUFB8/UQCRC2/NDUFA7/NDUFB10/NDUFA2/NDUFB4/MT-ND3/NDUFA3/COX4I1/NDUFA12/CHCHD2</t>
+    <t xml:space="preserve">COX5A/COX5B/COX4I1/CHCHD2/UQCRC2/NDUFB8/UQCRC1/MT-CO2/COX6B1/NDUFB10/NDUFA2/HCCS/NDUFA12/NDUFA7/NDUFS7/MT-ND3/NDUFB4/NDUFA3/NDUFB9</t>
   </si>
   <si>
     <t xml:space="preserve">31/156</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/DLST/ATP5F1A/PCCA/ALDOA/DLAT/IDH2/ACSL1/MMUT/PDHX/DMAC2L/NDUFB9/GCDH/NDUFB8/SLC25A13/NDUFA7/NDUFB10/ATP5ME/PDHA1/ATP5PO/NDUFA2/CBR4/NDUFB4/MT-ND3/PDPR/CKMT2/PDK2/NDUFA3/NDUFA12/PDHB/ACACA</t>
+    <t xml:space="preserve">PDK2/CKMT2/PDHB/PDHA1/DMAC2L/DLAT/IDH2/NDUFB8/ACSL1/NDUFB10/ALDOA/SLC25A13/PDHX/CBR4/ATP5PO/NDUFA2/DLST/MMUT/NDUFA12/PCCA/NDUFA7/NDUFS7/ATP5ME/MT-ND3/PDPR/NDUFB4/NDUFA3/NDUFB9/GCDH/ATP5F1A/ACACA</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006790</t>
@@ -5881,34 +5881,34 @@
     <t xml:space="preserve">20/156</t>
   </si>
   <si>
-    <t xml:space="preserve">GSTK1/DLST/PCCA/DLAT/MCCC2/ACSL1/APIP/MMUT/PDHX/GCDH/PDHA1/CBR4/OXSM/SUCLG1/PDPR/PDK2/ALDH7A1/PDHB/ACACA/ACSF2</t>
+    <t xml:space="preserve">PDK2/MCCC2/PDHB/APIP/PDHA1/ALDH7A1/DLAT/ACSL1/ACSF2/SUCLG1/PDHX/GSTK1/CBR4/DLST/MMUT/PCCA/OXSM/PDPR/GCDH/ACACA</t>
   </si>
   <si>
     <t xml:space="preserve">34/156</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/SLC16A1/CAMK2B/ATP5F1A/NNT/MT-CO2/COX5B/ANK2/CACNB1/VDAC1/UQCRC1/LETM1/COX6B1/COX5A/STIM1/FXN/DMAC2L/NDUFB9/NDUFB8/SLC25A13/NDUFA7/NDUFB10/ATP5ME/ATP5PO/NDUFA2/AFG3L2/NDUFB4/VDAC2/ANK3/MT-ND3/NDUFA3/COX4I1/CLIC5/NDUFA12</t>
+    <t xml:space="preserve">COX5A/SLC16A1/COX5B/COX4I1/DMAC2L/NDUFB8/LETM1/UQCRC1/ANK2/NNT/MT-CO2/ANK3/COX6B1/NDUFB10/SLC25A13/ATP5PO/NDUFA2/AFG3L2/STIM1/VDAC2/FXN/CLIC5/NDUFA12/VDAC1/NDUFA7/NDUFS7/ATP5ME/CACNB1/MT-ND3/NDUFB4/CAMK2B/NDUFA3/NDUFB9/ATP5F1A</t>
   </si>
   <si>
     <t xml:space="preserve">11/156</t>
   </si>
   <si>
-    <t xml:space="preserve">MFN2/SAMM50/MTX1/LETM1/MTCH2/TIMM10/APOO/TIMM9/TMEM11/TIMM13/SLC25A46</t>
+    <t xml:space="preserve">TIMM9/MFN2/TIMM13/APOO/TMEM11/TIMM10/SLC25A46/LETM1/SAMM50/MTX1/MTCH2</t>
   </si>
   <si>
     <t xml:space="preserve">59/156</t>
   </si>
   <si>
-    <t xml:space="preserve">MAN2C1/NDUFS7/SLC16A1/ASPA/IDH3G/DLST/ATP5F1A/NNT/IDH3A/GOT2/VDAC1/PCCA/ALDOA/GLUD1/DLAT/MCCC2/FH/IDH2/ACSL1/APIP/COQ3/MMUT/ECI2/PDHX/COQ8A/DMAC2L/NDUFB9/GCDH/MDH2/NDUFB8/ALDH4A1/SLC25A13/NDUFA7/NDUFB10/ATP5ME/PDHA1/ATP5PO/NDUFA2/CBR4/AUH/OXSM/NDUFB4/COQ5/HMGCL/PPTC7/SUCLG1/MT-ND3/PDPR/DECR1/CPT1A/PDK2/NDUFA3/CRAT/ALDH7A1/NDUFA12/PDHB/ACACA/CS/ACSF2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NDUFS7/SLC16A1/CAMK2B/ATP5F1A/NNT/MT-CO2/COX5B/ANK2/CACNB1/VDAC1/UQCRC1/LETM1/COX6B1/COX5A/STIM1/FXN/DMAC2L/NDUFB9/NDUFB8/SLC25A13/NDUFA7/NDUFB10/ATP5ME/ATP5PO/NDUFA2/AFG3L2/NDUFB4/ANK3/MT-ND3/NDUFA3/COX4I1/NDUFA12</t>
+    <t xml:space="preserve">GOT2/HMGCL/PDK2/MCCC2/PDHB/APIP/PDHA1/SLC16A1/ALDH4A1/ALDH7A1/PPTC7/DMAC2L/DLAT/IDH2/NDUFB8/CS/MAN2C1/ACSL1/ACSF2/FH/ASPA/CRAT/NNT/SUCLG1/NDUFB10/ALDOA/SLC25A13/PDHX/CBR4/ATP5PO/NDUFA2/AUH/DLST/COQ3/MMUT/MDH2/NDUFA12/PCCA/VDAC1/NDUFA7/NDUFS7/ATP5ME/IDH3G/OXSM/MT-ND3/PDPR/GLUD1/CPT1A/COQ5/NDUFB4/ECI2/NDUFA3/COQ8A/NDUFB9/GCDH/DECR1/ATP5F1A/IDH3A/ACACA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COX5A/SLC16A1/COX5B/COX4I1/DMAC2L/NDUFB8/LETM1/UQCRC1/ANK2/NNT/MT-CO2/ANK3/COX6B1/NDUFB10/SLC25A13/ATP5PO/NDUFA2/AFG3L2/STIM1/FXN/NDUFA12/VDAC1/NDUFA7/NDUFS7/ATP5ME/CACNB1/MT-ND3/NDUFB4/CAMK2B/NDUFA3/NDUFB9/ATP5F1A</t>
   </si>
   <si>
     <t xml:space="preserve">16/156</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/MT-CO2/COX5B/UQCRC1/COX6B1/COX5A/NDUFB9/NDUFB8/UQCRC2/NDUFA7/NDUFB10/NDUFA2/NDUFB4/MT-ND3/NDUFA3/COX4I1</t>
+    <t xml:space="preserve">COX5A/COX5B/COX4I1/UQCRC2/NDUFB8/UQCRC1/MT-CO2/COX6B1/NDUFB10/NDUFA2/NDUFA7/NDUFS7/MT-ND3/NDUFB4/NDUFA3/NDUFB9</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006086</t>
@@ -5920,16 +5920,16 @@
     <t xml:space="preserve">6/156</t>
   </si>
   <si>
-    <t xml:space="preserve">DLAT/PDHX/PDHA1/PDPR/PDK2/PDHB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NDUFS7/ATP5F1A/ALDOA/DMAC2L/NDUFB9/NDUFB8/SLC25A13/NDUFA7/NDUFB10/ATP5ME/ATP5PO/NDUFA2/NDUFB4/MT-ND3/NDUFA3/NDUFA12</t>
+    <t xml:space="preserve">PDK2/PDHB/PDHA1/DLAT/PDHX/PDPR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DMAC2L/NDUFB8/NDUFB10/ALDOA/SLC25A13/ATP5PO/NDUFA2/NDUFA12/NDUFA7/NDUFS7/ATP5ME/MT-ND3/NDUFB4/NDUFA3/NDUFB9/ATP5F1A</t>
   </si>
   <si>
     <t xml:space="preserve">9/156</t>
   </si>
   <si>
-    <t xml:space="preserve">SAMM50/MTX1/LETM1/TIMM10/APOO/TIMM9/TMEM11/TIMM13/SLC25A46</t>
+    <t xml:space="preserve">TIMM9/TIMM13/APOO/TMEM11/TIMM10/SLC25A46/LETM1/SAMM50/MTX1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:1901605</t>
@@ -5938,7 +5938,7 @@
     <t xml:space="preserve">alpha-amino acid metabolic process</t>
   </si>
   <si>
-    <t xml:space="preserve">ASPA/DLST/GOT2/GLUD1/MCCC2/FH/APIP/MMUT/GCDH/ALDH4A1/AUH/HMGCL/ALDH7A1</t>
+    <t xml:space="preserve">GOT2/HMGCL/MCCC2/APIP/ALDH4A1/ALDH7A1/FH/ASPA/AUH/DLST/MMUT/GLUD1/GCDH</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0006085</t>
@@ -5947,13 +5947,13 @@
     <t xml:space="preserve">acetyl-CoA biosynthetic process</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/ATP5F1A/NDUFB9/NDUFB8/NDUFA7/NDUFB10/ATP5ME/ATP5PO/NDUFA2/NDUFB4/MT-ND3/NDUFA3/NDUFA12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLC16A1/ASPA/VDAC1/PCCA/ALDOA/DLAT/IDH2/ACSL1/MMUT/ECI2/PDHX/GCDH/PDHA1/CBR4/AUH/OXSM/PDPR/DECR1/CPT1A/PDK2/CRAT/PDHB/ACACA/ACSF2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NDUFS7/DLST/ATP5F1A/NNT/GOT2/PCCA/ALDOA/DLAT/MCCC2/IDH2/ACSL1/MMUT/PDHX/DMAC2L/NDUFB9/GCDH/MDH2/NDUFB8/SLC25A13/NDUFA7/NDUFB10/ATP5ME/PDHA1/ATP5PO/NDUFA2/CBR4/OXSM/NDUFB4/SUCLG1/MT-ND3/PDPR/CKMT2/PDK2/NDUFA3/ALDH7A1/NDUFA12/PDHB/ACACA/ACSF2</t>
+    <t xml:space="preserve">NDUFB8/NDUFB10/ATP5PO/NDUFA2/NDUFA12/NDUFA7/NDUFS7/ATP5ME/MT-ND3/NDUFB4/NDUFA3/NDUFB9/ATP5F1A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PDK2/PDHB/PDHA1/SLC16A1/DLAT/IDH2/ACSL1/ACSF2/ASPA/CRAT/ALDOA/PDHX/CBR4/AUH/MMUT/PCCA/VDAC1/OXSM/PDPR/CPT1A/ECI2/GCDH/DECR1/ACACA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOT2/PDK2/MCCC2/CKMT2/PDHB/PDHA1/ALDH7A1/DMAC2L/DLAT/IDH2/NDUFB8/ACSL1/ACSF2/NNT/SUCLG1/NDUFB10/ALDOA/SLC25A13/PDHX/CBR4/ATP5PO/NDUFA2/DLST/MMUT/MDH2/NDUFA12/PCCA/NDUFA7/NDUFS7/ATP5ME/OXSM/MT-ND3/PDPR/NDUFB4/NDUFA3/NDUFB9/GCDH/ATP5F1A/ACACA</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0140053</t>
@@ -5962,13 +5962,13 @@
     <t xml:space="preserve">mitochondrial gene expression</t>
   </si>
   <si>
-    <t xml:space="preserve">MRPL12/MTIF2/MRPL37/TFAM/TRMT10C/SARS2/MRPL38/MTRES1/GFM1/TSFM</t>
+    <t xml:space="preserve">MRPL37/MRPL12/MTIF2/TSFM/TFAM/MRPL38/TRMT10C/SARS2/GFM1/MTRES1</t>
   </si>
   <si>
     <t xml:space="preserve">5/156</t>
   </si>
   <si>
-    <t xml:space="preserve">MT-CO2/COX5B/COX6B1/COX5A/COX4I1</t>
+    <t xml:space="preserve">COX5A/COX5B/COX4I1/MT-CO2/COX6B1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0016054</t>
@@ -5980,7 +5980,7 @@
     <t xml:space="preserve">74/1573</t>
   </si>
   <si>
-    <t xml:space="preserve">SLC16A1/DLST/GOT2/PCCA/GLUD1/DLAT/MCCC2/ECI2/GCDH/ALDH4A1/AUH/HMGCL/DECR1/CPT1A/CRAT/ALDH7A1</t>
+    <t xml:space="preserve">GOT2/HMGCL/MCCC2/SLC16A1/ALDH4A1/ALDH7A1/DLAT/CRAT/AUH/DLST/PCCA/GLUD1/CPT1A/ECI2/GCDH/DECR1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0046395</t>
@@ -5995,25 +5995,25 @@
     <t xml:space="preserve">cytochrome complex assembly</t>
   </si>
   <si>
-    <t xml:space="preserve">HCCS/MT-CO2/COX20/FXN/COX19/SLC25A46</t>
+    <t xml:space="preserve">SLC25A46/COX19/MT-CO2/HCCS/FXN/COX20</t>
   </si>
   <si>
     <t xml:space="preserve">116/155</t>
   </si>
   <si>
-    <t xml:space="preserve">GSTK1/NDUFS7/MRPL12/MTIF2/IDH3G/HCCS/DLST/ATP5F1A/MFN2/NNT/MT-CO2/PPIF/SAMM50/IDH3A/COX5B/MRPL37/MTX1/ANK2/GOT2/TFAM/VDAC1/PCCA/GLUD1/ATAD3A/DLAT/MCCC2/FH/UQCRC1/NFU1/LETM1/COX6B1/ENDOG/IDH2/ACSL1/COX5A/COX20/NDUFAF3/HSDL2/TMEM143/TRMT10C/COQ3/FXN/SARS2/MMUT/ECI2/MTCH2/PDHX/MRPL38/COQ8A/MTRES1/ATPAF2/DMAC2L/NDUFB9/MAOB/GCDH/LONP1/GFM1/MDH2/DNAJA3/NDUFB8/MAP2K2/ALDH4A1/SLC25A6/SLC25A13/TIMM10/UQCRC2/NDUFA7/NDUFB10/HTRA2/ATP5ME/PDHA1/ATP5PO/NLRX1/NDUFA2/CBR4/AUH/AFG3L2/OXSM/NDUFB4/COQ5/APOO/HMGCL/VDAC2/PPTC7/SUCLG1/MT-ND3/PLGRKT/PDPR/CKMT2/DECR1/CPT1A/PDK2/TIMM9/MAOA/BSG/NDUFA3/TSFM/CRAT/COX19/NDUFAF5/ALDH7A1/COX4I1/CLIC5/NDUFA12/AIFM1/CHCHD2/PDHB/TRAP1/TMEM11/TIMM13/ACACA/MPC2/SLC25A46/CS/ACSF2/SYNJ2BP</t>
+    <t xml:space="preserve">GOT2/HMGCL/PDK2/MCCC2/SYNJ2BP/CKMT2/PDHB/COX5A/TIMM9/PDHA1/MFN2/TIMM13/MRPL37/APOO/NDUFAF5/COX5B/ALDH4A1/COX4I1/ALDH7A1/MAOA/PPTC7/DMAC2L/ATPAF2/CHCHD2/TMEM11/MRPL12/DLAT/ATAD3A/UQCRC2/TIMM10/IDH2/MAP2K2/NDUFB8/DNAJA3/CS/SLC25A46/LETM1/UQCRC1/NFU1/ACSL1/ACSF2/FH/TRAP1/MTIF2/ENDOG/ANK2/TSFM/CRAT/COX19/NNT/PPIF/MT-CO2/SUCLG1/COX6B1/HTRA2/NDUFB10/TFAM/AIFM1/SLC25A13/SLC25A6/MRPL38/PDHX/GSTK1/CBR4/ATP5PO/NLRX1/NDUFA2/SAMM50/AFG3L2/AUH/TRMT10C/TMEM143/VDAC2/HCCS/DLST/FXN/COQ3/SARS2/MMUT/LONP1/GFM1/HSDL2/NDUFAF3/MDH2/CLIC5/NDUFA12/MTX1/PCCA/VDAC1/NDUFA7/NDUFS7/ATP5ME/IDH3G/COX20/OXSM/MT-ND3/PDPR/PLGRKT/GLUD1/CPT1A/COQ5/NDUFB4/MTCH2/ECI2/BSG/NDUFA3/MTRES1/COQ8A/NDUFB9/GCDH/MAOB/DECR1/ATP5F1A/IDH3A/ACACA/MPC2</t>
   </si>
   <si>
     <t xml:space="preserve">67/155</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/MRPL12/HCCS/ATP5F1A/MFN2/NNT/MT-CO2/PPIF/SAMM50/COX5B/MRPL37/MTX1/VDAC1/ATAD3A/UQCRC1/LETM1/COX6B1/ENDOG/ACSL1/COX5A/COX20/NDUFAF3/COQ3/MTCH2/MRPL38/COQ8A/ATPAF2/DMAC2L/NDUFB9/MAOB/NDUFB8/SLC25A6/SLC25A13/TIMM10/UQCRC2/NDUFA7/NDUFB10/HTRA2/ATP5ME/ATP5PO/NLRX1/NDUFA2/AFG3L2/NDUFB4/COQ5/APOO/VDAC2/PPTC7/MT-ND3/CKMT2/CPT1A/TIMM9/MAOA/NDUFA3/CRAT/COX19/NDUFAF5/COX4I1/NDUFA12/AIFM1/CHCHD2/TRAP1/TMEM11/TIMM13/MPC2/SLC25A46/SYNJ2BP</t>
+    <t xml:space="preserve">SYNJ2BP/CKMT2/COX5A/TIMM9/MFN2/TIMM13/MRPL37/APOO/NDUFAF5/COX5B/COX4I1/MAOA/PPTC7/DMAC2L/ATPAF2/CHCHD2/TMEM11/MRPL12/ATAD3A/UQCRC2/TIMM10/NDUFB8/SLC25A46/LETM1/UQCRC1/ACSL1/TRAP1/ENDOG/CRAT/COX19/NNT/PPIF/MT-CO2/COX6B1/HTRA2/NDUFB10/AIFM1/SLC25A13/SLC25A6/MRPL38/ATP5PO/NLRX1/NDUFA2/SAMM50/AFG3L2/VDAC2/HCCS/COQ3/NDUFAF3/NDUFA12/MTX1/VDAC1/NDUFA7/NDUFS7/ATP5ME/COX20/MT-ND3/CPT1A/COQ5/NDUFB4/MTCH2/NDUFA3/COQ8A/NDUFB9/MAOB/ATP5F1A/MPC2</t>
   </si>
   <si>
     <t xml:space="preserve">64/155</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/MRPL12/HCCS/ATP5F1A/MFN2/NNT/MT-CO2/SAMM50/COX5B/MRPL37/MTX1/VDAC1/ATAD3A/UQCRC1/LETM1/COX6B1/ENDOG/ACSL1/COX5A/COX20/NDUFAF3/COQ3/MTCH2/MRPL38/COQ8A/ATPAF2/DMAC2L/NDUFB9/MAOB/NDUFB8/SLC25A6/SLC25A13/TIMM10/UQCRC2/NDUFA7/NDUFB10/HTRA2/ATP5ME/ATP5PO/NLRX1/NDUFA2/AFG3L2/NDUFB4/COQ5/APOO/VDAC2/PPTC7/MT-ND3/CKMT2/CPT1A/TIMM9/MAOA/NDUFA3/CRAT/NDUFAF5/COX4I1/NDUFA12/AIFM1/TRAP1/TMEM11/TIMM13/MPC2/SLC25A46/SYNJ2BP</t>
+    <t xml:space="preserve">SYNJ2BP/CKMT2/COX5A/TIMM9/MFN2/TIMM13/MRPL37/APOO/NDUFAF5/COX5B/COX4I1/MAOA/PPTC7/DMAC2L/ATPAF2/TMEM11/MRPL12/ATAD3A/UQCRC2/TIMM10/NDUFB8/SLC25A46/LETM1/UQCRC1/ACSL1/TRAP1/ENDOG/CRAT/NNT/MT-CO2/COX6B1/HTRA2/NDUFB10/AIFM1/SLC25A13/SLC25A6/MRPL38/ATP5PO/NLRX1/NDUFA2/SAMM50/AFG3L2/VDAC2/HCCS/COQ3/NDUFAF3/NDUFA12/MTX1/VDAC1/NDUFA7/NDUFS7/ATP5ME/COX20/MT-ND3/CPT1A/COQ5/NDUFB4/MTCH2/NDUFA3/COQ8A/NDUFB9/MAOB/ATP5F1A/MPC2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005759</t>
@@ -6028,49 +6028,49 @@
     <t xml:space="preserve">183/1600</t>
   </si>
   <si>
-    <t xml:space="preserve">GSTK1/NDUFS7/MRPL12/MTIF2/IDH3G/DLST/ATP5F1A/MT-CO2/PPIF/IDH3A/MRPL37/GOT2/TFAM/VDAC1/PCCA/GLUD1/ATAD3A/DLAT/MCCC2/FH/UQCRC1/NFU1/IDH2/TRMT10C/COQ3/FXN/SARS2/MMUT/PDHX/MRPL38/MTRES1/GCDH/LONP1/GFM1/MDH2/DNAJA3/NDUFB8/ALDH4A1/PDHA1/CBR4/AUH/OXSM/COQ5/HMGCL/VDAC2/PPTC7/SUCLG1/PDPR/DECR1/PDK2/TSFM/ALDH7A1/PDHB/TRAP1/CS/ACSF2</t>
+    <t xml:space="preserve">GOT2/HMGCL/PDK2/MCCC2/PDHB/PDHA1/MRPL37/ALDH4A1/ALDH7A1/PPTC7/MRPL12/DLAT/ATAD3A/IDH2/NDUFB8/DNAJA3/CS/UQCRC1/NFU1/ACSF2/FH/TRAP1/MTIF2/TSFM/PPIF/MT-CO2/SUCLG1/TFAM/MRPL38/PDHX/GSTK1/CBR4/AUH/TRMT10C/VDAC2/DLST/FXN/COQ3/SARS2/MMUT/LONP1/GFM1/MDH2/PCCA/VDAC1/NDUFS7/IDH3G/OXSM/PDPR/GLUD1/COQ5/MTRES1/GCDH/DECR1/ATP5F1A/IDH3A</t>
   </si>
   <si>
     <t xml:space="preserve">69/155</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/MRPL12/HCCS/ATP5F1A/MFN2/NNT/MT-CO2/PPIF/SAMM50/COX5B/MRPL37/MTX1/XPO7/VDAC1/ATAD3A/UQCRC1/LETM1/COX6B1/ENDOG/ACSL1/COX5A/COX20/NDUFAF3/COQ3/MTCH2/MRPL38/COQ8A/ATPAF2/DMAC2L/NDUFB9/MAOB/NDUFB8/SLC25A6/SLC25A13/TIMM10/UQCRC2/NDUFA7/NDUFB10/HTRA2/ATP5ME/ATP5PO/NLRX1/NDUFA2/AFG3L2/NDUFB4/COQ5/APOO/VDAC2/PPTC7/MT-ND3/CKMT2/CPT1A/TIMM9/MAOA/NDUFA3/FXR1/CRAT/COX19/NDUFAF5/COX4I1/NDUFA12/AIFM1/CHCHD2/TRAP1/TMEM11/TIMM13/MPC2/SLC25A46/SYNJ2BP</t>
+    <t xml:space="preserve">SYNJ2BP/CKMT2/COX5A/TIMM9/MFN2/TIMM13/MRPL37/APOO/NDUFAF5/COX5B/COX4I1/MAOA/PPTC7/DMAC2L/ATPAF2/CHCHD2/TMEM11/MRPL12/ATAD3A/UQCRC2/TIMM10/NDUFB8/SLC25A46/LETM1/UQCRC1/ACSL1/TRAP1/ENDOG/CRAT/COX19/NNT/PPIF/MT-CO2/COX6B1/HTRA2/NDUFB10/XPO7/AIFM1/SLC25A13/SLC25A6/MRPL38/ATP5PO/NLRX1/NDUFA2/SAMM50/AFG3L2/VDAC2/HCCS/COQ3/NDUFAF3/NDUFA12/MTX1/VDAC1/NDUFA7/NDUFS7/ATP5ME/COX20/MT-ND3/CPT1A/COQ5/NDUFB4/MTCH2/NDUFA3/FXR1/COQ8A/NDUFB9/MAOB/ATP5F1A/MPC2</t>
   </si>
   <si>
     <t xml:space="preserve">51/155</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/MRPL12/HCCS/ATP5F1A/NNT/MT-CO2/SAMM50/COX5B/MRPL37/MTX1/ATAD3A/UQCRC1/LETM1/COX6B1/ENDOG/COX5A/COX20/NDUFAF3/COQ3/MRPL38/COQ8A/ATPAF2/DMAC2L/NDUFB9/NDUFB8/SLC25A6/SLC25A13/TIMM10/UQCRC2/NDUFA7/NDUFB10/ATP5ME/ATP5PO/NDUFA2/AFG3L2/NDUFB4/COQ5/APOO/MT-ND3/CKMT2/TIMM9/NDUFA3/CRAT/NDUFAF5/COX4I1/NDUFA12/AIFM1/TRAP1/TMEM11/TIMM13/MPC2</t>
+    <t xml:space="preserve">CKMT2/COX5A/TIMM9/TIMM13/MRPL37/APOO/NDUFAF5/COX5B/COX4I1/DMAC2L/ATPAF2/TMEM11/MRPL12/ATAD3A/UQCRC2/TIMM10/NDUFB8/LETM1/UQCRC1/TRAP1/ENDOG/CRAT/NNT/MT-CO2/COX6B1/NDUFB10/AIFM1/SLC25A13/SLC25A6/MRPL38/ATP5PO/NDUFA2/SAMM50/AFG3L2/HCCS/COQ3/NDUFAF3/NDUFA12/MTX1/NDUFA7/NDUFS7/ATP5ME/COX20/MT-ND3/COQ5/NDUFB4/NDUFA3/COQ8A/NDUFB9/ATP5F1A/MPC2</t>
   </si>
   <si>
     <t xml:space="preserve">22/155</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/ATP5F1A/NNT/MT-CO2/COX5B/UQCRC1/COX6B1/COX5A/DMAC2L/NDUFB9/NDUFB8/UQCRC2/NDUFA7/NDUFB10/ATP5ME/ATP5PO/NDUFA2/NDUFB4/MT-ND3/NDUFA3/COX4I1/NDUFA12</t>
+    <t xml:space="preserve">COX5A/COX5B/COX4I1/DMAC2L/UQCRC2/NDUFB8/UQCRC1/NNT/MT-CO2/COX6B1/NDUFB10/ATP5PO/NDUFA2/NDUFA12/NDUFA7/NDUFS7/ATP5ME/MT-ND3/NDUFB4/NDUFA3/NDUFB9/ATP5F1A</t>
   </si>
   <si>
     <t xml:space="preserve">17/155</t>
   </si>
   <si>
-    <t xml:space="preserve">MRPL12/PPIF/SAMM50/MRPL37/MTX1/VDAC1/UQCRC1/TRMT10C/FXN/MRPL38/SLC25A6/TIMM10/AFG3L2/APOO/TIMM9/TIMM13/MPC2</t>
+    <t xml:space="preserve">TIMM9/TIMM13/MRPL37/APOO/MRPL12/TIMM10/UQCRC1/PPIF/SLC25A6/MRPL38/SAMM50/AFG3L2/TRMT10C/FXN/MTX1/VDAC1/MPC2</t>
   </si>
   <si>
     <t xml:space="preserve">19/155</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/IDH3G/DLST/IDH3A/DLAT/PDHX/NDUFB9/NDUFB8/NDUFA7/NDUFB10/PDHA1/NDUFA2/CBR4/NDUFB4/MT-ND3/PDK2/NDUFA3/NDUFA12/PDHB</t>
+    <t xml:space="preserve">PDK2/PDHB/PDHA1/DLAT/NDUFB8/NDUFB10/PDHX/CBR4/NDUFA2/DLST/NDUFA12/NDUFA7/NDUFS7/IDH3G/MT-ND3/NDUFB4/NDUFA3/NDUFB9/IDH3A</t>
   </si>
   <si>
     <t xml:space="preserve">73/155</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/MRPL12/CAMK2B/HCCS/ATP5F1A/MFN2/NNT/MT-CO2/SAMM50/COX5B/MRPL37/MTX1/VDAC1/ATAD3A/UQCRC1/LETM1/COX6B1/ENDOG/ACSL1/COX5A/COX20/NDUFAF3/STIM1/COQ3/MTCH2/VPS4B/MRPL38/COQ8A/ATPAF2/DMAC2L/NDUFB9/MAOB/NDUFB8/MAP2K2/SLC25A6/SLC25A13/TIMM10/UQCRC2/RRAGC/NDUFA7/NDUFB10/HTRA2/ATP5ME/ATP5PO/NLRX1/NDUFA2/AFG3L2/NDUFB4/COQ5/APOO/VDAC2/PPTC7/MT-ND3/CKMT2/CPT1A/TIMM9/MAOA/BSG/NDUFA3/CRAT/NDUFAF5/ALDH7A1/COX4I1/SGCA/NDUFA12/AIFM1/SNX5/TRAP1/TMEM11/TIMM13/MPC2/SLC25A46/SYNJ2BP</t>
+    <t xml:space="preserve">SYNJ2BP/CKMT2/COX5A/TIMM9/MFN2/TIMM13/MRPL37/APOO/NDUFAF5/COX5B/COX4I1/ALDH7A1/MAOA/PPTC7/DMAC2L/ATPAF2/TMEM11/MRPL12/ATAD3A/UQCRC2/TIMM10/MAP2K2/NDUFB8/SLC25A46/LETM1/UQCRC1/ACSL1/VPS4B/TRAP1/ENDOG/CRAT/NNT/MT-CO2/COX6B1/HTRA2/NDUFB10/AIFM1/SNX5/SLC25A13/SLC25A6/MRPL38/ATP5PO/NLRX1/NDUFA2/SAMM50/AFG3L2/STIM1/VDAC2/HCCS/COQ3/NDUFAF3/NDUFA12/SGCA/MTX1/VDAC1/RRAGC/NDUFA7/NDUFS7/ATP5ME/COX20/MT-ND3/CPT1A/COQ5/NDUFB4/CAMK2B/MTCH2/BSG/NDUFA3/COQ8A/NDUFB9/MAOB/ATP5F1A/MPC2</t>
   </si>
   <si>
     <t xml:space="preserve">24/155</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/ATP5F1A/MT-CO2/COX5B/CACNB1/UQCRC1/COX6B1/COX5A/DMAC2L/NDUFB9/NDUFB8/UQCRC2/NDUFA7/NDUFB10/ATP5ME/ATP5PO/NDUFA2/NDUFB4/MT-ND3/NDUFA3/COX4I1/CLIC5/NDUFA12/MPC2</t>
+    <t xml:space="preserve">COX5A/COX5B/COX4I1/DMAC2L/UQCRC2/NDUFB8/UQCRC1/MT-CO2/COX6B1/NDUFB10/ATP5PO/NDUFA2/CLIC5/NDUFA12/NDUFA7/NDUFS7/ATP5ME/CACNB1/MT-ND3/NDUFB4/NDUFA3/NDUFB9/ATP5F1A/MPC2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005741</t>
@@ -6082,7 +6082,7 @@
     <t xml:space="preserve">15/155</t>
   </si>
   <si>
-    <t xml:space="preserve">MFN2/SAMM50/MTX1/VDAC1/ACSL1/MTCH2/MAOB/NLRX1/APOO/VDAC2/PPTC7/CPT1A/MAOA/SLC25A46/SYNJ2BP</t>
+    <t xml:space="preserve">SYNJ2BP/MFN2/APOO/MAOA/PPTC7/SLC25A46/ACSL1/NLRX1/SAMM50/VDAC2/MTX1/VDAC1/CPT1A/MTCH2/MAOB</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0019867</t>
@@ -6103,13 +6103,13 @@
     <t xml:space="preserve">36/155</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/ATP5F1A/MT-CO2/PPIF/SAMM50/COX5B/MTX1/CACNB1/VDAC1/UQCRC1/COX6B1/COX5A/DMAC2L/NDUFB9/NDUFB8/SLC25A6/TIMM10/UQCRC2/NDUFA7/NDUFB10/HTRA2/ATP5ME/ATP5PO/NDUFA2/AFG3L2/NDUFB4/APOO/VDAC2/MT-ND3/NDUFA3/COX4I1/SGCA/CLIC5/NDUFA12/SNX5/MPC2</t>
+    <t xml:space="preserve">COX5A/APOO/COX5B/COX4I1/DMAC2L/UQCRC2/TIMM10/NDUFB8/UQCRC1/PPIF/MT-CO2/COX6B1/HTRA2/NDUFB10/SNX5/SLC25A6/ATP5PO/NDUFA2/SAMM50/AFG3L2/VDAC2/CLIC5/NDUFA12/SGCA/MTX1/VDAC1/NDUFA7/NDUFS7/ATP5ME/CACNB1/MT-ND3/NDUFB4/NDUFA3/NDUFB9/ATP5F1A/MPC2</t>
   </si>
   <si>
     <t xml:space="preserve">7/155</t>
   </si>
   <si>
-    <t xml:space="preserve">SAMM50/MTX1/SLC25A6/TIMM10/AFG3L2/APOO/MPC2</t>
+    <t xml:space="preserve">APOO/TIMM10/SLC25A6/SAMM50/AFG3L2/MTX1/MPC2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0045240</t>
@@ -6121,7 +6121,7 @@
     <t xml:space="preserve">6/155</t>
   </si>
   <si>
-    <t xml:space="preserve">DLST/DLAT/PDHX/PDHA1/PDK2/PDHB</t>
+    <t xml:space="preserve">PDK2/PDHB/PDHA1/DLAT/PDHX/DLST</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0009295</t>
@@ -6130,7 +6130,7 @@
     <t xml:space="preserve">nucleoid</t>
   </si>
   <si>
-    <t xml:space="preserve">TFAM/VDAC1/ATAD3A/TRMT10C/LONP1/DNAJA3/VDAC2</t>
+    <t xml:space="preserve">ATAD3A/DNAJA3/TFAM/TRMT10C/VDAC2/LONP1/VDAC1</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0042645</t>
@@ -6142,13 +6142,13 @@
     <t xml:space="preserve">10/155</t>
   </si>
   <si>
-    <t xml:space="preserve">COX5A/TIMM10/HTRA2/TIMM9/COX19/COX4I1/AIFM1/CHCHD2/TRAP1/TIMM13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MT-CO2/COX5B/UQCRC1/COX6B1/COX5A/UQCRC2/COX4I1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NDUFS7/NDUFB9/NDUFB8/NDUFA7/NDUFB10/NDUFA2/NDUFB4/MT-ND3/NDUFA3/NDUFA12</t>
+    <t xml:space="preserve">COX5A/TIMM9/TIMM13/COX4I1/CHCHD2/TIMM10/TRAP1/COX19/HTRA2/AIFM1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COX5A/COX5B/COX4I1/UQCRC2/UQCRC1/MT-CO2/COX6B1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NDUFB8/NDUFB10/NDUFA2/NDUFA12/NDUFA7/NDUFS7/MT-ND3/NDUFB4/NDUFA3/NDUFB9</t>
   </si>
   <si>
     <t xml:space="preserve">GO:1902493</t>
@@ -6160,7 +6160,7 @@
     <t xml:space="preserve">5/155</t>
   </si>
   <si>
-    <t xml:space="preserve">DLAT/PDHX/PDHA1/PDK2/PDHB</t>
+    <t xml:space="preserve">PDK2/PDHB/PDHA1/DLAT/PDHX</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0005777</t>
@@ -6172,7 +6172,7 @@
     <t xml:space="preserve">8/155</t>
   </si>
   <si>
-    <t xml:space="preserve">GSTK1/IDH2/ACSL1/HSDL2/ECI2/MAP2K2/HMGCL/CRAT</t>
+    <t xml:space="preserve">HMGCL/IDH2/MAP2K2/ACSL1/CRAT/GSTK1/HSDL2/ECI2</t>
   </si>
   <si>
     <t xml:space="preserve">GO:0042579</t>
@@ -6184,40 +6184,40 @@
     <t xml:space="preserve">28/155</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/SLC16A1/ATP5F1A/NNT/MT-CO2/COX5B/CACNB1/VDAC1/UQCRC1/LETM1/COX6B1/COX5A/DMAC2L/NDUFB9/NDUFB8/SLC25A13/NDUFA7/NDUFB10/ATP5ME/ATP5PO/NDUFA2/NDUFB4/VDAC2/MT-ND3/NDUFA3/COX4I1/CLIC5/NDUFA12</t>
+    <t xml:space="preserve">COX5A/SLC16A1/COX5B/COX4I1/DMAC2L/NDUFB8/LETM1/UQCRC1/NNT/MT-CO2/COX6B1/NDUFB10/SLC25A13/ATP5PO/NDUFA2/VDAC2/CLIC5/NDUFA12/VDAC1/NDUFA7/NDUFS7/ATP5ME/CACNB1/MT-ND3/NDUFB4/NDUFA3/NDUFB9/ATP5F1A</t>
   </si>
   <si>
     <t xml:space="preserve">30/155</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/SLC16A1/ATP5F1A/NNT/MT-CO2/COX5B/CACNB1/VDAC1/UQCRC1/LETM1/COX6B1/COX5A/DMAC2L/NDUFB9/NDUFB8/SLC25A6/SLC25A13/NDUFA7/NDUFB10/ATP5ME/ATP5PO/NDUFA2/NDUFB4/VDAC2/MT-ND3/NDUFA3/COX4I1/CLIC5/NDUFA12/MPC2</t>
+    <t xml:space="preserve">COX5A/SLC16A1/COX5B/COX4I1/DMAC2L/NDUFB8/LETM1/UQCRC1/NNT/MT-CO2/COX6B1/NDUFB10/SLC25A13/SLC25A6/ATP5PO/NDUFA2/VDAC2/CLIC5/NDUFA12/VDAC1/NDUFA7/NDUFS7/ATP5ME/CACNB1/MT-ND3/NDUFB4/NDUFA3/NDUFB9/ATP5F1A/MPC2</t>
   </si>
   <si>
     <t xml:space="preserve">25/155</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/SLC16A1/ATP5F1A/NNT/MT-CO2/COX5B/CACNB1/UQCRC1/LETM1/COX6B1/COX5A/DMAC2L/NDUFB9/NDUFB8/SLC25A13/NDUFA7/NDUFB10/ATP5ME/ATP5PO/NDUFA2/NDUFB4/MT-ND3/NDUFA3/COX4I1/NDUFA12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NDUFS7/NNT/MT-CO2/COX5B/UQCRC1/COX6B1/COX5A/NDUFB9/NDUFB8/NDUFA7/NDUFB10/NDUFA2/NDUFB4/MT-ND3/NDUFA3/COX4I1/NDUFA12</t>
+    <t xml:space="preserve">COX5A/SLC16A1/COX5B/COX4I1/DMAC2L/NDUFB8/LETM1/UQCRC1/NNT/MT-CO2/COX6B1/NDUFB10/SLC25A13/ATP5PO/NDUFA2/NDUFA12/NDUFA7/NDUFS7/ATP5ME/CACNB1/MT-ND3/NDUFB4/NDUFA3/NDUFB9/ATP5F1A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COX5A/COX5B/COX4I1/NDUFB8/UQCRC1/NNT/MT-CO2/COX6B1/NDUFB10/NDUFA2/NDUFA12/NDUFA7/NDUFS7/MT-ND3/NDUFB4/NDUFA3/NDUFB9</t>
   </si>
   <si>
     <t xml:space="preserve">31/155</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/SLC16A1/ATP5F1A/NNT/MT-CO2/COX5B/CACNB1/VDAC1/UQCRC1/LETM1/COX6B1/COX5A/DMAC2L/NDUFB9/NDUFB8/SLC25A6/SLC25A13/NDUFA7/NDUFB10/ATP5ME/ATP5PO/NDUFA2/NDUFB4/VDAC2/MT-ND3/TIMM9/NDUFA3/COX4I1/CLIC5/NDUFA12/MPC2</t>
+    <t xml:space="preserve">COX5A/TIMM9/SLC16A1/COX5B/COX4I1/DMAC2L/NDUFB8/LETM1/UQCRC1/NNT/MT-CO2/COX6B1/NDUFB10/SLC25A13/SLC25A6/ATP5PO/NDUFA2/VDAC2/CLIC5/NDUFA12/VDAC1/NDUFA7/NDUFS7/ATP5ME/CACNB1/MT-ND3/NDUFB4/NDUFA3/NDUFB9/ATP5F1A/MPC2</t>
   </si>
   <si>
     <t xml:space="preserve">21/155</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/SLC16A1/NNT/MT-CO2/COX5B/UQCRC1/LETM1/COX6B1/COX5A/NDUFB9/NDUFB8/SLC25A6/SLC25A13/NDUFA7/NDUFB10/NDUFA2/NDUFB4/MT-ND3/NDUFA3/COX4I1/NDUFA12</t>
+    <t xml:space="preserve">COX5A/SLC16A1/COX5B/COX4I1/NDUFB8/LETM1/UQCRC1/NNT/MT-CO2/COX6B1/NDUFB10/SLC25A13/SLC25A6/NDUFA2/NDUFA12/NDUFA7/NDUFS7/MT-ND3/NDUFB4/NDUFA3/NDUFB9</t>
   </si>
   <si>
     <t xml:space="preserve">18/155</t>
   </si>
   <si>
-    <t xml:space="preserve">NDUFS7/MT-CO2/COX5B/UQCRC1/COX6B1/COX5A/NDUFB9/MAOB/NDUFB8/ALDH4A1/NDUFA7/NDUFB10/NDUFA2/NDUFB4/MT-ND3/NDUFA3/COX4I1/NDUFA12</t>
+    <t xml:space="preserve">COX5A/COX5B/ALDH4A1/COX4I1/NDUFB8/UQCRC1/MT-CO2/COX6B1/NDUFB10/NDUFA2/NDUFA12/NDUFA7/NDUFS7/MT-ND3/NDUFB4/NDUFA3/NDUFB9/MAOB</t>
   </si>
   <si>
     <t xml:space="preserve">gene</t>

</xml_diff>